<commit_message>
updating numbers to match pregnancies
</commit_message>
<xml_diff>
--- a/Burden-of-Illness-Tool/MADMC B19 Pregancy Outcome Estimate Tool_Sept2025.xlsx
+++ b/Burden-of-Illness-Tool/MADMC B19 Pregancy Outcome Estimate Tool_Sept2025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\margo\OneDrive\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ritesh/Desktop/Scenario-Modeling-of-Human-Parvovirus-B19/Burden-of-Illness-Tool/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9872890A-4F0E-44D4-A72B-B794578B8A3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48435279-3A36-2144-A09E-09DC83770885}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="2" r:id="rId1"/>
@@ -1925,6 +1925,13 @@
   <fonts count="31" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -2129,13 +2136,6 @@
     </font>
     <font>
       <b/>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -2628,9 +2628,9 @@
   </borders>
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="174">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -2639,8 +2639,8 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -2648,14 +2648,14 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="4" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2688,13 +2688,13 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="9" fontId="3" fillId="5" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="9" fontId="4" fillId="5" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2707,7 +2707,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -2716,30 +2716,30 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1" indent="2"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -2754,16 +2754,16 @@
     <xf numFmtId="9" fontId="0" fillId="4" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="4" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2775,10 +2775,10 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="4" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2790,25 +2790,25 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="4"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="4"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="15" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -2816,35 +2816,35 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="3" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2874,13 +2874,13 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -2889,54 +2889,54 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2965,7 +2965,7 @@
     <xf numFmtId="3" fontId="0" fillId="2" borderId="35" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="30" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="30" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2992,7 +2992,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="35" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="4" borderId="35" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="3" fillId="4" borderId="35" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="4" borderId="35" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3007,7 +3007,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="36" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="4" borderId="36" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="3" fillId="4" borderId="36" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="4" borderId="36" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3016,65 +3016,83 @@
     <xf numFmtId="3" fontId="0" fillId="4" borderId="34" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="3" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="3" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="8" borderId="35" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="30" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -3100,31 +3118,13 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -5469,15 +5469,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>3540125</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>171450</xdr:rowOff>
+      <xdr:colOff>4441825</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>7067550</xdr:colOff>
+      <xdr:colOff>7969250</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>867081</xdr:rowOff>
+      <xdr:rowOff>905181</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5506,8 +5506,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4721225" y="714375"/>
-          <a:ext cx="3527425" cy="879781"/>
+          <a:off x="5737225" y="781050"/>
+          <a:ext cx="3527425" cy="886131"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5910,26 +5910,26 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2D67F48-99C5-4DBB-9139-21F0A09DC1AF}">
   <dimension ref="B4:L48"/>
-  <sheetFormatPr defaultColWidth="8.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="8.453125" style="90"/>
-    <col min="3" max="3" width="162.453125" style="90" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.453125" style="90" customWidth="1"/>
-    <col min="5" max="12" width="11.6328125" style="90" customWidth="1"/>
-    <col min="13" max="16384" width="8.453125" style="90"/>
+    <col min="1" max="2" width="8.5" style="90"/>
+    <col min="3" max="3" width="162.5" style="90" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.5" style="90" customWidth="1"/>
+    <col min="5" max="12" width="11.6640625" style="90" customWidth="1"/>
+    <col min="13" max="16384" width="8.5" style="90"/>
   </cols>
   <sheetData>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B4" s="18"/>
       <c r="C4" s="18"/>
       <c r="D4" s="18"/>
     </row>
-    <row r="5" spans="2:12" ht="79" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:12" ht="79" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="18"/>
       <c r="C5" s="18"/>
       <c r="D5" s="18"/>
     </row>
-    <row r="6" spans="2:12" ht="32.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:12" ht="32.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="18"/>
       <c r="C6" s="91" t="s">
         <v>139</v>
@@ -5944,7 +5944,7 @@
       <c r="K6" s="92"/>
       <c r="L6" s="92"/>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B7" s="18"/>
       <c r="C7" s="32"/>
       <c r="D7" s="32"/>
@@ -5957,12 +5957,12 @@
       <c r="K7" s="92"/>
       <c r="L7" s="92"/>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B8" s="18"/>
       <c r="C8" s="18"/>
       <c r="D8" s="18"/>
     </row>
-    <row r="9" spans="2:12" ht="63" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:12" ht="66" x14ac:dyDescent="0.2">
       <c r="B9" s="18"/>
       <c r="C9" s="93" t="s">
         <v>140</v>
@@ -5977,7 +5977,7 @@
       <c r="K9" s="95"/>
       <c r="L9" s="95"/>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B10" s="18"/>
       <c r="C10" s="45"/>
       <c r="D10" s="94"/>
@@ -5990,7 +5990,7 @@
       <c r="K10" s="95"/>
       <c r="L10" s="95"/>
     </row>
-    <row r="11" spans="2:12" ht="42" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:12" ht="44" x14ac:dyDescent="0.2">
       <c r="B11" s="18"/>
       <c r="C11" s="93" t="s">
         <v>149</v>
@@ -6005,7 +6005,7 @@
       <c r="K11" s="95"/>
       <c r="L11" s="95"/>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B12" s="18"/>
       <c r="C12" s="45"/>
       <c r="D12" s="94"/>
@@ -6018,7 +6018,7 @@
       <c r="K12" s="95"/>
       <c r="L12" s="95"/>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B13" s="18"/>
       <c r="C13" s="45"/>
       <c r="D13" s="94"/>
@@ -6031,7 +6031,7 @@
       <c r="K13" s="95"/>
       <c r="L13" s="95"/>
     </row>
-    <row r="14" spans="2:12" ht="21" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:12" ht="21" x14ac:dyDescent="0.2">
       <c r="B14" s="18"/>
       <c r="C14" s="96" t="s">
         <v>109</v>
@@ -6046,7 +6046,7 @@
       <c r="K14" s="95"/>
       <c r="L14" s="95"/>
     </row>
-    <row r="15" spans="2:12" ht="21" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:12" ht="23" x14ac:dyDescent="0.2">
       <c r="B15" s="18"/>
       <c r="C15" s="97" t="s">
         <v>150</v>
@@ -6060,7 +6060,7 @@
       <c r="J15" s="95"/>
       <c r="K15" s="95"/>
     </row>
-    <row r="16" spans="2:12" ht="42" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:12" ht="23" x14ac:dyDescent="0.2">
       <c r="B16" s="18"/>
       <c r="C16" s="97" t="s">
         <v>107</v>
@@ -6074,7 +6074,7 @@
       <c r="J16" s="95"/>
       <c r="K16" s="95"/>
     </row>
-    <row r="17" spans="2:12" ht="21" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:12" ht="23" x14ac:dyDescent="0.2">
       <c r="B17" s="18"/>
       <c r="C17" s="97" t="s">
         <v>108</v>
@@ -6088,12 +6088,12 @@
       <c r="J17" s="95"/>
       <c r="K17" s="95"/>
     </row>
-    <row r="18" spans="2:12" ht="21" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:12" ht="21" x14ac:dyDescent="0.2">
       <c r="B18" s="18"/>
       <c r="C18" s="98"/>
       <c r="D18" s="18"/>
     </row>
-    <row r="19" spans="2:12" ht="105" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:12" ht="110" x14ac:dyDescent="0.2">
       <c r="B19" s="18"/>
       <c r="C19" s="93" t="s">
         <v>106</v>
@@ -6108,7 +6108,7 @@
       <c r="K19" s="95"/>
       <c r="L19" s="95"/>
     </row>
-    <row r="20" spans="2:12" ht="21" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:12" ht="21" x14ac:dyDescent="0.2">
       <c r="B20" s="18"/>
       <c r="C20" s="99"/>
       <c r="D20" s="94"/>
@@ -6121,7 +6121,7 @@
       <c r="K20" s="95"/>
       <c r="L20" s="95"/>
     </row>
-    <row r="21" spans="2:12" ht="21" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:12" ht="21" x14ac:dyDescent="0.2">
       <c r="B21" s="18"/>
       <c r="C21" s="99"/>
       <c r="D21" s="94"/>
@@ -6134,7 +6134,7 @@
       <c r="K21" s="95"/>
       <c r="L21" s="95"/>
     </row>
-    <row r="22" spans="2:12" ht="21" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:12" ht="21" x14ac:dyDescent="0.2">
       <c r="B22" s="18"/>
       <c r="C22" s="99"/>
       <c r="D22" s="94"/>
@@ -6147,37 +6147,37 @@
       <c r="K22" s="95"/>
       <c r="L22" s="95"/>
     </row>
-    <row r="23" spans="2:12" ht="21" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:12" ht="21" x14ac:dyDescent="0.2">
       <c r="B23" s="18"/>
       <c r="C23" s="99"/>
       <c r="D23" s="18"/>
     </row>
-    <row r="24" spans="2:12" ht="21" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:12" ht="21" x14ac:dyDescent="0.2">
       <c r="B24" s="18"/>
       <c r="C24" s="99"/>
       <c r="D24" s="18"/>
     </row>
-    <row r="25" spans="2:12" ht="21" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:12" ht="21" x14ac:dyDescent="0.2">
       <c r="B25" s="18"/>
       <c r="C25" s="99"/>
       <c r="D25" s="18"/>
     </row>
-    <row r="26" spans="2:12" ht="21" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:12" ht="21" x14ac:dyDescent="0.2">
       <c r="B26" s="18"/>
       <c r="C26" s="99"/>
       <c r="D26" s="18"/>
     </row>
-    <row r="27" spans="2:12" ht="21" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:12" ht="21" x14ac:dyDescent="0.2">
       <c r="B27" s="18"/>
       <c r="C27" s="99"/>
       <c r="D27" s="18"/>
     </row>
-    <row r="28" spans="2:12" ht="21" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:12" ht="21" x14ac:dyDescent="0.2">
       <c r="B28" s="18"/>
       <c r="C28" s="99"/>
       <c r="D28" s="18"/>
     </row>
-    <row r="29" spans="2:12" ht="210" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:12" ht="220" x14ac:dyDescent="0.2">
       <c r="B29" s="18"/>
       <c r="C29" s="93" t="s">
         <v>105</v>
@@ -6192,12 +6192,12 @@
       <c r="K29" s="95"/>
       <c r="L29" s="95"/>
     </row>
-    <row r="30" spans="2:12" ht="21" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:12" ht="21" x14ac:dyDescent="0.2">
       <c r="B30" s="18"/>
       <c r="C30" s="96"/>
       <c r="D30" s="18"/>
     </row>
-    <row r="31" spans="2:12" ht="168" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:12" ht="154" x14ac:dyDescent="0.2">
       <c r="B31" s="18"/>
       <c r="C31" s="93" t="s">
         <v>133</v>
@@ -6212,7 +6212,7 @@
       <c r="K31" s="95"/>
       <c r="L31" s="95"/>
     </row>
-    <row r="32" spans="2:12" ht="21" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:12" ht="21" x14ac:dyDescent="0.2">
       <c r="B32" s="18"/>
       <c r="C32" s="100"/>
       <c r="D32" s="94"/>
@@ -6225,7 +6225,7 @@
       <c r="K32" s="95"/>
       <c r="L32" s="95"/>
     </row>
-    <row r="33" spans="2:12" ht="21" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:12" ht="21" x14ac:dyDescent="0.2">
       <c r="B33" s="18"/>
       <c r="C33" s="96" t="s">
         <v>104</v>
@@ -6240,17 +6240,17 @@
       <c r="K33" s="95"/>
       <c r="L33" s="95"/>
     </row>
-    <row r="34" spans="2:12" ht="21" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:12" ht="21" x14ac:dyDescent="0.2">
       <c r="B34" s="18"/>
       <c r="C34" s="101"/>
       <c r="D34" s="18"/>
     </row>
-    <row r="35" spans="2:12" ht="21" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:12" ht="21" x14ac:dyDescent="0.2">
       <c r="B35" s="11"/>
       <c r="C35" s="102"/>
       <c r="D35" s="11"/>
     </row>
-    <row r="36" spans="2:12" ht="42" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:12" ht="44" x14ac:dyDescent="0.2">
       <c r="B36" s="11"/>
       <c r="C36" s="103" t="s">
         <v>103</v>
@@ -6265,80 +6265,80 @@
       <c r="K36" s="95"/>
       <c r="L36" s="95"/>
     </row>
-    <row r="37" spans="2:12" ht="21" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:12" ht="21" x14ac:dyDescent="0.2">
       <c r="B37" s="11"/>
       <c r="C37" s="105"/>
       <c r="D37" s="11"/>
     </row>
-    <row r="38" spans="2:12" ht="63" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:12" ht="66" x14ac:dyDescent="0.2">
       <c r="B38" s="11"/>
       <c r="C38" s="103" t="s">
         <v>136</v>
       </c>
       <c r="D38" s="106"/>
     </row>
-    <row r="39" spans="2:12" ht="21" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:12" ht="21" x14ac:dyDescent="0.2">
       <c r="B39" s="11"/>
       <c r="C39" s="103"/>
       <c r="D39" s="106"/>
     </row>
-    <row r="40" spans="2:12" ht="17" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B40" s="11"/>
       <c r="C40" s="105" t="s">
         <v>137</v>
       </c>
       <c r="D40" s="11"/>
     </row>
-    <row r="41" spans="2:12" ht="17" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B41" s="11"/>
       <c r="C41" s="105"/>
       <c r="D41" s="11"/>
     </row>
-    <row r="42" spans="2:12" ht="21" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:12" ht="21" x14ac:dyDescent="0.2">
       <c r="B42" s="11"/>
       <c r="C42" s="107" t="s">
         <v>102</v>
       </c>
       <c r="D42" s="11"/>
     </row>
-    <row r="43" spans="2:12" ht="21" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:12" ht="21" x14ac:dyDescent="0.2">
       <c r="B43" s="11"/>
       <c r="C43" s="108" t="s">
         <v>134</v>
       </c>
       <c r="D43" s="11"/>
     </row>
-    <row r="44" spans="2:12" ht="21" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:12" ht="21" x14ac:dyDescent="0.2">
       <c r="B44" s="11"/>
       <c r="C44" s="102"/>
       <c r="D44" s="11"/>
     </row>
-    <row r="45" spans="2:12" ht="21" x14ac:dyDescent="0.35">
+    <row r="45" spans="2:12" ht="21" x14ac:dyDescent="0.2">
       <c r="B45" s="11"/>
       <c r="C45" s="102" t="s">
         <v>141</v>
       </c>
       <c r="D45" s="11"/>
     </row>
-    <row r="46" spans="2:12" ht="21" x14ac:dyDescent="0.35">
+    <row r="46" spans="2:12" ht="21" x14ac:dyDescent="0.2">
       <c r="B46" s="11"/>
       <c r="C46" s="109" t="s">
         <v>138</v>
       </c>
       <c r="D46" s="11"/>
     </row>
-    <row r="47" spans="2:12" ht="21" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:12" ht="21" x14ac:dyDescent="0.2">
       <c r="B47" s="11"/>
       <c r="C47" s="102"/>
       <c r="D47" s="11"/>
     </row>
-    <row r="48" spans="2:12" ht="62" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:12" ht="62" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B48" s="11"/>
       <c r="C48" s="11"/>
       <c r="D48" s="11"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
+  <sheetProtection selectLockedCells="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -6347,63 +6347,63 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4E0B51A-7E99-B445-9709-9B3BD93CABEF}">
   <dimension ref="A1:AC49"/>
-  <sheetFormatPr defaultColWidth="10.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.81640625" style="6" customWidth="1"/>
-    <col min="2" max="2" width="28.08984375" style="6" customWidth="1"/>
-    <col min="3" max="3" width="26.90625" style="6" customWidth="1"/>
-    <col min="4" max="17" width="10.81640625" style="6" customWidth="1"/>
-    <col min="18" max="23" width="10.81640625" style="6"/>
-    <col min="24" max="27" width="10.81640625" style="6" customWidth="1"/>
-    <col min="28" max="16384" width="10.81640625" style="6"/>
+    <col min="1" max="1" width="10.83203125" style="6" customWidth="1"/>
+    <col min="2" max="2" width="28.1640625" style="6" customWidth="1"/>
+    <col min="3" max="3" width="26.83203125" style="6" customWidth="1"/>
+    <col min="4" max="17" width="10.83203125" style="6" customWidth="1"/>
+    <col min="18" max="23" width="10.83203125" style="6"/>
+    <col min="24" max="27" width="10.83203125" style="6" customWidth="1"/>
+    <col min="28" max="16384" width="10.83203125" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" s="26" customFormat="1" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:29" s="26" customFormat="1" ht="24" x14ac:dyDescent="0.3">
       <c r="B1" s="25" t="s">
         <v>145</v>
       </c>
       <c r="C1" s="25"/>
       <c r="E1" s="27"/>
     </row>
-    <row r="3" spans="1:29" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="151" t="s">
+    <row r="3" spans="1:29" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B3" s="144" t="s">
         <v>143</v>
       </c>
-      <c r="C3" s="151"/>
-      <c r="D3" s="151"/>
-      <c r="E3" s="151"/>
-      <c r="F3" s="151"/>
-      <c r="G3" s="151"/>
-      <c r="H3" s="151"/>
-      <c r="I3" s="151"/>
-      <c r="J3" s="151"/>
-      <c r="K3" s="151"/>
-      <c r="L3" s="151"/>
-      <c r="M3" s="151"/>
-      <c r="N3" s="151"/>
-      <c r="O3" s="151"/>
-      <c r="P3" s="151"/>
-      <c r="Q3" s="151"/>
-    </row>
-    <row r="4" spans="1:29" x14ac:dyDescent="0.35">
-      <c r="B4" s="151"/>
-      <c r="C4" s="151"/>
-      <c r="D4" s="151"/>
-      <c r="E4" s="151"/>
-      <c r="F4" s="151"/>
-      <c r="G4" s="151"/>
-      <c r="H4" s="151"/>
-      <c r="I4" s="151"/>
-      <c r="J4" s="151"/>
-      <c r="K4" s="151"/>
-      <c r="L4" s="151"/>
-      <c r="M4" s="151"/>
-      <c r="N4" s="151"/>
-      <c r="O4" s="151"/>
-      <c r="P4" s="151"/>
-      <c r="Q4" s="151"/>
-    </row>
-    <row r="5" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="C3" s="144"/>
+      <c r="D3" s="144"/>
+      <c r="E3" s="144"/>
+      <c r="F3" s="144"/>
+      <c r="G3" s="144"/>
+      <c r="H3" s="144"/>
+      <c r="I3" s="144"/>
+      <c r="J3" s="144"/>
+      <c r="K3" s="144"/>
+      <c r="L3" s="144"/>
+      <c r="M3" s="144"/>
+      <c r="N3" s="144"/>
+      <c r="O3" s="144"/>
+      <c r="P3" s="144"/>
+      <c r="Q3" s="144"/>
+    </row>
+    <row r="4" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="B4" s="144"/>
+      <c r="C4" s="144"/>
+      <c r="D4" s="144"/>
+      <c r="E4" s="144"/>
+      <c r="F4" s="144"/>
+      <c r="G4" s="144"/>
+      <c r="H4" s="144"/>
+      <c r="I4" s="144"/>
+      <c r="J4" s="144"/>
+      <c r="K4" s="144"/>
+      <c r="L4" s="144"/>
+      <c r="M4" s="144"/>
+      <c r="N4" s="144"/>
+      <c r="O4" s="144"/>
+      <c r="P4" s="144"/>
+      <c r="Q4" s="144"/>
+    </row>
+    <row r="5" spans="1:29" ht="16" x14ac:dyDescent="0.2">
       <c r="B5" s="111"/>
       <c r="C5" s="111"/>
       <c r="D5" s="111"/>
@@ -6421,7 +6421,7 @@
       <c r="P5" s="111"/>
       <c r="Q5" s="111"/>
     </row>
-    <row r="6" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
@@ -6442,7 +6442,7 @@
       <c r="R6" s="3"/>
       <c r="X6" s="9"/>
     </row>
-    <row r="7" spans="1:29" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:29" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3"/>
       <c r="B7" s="4" t="s">
         <v>38</v>
@@ -6466,7 +6466,7 @@
       <c r="Q7" s="33"/>
       <c r="R7" s="18"/>
     </row>
-    <row r="8" spans="1:29" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:29" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3"/>
       <c r="B8" s="140" t="s">
         <v>21</v>
@@ -6483,17 +6483,17 @@
       <c r="F8" s="32"/>
       <c r="G8" s="4"/>
       <c r="H8" s="3"/>
-      <c r="I8" s="152" t="str">
+      <c r="I8" s="145" t="str">
         <f>_xlfn.CONCAT("Based on ", C9, " pregnancies in the population and historic estimates of parvovirus immunity, mother infection risk, fetal infection risk, and risk of severe fetal outcomes (Table 1), the expected number of severe fetal outcomes due to parvovirus is ",C22,". Under a best case scenario of higher immunity, lower infection rates, and lower complication rates, the number of severe fetal outcomes due to PVB19 could be as low as ", F22, ", while under a worst case scenario the number of severe fetal outcomes may be as high as ", G22, " in the population with ", C9, " pregnancies (Figure 1, Table 2).")</f>
         <v>Based on 100000 pregnancies in the population and historic estimates of parvovirus immunity, mother infection risk, fetal infection risk, and risk of severe fetal outcomes (Table 1), the expected number of severe fetal outcomes due to parvovirus is . Under a best case scenario of higher immunity, lower infection rates, and lower complication rates, the number of severe fetal outcomes due to PVB19 could be as low as , while under a worst case scenario the number of severe fetal outcomes may be as high as  in the population with 100000 pregnancies (Figure 1, Table 2).</v>
       </c>
-      <c r="J8" s="152"/>
-      <c r="K8" s="152"/>
-      <c r="L8" s="152"/>
-      <c r="M8" s="152"/>
-      <c r="N8" s="152"/>
-      <c r="O8" s="152"/>
-      <c r="P8" s="152"/>
+      <c r="J8" s="145"/>
+      <c r="K8" s="145"/>
+      <c r="L8" s="145"/>
+      <c r="M8" s="145"/>
+      <c r="N8" s="145"/>
+      <c r="O8" s="145"/>
+      <c r="P8" s="145"/>
       <c r="Q8" s="33"/>
       <c r="R8" s="18"/>
       <c r="X8" s="9"/>
@@ -6503,7 +6503,7 @@
       <c r="AB8" s="10"/>
       <c r="AC8" s="10"/>
     </row>
-    <row r="9" spans="1:29" ht="27" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:29" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="3"/>
       <c r="B9" s="118" t="s">
         <v>110</v>
@@ -6520,14 +6520,14 @@
       <c r="F9" s="71"/>
       <c r="G9" s="4"/>
       <c r="H9" s="33"/>
-      <c r="I9" s="152"/>
-      <c r="J9" s="152"/>
-      <c r="K9" s="152"/>
-      <c r="L9" s="152"/>
-      <c r="M9" s="152"/>
-      <c r="N9" s="152"/>
-      <c r="O9" s="152"/>
-      <c r="P9" s="152"/>
+      <c r="I9" s="145"/>
+      <c r="J9" s="145"/>
+      <c r="K9" s="145"/>
+      <c r="L9" s="145"/>
+      <c r="M9" s="145"/>
+      <c r="N9" s="145"/>
+      <c r="O9" s="145"/>
+      <c r="P9" s="145"/>
       <c r="Q9" s="33"/>
       <c r="R9" s="18"/>
       <c r="X9" s="8"/>
@@ -6537,7 +6537,7 @@
       <c r="AB9" s="69"/>
       <c r="AC9" s="69"/>
     </row>
-    <row r="10" spans="1:29" ht="31" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:29" ht="34" x14ac:dyDescent="0.2">
       <c r="A10" s="3"/>
       <c r="B10" s="121" t="s">
         <v>111</v>
@@ -6554,14 +6554,14 @@
       <c r="F10" s="72"/>
       <c r="G10" s="4"/>
       <c r="H10" s="33"/>
-      <c r="I10" s="152"/>
-      <c r="J10" s="152"/>
-      <c r="K10" s="152"/>
-      <c r="L10" s="152"/>
-      <c r="M10" s="152"/>
-      <c r="N10" s="152"/>
-      <c r="O10" s="152"/>
-      <c r="P10" s="152"/>
+      <c r="I10" s="145"/>
+      <c r="J10" s="145"/>
+      <c r="K10" s="145"/>
+      <c r="L10" s="145"/>
+      <c r="M10" s="145"/>
+      <c r="N10" s="145"/>
+      <c r="O10" s="145"/>
+      <c r="P10" s="145"/>
       <c r="Q10" s="33"/>
       <c r="R10" s="18"/>
       <c r="X10" s="8"/>
@@ -6571,7 +6571,7 @@
       <c r="AB10" s="69"/>
       <c r="AC10" s="69"/>
     </row>
-    <row r="11" spans="1:29" ht="50" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:29" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="3"/>
       <c r="B11" s="121" t="s">
         <v>112</v>
@@ -6605,7 +6605,7 @@
       <c r="AB11" s="69"/>
       <c r="AC11" s="69"/>
     </row>
-    <row r="12" spans="1:29" ht="46" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:29" ht="51" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3"/>
       <c r="B12" s="123" t="s">
         <v>118</v>
@@ -6639,14 +6639,14 @@
       <c r="AB12" s="69"/>
       <c r="AC12" s="69"/>
     </row>
-    <row r="13" spans="1:29" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:29" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="3"/>
-      <c r="B13" s="146" t="s">
+      <c r="B13" s="149" t="s">
         <v>114</v>
       </c>
-      <c r="C13" s="146"/>
-      <c r="D13" s="146"/>
-      <c r="E13" s="146"/>
+      <c r="C13" s="149"/>
+      <c r="D13" s="149"/>
+      <c r="E13" s="149"/>
       <c r="F13" s="72"/>
       <c r="G13" s="3"/>
       <c r="H13" s="3"/>
@@ -6661,7 +6661,7 @@
       <c r="Q13" s="3"/>
       <c r="R13" s="3"/>
     </row>
-    <row r="14" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A14" s="3"/>
       <c r="B14" s="3"/>
       <c r="C14" s="38"/>
@@ -6681,7 +6681,7 @@
       <c r="Q14" s="3"/>
       <c r="R14" s="3"/>
     </row>
-    <row r="15" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A15" s="3"/>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
@@ -6701,7 +6701,7 @@
       <c r="Q15" s="3"/>
       <c r="R15" s="3"/>
     </row>
-    <row r="16" spans="1:29" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:29" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3"/>
       <c r="B16" s="4" t="s">
         <v>100</v>
@@ -6723,22 +6723,22 @@
       <c r="Q16" s="3"/>
       <c r="R16" s="3"/>
     </row>
-    <row r="17" spans="1:18" ht="33.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:18" ht="33.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3"/>
-      <c r="B17" s="147" t="s">
+      <c r="B17" s="150" t="s">
         <v>99</v>
       </c>
       <c r="C17" s="77" t="s">
         <v>6</v>
       </c>
-      <c r="D17" s="149" t="s">
+      <c r="D17" s="152" t="s">
         <v>16</v>
       </c>
-      <c r="E17" s="150"/>
-      <c r="F17" s="149" t="s">
+      <c r="E17" s="153"/>
+      <c r="F17" s="152" t="s">
         <v>19</v>
       </c>
-      <c r="G17" s="150"/>
+      <c r="G17" s="153"/>
       <c r="H17" s="75"/>
       <c r="I17" s="5"/>
       <c r="J17" s="5"/>
@@ -6751,9 +6751,9 @@
       <c r="Q17" s="3"/>
       <c r="R17" s="3"/>
     </row>
-    <row r="18" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:18" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3"/>
-      <c r="B18" s="148"/>
+      <c r="B18" s="151"/>
       <c r="C18" s="78" t="s">
         <v>41</v>
       </c>
@@ -6781,7 +6781,7 @@
       <c r="Q18" s="3"/>
       <c r="R18" s="3"/>
     </row>
-    <row r="19" spans="1:18" ht="29" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:18" ht="32" x14ac:dyDescent="0.2">
       <c r="A19" s="3"/>
       <c r="B19" s="127" t="s">
         <v>115</v>
@@ -6818,7 +6818,7 @@
       <c r="Q19" s="3"/>
       <c r="R19" s="3"/>
     </row>
-    <row r="20" spans="1:18" ht="29" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:18" ht="32" x14ac:dyDescent="0.2">
       <c r="A20" s="3"/>
       <c r="B20" s="121" t="s">
         <v>116</v>
@@ -6855,7 +6855,7 @@
       <c r="Q20" s="3"/>
       <c r="R20" s="3"/>
     </row>
-    <row r="21" spans="1:18" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:18" ht="33" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3"/>
       <c r="B21" s="123" t="s">
         <v>117</v>
@@ -6892,7 +6892,7 @@
       <c r="Q21" s="3"/>
       <c r="R21" s="3"/>
     </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A22" s="3"/>
       <c r="B22" s="39" t="s">
         <v>135</v>
@@ -6914,7 +6914,7 @@
       <c r="Q22" s="3"/>
       <c r="R22" s="3"/>
     </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A23" s="3"/>
       <c r="B23" s="39" t="s">
         <v>36</v>
@@ -6936,16 +6936,16 @@
       <c r="Q23" s="3"/>
       <c r="R23" s="3"/>
     </row>
-    <row r="24" spans="1:18" ht="44" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:18" ht="44" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="3"/>
-      <c r="B24" s="145" t="s">
+      <c r="B24" s="148" t="s">
         <v>35</v>
       </c>
-      <c r="C24" s="145"/>
-      <c r="D24" s="145"/>
-      <c r="E24" s="145"/>
-      <c r="F24" s="145"/>
-      <c r="G24" s="145"/>
+      <c r="C24" s="148"/>
+      <c r="D24" s="148"/>
+      <c r="E24" s="148"/>
+      <c r="F24" s="148"/>
+      <c r="G24" s="148"/>
       <c r="H24" s="38"/>
       <c r="I24" s="38"/>
       <c r="J24" s="3"/>
@@ -6958,16 +6958,16 @@
       <c r="Q24" s="3"/>
       <c r="R24" s="3"/>
     </row>
-    <row r="25" spans="1:18" ht="45" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:18" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="3"/>
-      <c r="B25" s="145" t="s">
+      <c r="B25" s="148" t="s">
         <v>39</v>
       </c>
-      <c r="C25" s="145"/>
-      <c r="D25" s="145"/>
-      <c r="E25" s="145"/>
-      <c r="F25" s="145"/>
-      <c r="G25" s="145"/>
+      <c r="C25" s="148"/>
+      <c r="D25" s="148"/>
+      <c r="E25" s="148"/>
+      <c r="F25" s="148"/>
+      <c r="G25" s="148"/>
       <c r="H25" s="38"/>
       <c r="I25" s="44"/>
       <c r="J25" s="74"/>
@@ -6980,7 +6980,7 @@
       <c r="Q25" s="74"/>
       <c r="R25" s="3"/>
     </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A26" s="3"/>
       <c r="B26" s="3"/>
       <c r="C26" s="38"/>
@@ -7000,7 +7000,7 @@
       <c r="Q26" s="74"/>
       <c r="R26" s="3"/>
     </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A27" s="3"/>
       <c r="B27" s="3"/>
       <c r="C27" s="38"/>
@@ -7020,7 +7020,7 @@
       <c r="Q27" s="3"/>
       <c r="R27" s="3"/>
     </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A28" s="3"/>
       <c r="B28" s="3"/>
       <c r="C28" s="38"/>
@@ -7040,7 +7040,7 @@
       <c r="Q28" s="3"/>
       <c r="R28" s="3"/>
     </row>
-    <row r="29" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A29" s="3"/>
       <c r="B29" s="3"/>
       <c r="C29" s="37"/>
@@ -7060,7 +7060,7 @@
       <c r="Q29" s="3"/>
       <c r="R29" s="3"/>
     </row>
-    <row r="30" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A30" s="3"/>
       <c r="B30" s="3"/>
       <c r="C30" s="3"/>
@@ -7080,7 +7080,7 @@
       <c r="Q30" s="3"/>
       <c r="R30" s="3"/>
     </row>
-    <row r="31" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A31" s="3"/>
       <c r="B31" s="3"/>
       <c r="C31" s="37"/>
@@ -7100,7 +7100,7 @@
       <c r="Q31" s="3"/>
       <c r="R31" s="3"/>
     </row>
-    <row r="32" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A32" s="3"/>
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
@@ -7120,7 +7120,7 @@
       <c r="Q32" s="3"/>
       <c r="R32" s="3"/>
     </row>
-    <row r="33" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A33" s="3"/>
       <c r="B33" s="3"/>
       <c r="C33" s="37"/>
@@ -7140,7 +7140,7 @@
       <c r="Q33" s="3"/>
       <c r="R33" s="3"/>
     </row>
-    <row r="34" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="3"/>
       <c r="B34" s="3"/>
       <c r="C34" s="3"/>
@@ -7160,7 +7160,7 @@
       <c r="Q34" s="3"/>
       <c r="R34" s="3"/>
     </row>
-    <row r="35" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="3"/>
       <c r="B35" s="3"/>
       <c r="C35" s="4"/>
@@ -7180,7 +7180,7 @@
       <c r="Q35" s="3"/>
       <c r="R35" s="3"/>
     </row>
-    <row r="36" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="3"/>
       <c r="B36" s="4" t="s">
         <v>8</v>
@@ -7202,16 +7202,16 @@
       <c r="Q36" s="3"/>
       <c r="R36" s="3"/>
     </row>
-    <row r="37" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="3"/>
-      <c r="B37" s="153" t="s">
+      <c r="B37" s="147" t="s">
         <v>24</v>
       </c>
-      <c r="C37" s="153"/>
-      <c r="D37" s="153"/>
-      <c r="E37" s="153"/>
-      <c r="F37" s="153"/>
-      <c r="G37" s="153"/>
+      <c r="C37" s="147"/>
+      <c r="D37" s="147"/>
+      <c r="E37" s="147"/>
+      <c r="F37" s="147"/>
+      <c r="G37" s="147"/>
       <c r="H37" s="3"/>
       <c r="I37" s="36"/>
       <c r="J37" s="3"/>
@@ -7224,16 +7224,16 @@
       <c r="Q37" s="3"/>
       <c r="R37" s="3"/>
     </row>
-    <row r="38" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A38" s="3"/>
-      <c r="B38" s="144" t="s">
+      <c r="B38" s="146" t="s">
         <v>25</v>
       </c>
-      <c r="C38" s="144"/>
-      <c r="D38" s="144"/>
-      <c r="E38" s="144"/>
-      <c r="F38" s="144"/>
-      <c r="G38" s="144"/>
+      <c r="C38" s="146"/>
+      <c r="D38" s="146"/>
+      <c r="E38" s="146"/>
+      <c r="F38" s="146"/>
+      <c r="G38" s="146"/>
       <c r="H38" s="33"/>
       <c r="I38" s="34"/>
       <c r="J38" s="3"/>
@@ -7246,16 +7246,16 @@
       <c r="Q38" s="3"/>
       <c r="R38" s="3"/>
     </row>
-    <row r="39" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A39" s="3"/>
-      <c r="B39" s="144" t="s">
+      <c r="B39" s="146" t="s">
         <v>30</v>
       </c>
-      <c r="C39" s="144"/>
-      <c r="D39" s="144"/>
-      <c r="E39" s="144"/>
-      <c r="F39" s="144"/>
-      <c r="G39" s="144"/>
+      <c r="C39" s="146"/>
+      <c r="D39" s="146"/>
+      <c r="E39" s="146"/>
+      <c r="F39" s="146"/>
+      <c r="G39" s="146"/>
       <c r="H39" s="33"/>
       <c r="I39" s="34"/>
       <c r="J39" s="3"/>
@@ -7268,16 +7268,16 @@
       <c r="Q39" s="3"/>
       <c r="R39" s="3"/>
     </row>
-    <row r="40" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="3"/>
-      <c r="B40" s="144" t="s">
+      <c r="B40" s="146" t="s">
         <v>31</v>
       </c>
-      <c r="C40" s="144"/>
-      <c r="D40" s="144"/>
-      <c r="E40" s="144"/>
-      <c r="F40" s="144"/>
-      <c r="G40" s="144"/>
+      <c r="C40" s="146"/>
+      <c r="D40" s="146"/>
+      <c r="E40" s="146"/>
+      <c r="F40" s="146"/>
+      <c r="G40" s="146"/>
       <c r="H40" s="33"/>
       <c r="I40" s="34"/>
       <c r="J40" s="3"/>
@@ -7290,16 +7290,16 @@
       <c r="Q40" s="3"/>
       <c r="R40" s="3"/>
     </row>
-    <row r="41" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="3"/>
-      <c r="B41" s="144" t="s">
+      <c r="B41" s="146" t="s">
         <v>32</v>
       </c>
-      <c r="C41" s="144"/>
-      <c r="D41" s="144"/>
-      <c r="E41" s="144"/>
-      <c r="F41" s="144"/>
-      <c r="G41" s="144"/>
+      <c r="C41" s="146"/>
+      <c r="D41" s="146"/>
+      <c r="E41" s="146"/>
+      <c r="F41" s="146"/>
+      <c r="G41" s="146"/>
       <c r="H41" s="33"/>
       <c r="I41" s="34"/>
       <c r="J41" s="3"/>
@@ -7312,7 +7312,7 @@
       <c r="Q41" s="3"/>
       <c r="R41" s="3"/>
     </row>
-    <row r="42" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="3"/>
       <c r="B42" s="3"/>
       <c r="C42" s="3"/>
@@ -7332,18 +7332,18 @@
       <c r="Q42" s="3"/>
       <c r="R42" s="3"/>
     </row>
-    <row r="43" spans="1:18" ht="146" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="44" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:18" ht="146" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="44" spans="1:18" x14ac:dyDescent="0.2">
       <c r="B44" s="9" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="45" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:18" x14ac:dyDescent="0.2">
       <c r="B45" s="6" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="46" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:18" x14ac:dyDescent="0.2">
       <c r="B46" s="42" t="s">
         <v>33</v>
       </c>
@@ -7363,7 +7363,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="47" spans="1:18" ht="29" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:18" ht="32" x14ac:dyDescent="0.2">
       <c r="B47" s="40" t="s">
         <v>119</v>
       </c>
@@ -7388,7 +7388,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="48" spans="1:18" ht="29" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:18" ht="32" x14ac:dyDescent="0.2">
       <c r="B48" s="40" t="s">
         <v>120</v>
       </c>
@@ -7413,7 +7413,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="49" spans="2:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="49" spans="2:7" ht="32" x14ac:dyDescent="0.2">
       <c r="B49" s="40" t="s">
         <v>121</v>
       </c>
@@ -7439,13 +7439,8 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
+  <sheetProtection selectLockedCells="1"/>
   <mergeCells count="13">
-    <mergeCell ref="B3:Q4"/>
-    <mergeCell ref="I8:P10"/>
-    <mergeCell ref="B38:G38"/>
-    <mergeCell ref="B37:G37"/>
-    <mergeCell ref="B39:G39"/>
     <mergeCell ref="B41:G41"/>
     <mergeCell ref="B24:G24"/>
     <mergeCell ref="B25:G25"/>
@@ -7454,6 +7449,11 @@
     <mergeCell ref="D17:E17"/>
     <mergeCell ref="F17:G17"/>
     <mergeCell ref="B40:G40"/>
+    <mergeCell ref="B3:Q4"/>
+    <mergeCell ref="I8:P10"/>
+    <mergeCell ref="B38:G38"/>
+    <mergeCell ref="B37:G37"/>
+    <mergeCell ref="B39:G39"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -7464,27 +7464,27 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A54D747-3B89-BC41-8182-1F289A700DB3}">
   <dimension ref="B1:AH127"/>
-  <sheetFormatPr defaultColWidth="8.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="5.453125" style="6" customWidth="1"/>
-    <col min="2" max="2" width="3.81640625" style="6" customWidth="1"/>
-    <col min="3" max="3" width="35.1796875" style="6" customWidth="1"/>
-    <col min="4" max="4" width="11.453125" style="6" customWidth="1"/>
-    <col min="5" max="5" width="3.453125" style="6" customWidth="1"/>
-    <col min="6" max="6" width="6.453125" style="6" customWidth="1"/>
-    <col min="7" max="7" width="4.453125" style="6" customWidth="1"/>
-    <col min="8" max="19" width="7.1796875" style="6" customWidth="1"/>
-    <col min="20" max="20" width="7.453125" style="6" customWidth="1"/>
-    <col min="21" max="21" width="74.81640625" style="6" customWidth="1"/>
-    <col min="22" max="22" width="23.7265625" style="6" customWidth="1"/>
-    <col min="23" max="27" width="16.453125" style="50" customWidth="1"/>
-    <col min="28" max="28" width="14.453125" style="6" customWidth="1"/>
-    <col min="29" max="29" width="8.453125" style="6"/>
-    <col min="30" max="34" width="14.453125" style="11" customWidth="1"/>
-    <col min="35" max="16384" width="8.453125" style="6"/>
+    <col min="1" max="1" width="5.5" style="6" customWidth="1"/>
+    <col min="2" max="2" width="3.83203125" style="6" customWidth="1"/>
+    <col min="3" max="3" width="35.1640625" style="6" customWidth="1"/>
+    <col min="4" max="4" width="11.5" style="6" customWidth="1"/>
+    <col min="5" max="5" width="3.5" style="6" customWidth="1"/>
+    <col min="6" max="6" width="6.5" style="6" customWidth="1"/>
+    <col min="7" max="7" width="4.5" style="6" customWidth="1"/>
+    <col min="8" max="19" width="7.1640625" style="6" customWidth="1"/>
+    <col min="20" max="20" width="7.5" style="6" customWidth="1"/>
+    <col min="21" max="21" width="74.83203125" style="6" customWidth="1"/>
+    <col min="22" max="22" width="23.6640625" style="6" customWidth="1"/>
+    <col min="23" max="27" width="16.5" style="50" customWidth="1"/>
+    <col min="28" max="28" width="14.5" style="6" customWidth="1"/>
+    <col min="29" max="29" width="8.5" style="6"/>
+    <col min="30" max="34" width="14.5" style="11" customWidth="1"/>
+    <col min="35" max="16384" width="8.5" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:34" s="26" customFormat="1" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="2:34" s="26" customFormat="1" ht="24" x14ac:dyDescent="0.3">
       <c r="C1" s="25" t="s">
         <v>12</v>
       </c>
@@ -7500,31 +7500,31 @@
       <c r="AG1" s="56"/>
       <c r="AH1" s="56"/>
     </row>
-    <row r="2" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:34" x14ac:dyDescent="0.2">
       <c r="F2" s="7"/>
     </row>
-    <row r="3" spans="2:34" ht="51" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C3" s="154" t="s">
+    <row r="3" spans="2:34" ht="51" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C3" s="161" t="s">
         <v>144</v>
       </c>
-      <c r="D3" s="154"/>
-      <c r="E3" s="154"/>
-      <c r="F3" s="154"/>
-      <c r="G3" s="154"/>
-      <c r="H3" s="154"/>
-      <c r="I3" s="154"/>
-      <c r="J3" s="154"/>
-      <c r="K3" s="154"/>
-      <c r="L3" s="154"/>
-      <c r="M3" s="154"/>
-      <c r="N3" s="154"/>
-      <c r="O3" s="154"/>
-      <c r="P3" s="154"/>
-      <c r="Q3" s="154"/>
-      <c r="R3" s="154"/>
-      <c r="S3" s="154"/>
-    </row>
-    <row r="5" spans="2:34" ht="26.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="D3" s="161"/>
+      <c r="E3" s="161"/>
+      <c r="F3" s="161"/>
+      <c r="G3" s="161"/>
+      <c r="H3" s="161"/>
+      <c r="I3" s="161"/>
+      <c r="J3" s="161"/>
+      <c r="K3" s="161"/>
+      <c r="L3" s="161"/>
+      <c r="M3" s="161"/>
+      <c r="N3" s="161"/>
+      <c r="O3" s="161"/>
+      <c r="P3" s="161"/>
+      <c r="Q3" s="161"/>
+      <c r="R3" s="161"/>
+      <c r="S3" s="161"/>
+    </row>
+    <row r="5" spans="2:34" ht="26.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B5" s="3"/>
       <c r="C5" s="4" t="s">
         <v>38</v>
@@ -7534,20 +7534,20 @@
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
-      <c r="I5" s="155" t="str">
+      <c r="I5" s="162" t="str">
         <f>_xlfn.CONCAT("Figure 1. Estimated Number of Severe Fetal Outcomes Under Potential Immunity and Infection Rate Scenarios, based on ",D7," Pregnancies")</f>
         <v>Figure 1. Estimated Number of Severe Fetal Outcomes Under Potential Immunity and Infection Rate Scenarios, based on 100000 Pregnancies</v>
       </c>
-      <c r="J5" s="155"/>
-      <c r="K5" s="155"/>
-      <c r="L5" s="155"/>
-      <c r="M5" s="155"/>
-      <c r="N5" s="155"/>
-      <c r="O5" s="155"/>
-      <c r="P5" s="155"/>
-      <c r="Q5" s="155"/>
-      <c r="R5" s="155"/>
-      <c r="S5" s="155"/>
+      <c r="J5" s="162"/>
+      <c r="K5" s="162"/>
+      <c r="L5" s="162"/>
+      <c r="M5" s="162"/>
+      <c r="N5" s="162"/>
+      <c r="O5" s="162"/>
+      <c r="P5" s="162"/>
+      <c r="Q5" s="162"/>
+      <c r="R5" s="162"/>
+      <c r="S5" s="162"/>
       <c r="T5" s="3"/>
       <c r="W5" s="51" t="s">
         <v>22</v>
@@ -7556,7 +7556,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="2:34" ht="29" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="2:34" ht="29" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B6" s="3"/>
       <c r="C6" s="80" t="s">
         <v>21</v>
@@ -7568,17 +7568,17 @@
       <c r="F6" s="3"/>
       <c r="G6" s="3"/>
       <c r="H6" s="3"/>
-      <c r="I6" s="155"/>
-      <c r="J6" s="155"/>
-      <c r="K6" s="155"/>
-      <c r="L6" s="155"/>
-      <c r="M6" s="155"/>
-      <c r="N6" s="155"/>
-      <c r="O6" s="155"/>
-      <c r="P6" s="155"/>
-      <c r="Q6" s="155"/>
-      <c r="R6" s="155"/>
-      <c r="S6" s="155"/>
+      <c r="I6" s="162"/>
+      <c r="J6" s="162"/>
+      <c r="K6" s="162"/>
+      <c r="L6" s="162"/>
+      <c r="M6" s="162"/>
+      <c r="N6" s="162"/>
+      <c r="O6" s="162"/>
+      <c r="P6" s="162"/>
+      <c r="Q6" s="162"/>
+      <c r="R6" s="162"/>
+      <c r="S6" s="162"/>
       <c r="T6" s="3"/>
       <c r="W6" s="52" t="s">
         <v>4</v>
@@ -7611,7 +7611,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="2:34" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:34" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="3"/>
       <c r="C7" s="112" t="s">
         <v>37</v>
@@ -7621,7 +7621,7 @@
       </c>
       <c r="E7" s="46"/>
       <c r="F7" s="3"/>
-      <c r="G7" s="156" t="s">
+      <c r="G7" s="160" t="s">
         <v>127</v>
       </c>
       <c r="H7" s="13">
@@ -7709,7 +7709,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="2:34" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:34" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="3"/>
       <c r="C8" s="114" t="s">
         <v>122</v>
@@ -7719,7 +7719,7 @@
       </c>
       <c r="E8" s="47"/>
       <c r="F8" s="3"/>
-      <c r="G8" s="156"/>
+      <c r="G8" s="160"/>
       <c r="H8" s="13">
         <v>0.7</v>
       </c>
@@ -7805,7 +7805,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="2:34" ht="29" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="2:34" ht="29" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B9" s="3"/>
       <c r="C9" s="114" t="s">
         <v>123</v>
@@ -7815,7 +7815,7 @@
       </c>
       <c r="E9" s="47"/>
       <c r="F9" s="3"/>
-      <c r="G9" s="156"/>
+      <c r="G9" s="160"/>
       <c r="H9" s="13">
         <v>0.65</v>
       </c>
@@ -7901,7 +7901,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="2:34" ht="29" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="2:34" ht="29" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B10" s="3"/>
       <c r="C10" s="116" t="s">
         <v>124</v>
@@ -7911,7 +7911,7 @@
       </c>
       <c r="E10" s="48"/>
       <c r="F10" s="3"/>
-      <c r="G10" s="156"/>
+      <c r="G10" s="160"/>
       <c r="H10" s="13">
         <v>0.6</v>
       </c>
@@ -7997,13 +7997,13 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="2:34" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:34" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="3"/>
       <c r="C11" s="33"/>
       <c r="D11" s="48"/>
       <c r="E11" s="48"/>
       <c r="F11" s="3"/>
-      <c r="G11" s="156"/>
+      <c r="G11" s="160"/>
       <c r="H11" s="13">
         <v>0.55000000000000004</v>
       </c>
@@ -8089,13 +8089,13 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="2:34" ht="29" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="2:34" ht="29" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
-      <c r="G12" s="156"/>
+      <c r="G12" s="160"/>
       <c r="H12" s="13">
         <v>0.5</v>
       </c>
@@ -8181,7 +8181,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="2:34" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:34" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="3"/>
       <c r="C13" s="23" t="s">
         <v>7</v>
@@ -8189,7 +8189,7 @@
       <c r="D13" s="24"/>
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
-      <c r="G13" s="156"/>
+      <c r="G13" s="160"/>
       <c r="H13" s="13">
         <v>0.45</v>
       </c>
@@ -8275,15 +8275,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="2:34" ht="29" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="2:34" ht="29" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B14" s="3"/>
-      <c r="C14" s="157" t="s">
+      <c r="C14" s="163" t="s">
         <v>46</v>
       </c>
-      <c r="D14" s="158"/>
+      <c r="D14" s="164"/>
       <c r="E14" s="45"/>
       <c r="F14" s="3"/>
-      <c r="G14" s="156"/>
+      <c r="G14" s="160"/>
       <c r="H14" s="13">
         <v>0.4</v>
       </c>
@@ -8369,13 +8369,13 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="2:34" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:34" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="3"/>
-      <c r="C15" s="159"/>
-      <c r="D15" s="158"/>
+      <c r="C15" s="165"/>
+      <c r="D15" s="164"/>
       <c r="E15" s="45"/>
       <c r="F15" s="3"/>
-      <c r="G15" s="156"/>
+      <c r="G15" s="160"/>
       <c r="H15" s="13">
         <v>0.35</v>
       </c>
@@ -8461,15 +8461,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="2:34" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:34" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="3"/>
-      <c r="C16" s="160" t="s">
+      <c r="C16" s="166" t="s">
         <v>47</v>
       </c>
-      <c r="D16" s="161"/>
+      <c r="D16" s="167"/>
       <c r="E16" s="34"/>
       <c r="F16" s="3"/>
-      <c r="G16" s="156"/>
+      <c r="G16" s="160"/>
       <c r="H16" s="13">
         <v>0.3</v>
       </c>
@@ -8555,15 +8555,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="2:34" ht="17" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="2:34" ht="17" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B17" s="3"/>
-      <c r="C17" s="160" t="s">
+      <c r="C17" s="166" t="s">
         <v>125</v>
       </c>
-      <c r="D17" s="161"/>
+      <c r="D17" s="167"/>
       <c r="E17" s="34"/>
       <c r="F17" s="3"/>
-      <c r="G17" s="156"/>
+      <c r="G17" s="160"/>
       <c r="H17" s="13">
         <v>0.25</v>
       </c>
@@ -8649,10 +8649,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:34" x14ac:dyDescent="0.2">
       <c r="B18" s="3"/>
-      <c r="C18" s="162"/>
-      <c r="D18" s="161"/>
+      <c r="C18" s="168"/>
+      <c r="D18" s="167"/>
       <c r="E18" s="34"/>
       <c r="F18" s="3"/>
       <c r="G18" s="3"/>
@@ -8728,27 +8728,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:34" x14ac:dyDescent="0.2">
       <c r="B19" s="3"/>
-      <c r="C19" s="162"/>
-      <c r="D19" s="161"/>
+      <c r="C19" s="168"/>
+      <c r="D19" s="167"/>
       <c r="E19" s="34"/>
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
       <c r="H19" s="3"/>
-      <c r="I19" s="165" t="s">
+      <c r="I19" s="154" t="s">
         <v>126</v>
       </c>
-      <c r="J19" s="165"/>
-      <c r="K19" s="165"/>
-      <c r="L19" s="165"/>
-      <c r="M19" s="165"/>
-      <c r="N19" s="165"/>
-      <c r="O19" s="165"/>
-      <c r="P19" s="165"/>
-      <c r="Q19" s="165"/>
-      <c r="R19" s="165"/>
-      <c r="S19" s="165"/>
+      <c r="J19" s="154"/>
+      <c r="K19" s="154"/>
+      <c r="L19" s="154"/>
+      <c r="M19" s="154"/>
+      <c r="N19" s="154"/>
+      <c r="O19" s="154"/>
+      <c r="P19" s="154"/>
+      <c r="Q19" s="154"/>
+      <c r="R19" s="154"/>
+      <c r="S19" s="154"/>
       <c r="T19" s="3"/>
       <c r="W19" s="53">
         <v>0.01</v>
@@ -8787,10 +8787,10 @@
         <v>75</v>
       </c>
     </row>
-    <row r="20" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:34" x14ac:dyDescent="0.2">
       <c r="B20" s="3"/>
-      <c r="C20" s="162"/>
-      <c r="D20" s="161"/>
+      <c r="C20" s="168"/>
+      <c r="D20" s="167"/>
       <c r="E20" s="34"/>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
@@ -8846,10 +8846,10 @@
         <v>150</v>
       </c>
     </row>
-    <row r="21" spans="2:34" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="2:34" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B21" s="3"/>
-      <c r="C21" s="163"/>
-      <c r="D21" s="164"/>
+      <c r="C21" s="169"/>
+      <c r="D21" s="170"/>
       <c r="E21" s="34"/>
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
@@ -8905,7 +8905,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="22" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:34" x14ac:dyDescent="0.2">
       <c r="B22" s="3"/>
       <c r="C22" s="33"/>
       <c r="D22" s="3"/>
@@ -8962,7 +8962,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="23" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:34" x14ac:dyDescent="0.2">
       <c r="B23" s="3"/>
       <c r="C23" s="33"/>
       <c r="D23" s="3"/>
@@ -9019,7 +9019,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="24" spans="2:34" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:34" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" s="3"/>
       <c r="C24" s="61" t="s">
         <v>8</v>
@@ -9029,20 +9029,20 @@
       <c r="F24" s="3"/>
       <c r="G24" s="3"/>
       <c r="H24" s="3"/>
-      <c r="I24" s="168" t="str">
+      <c r="I24" s="157" t="str">
         <f>_xlfn.CONCAT("Figure 2. Estimated Number of Severe Fetal Outcomes Under all Possible Immunity and Infection Rate Scenarios, based on ",D7," Pregnancies")</f>
         <v>Figure 2. Estimated Number of Severe Fetal Outcomes Under all Possible Immunity and Infection Rate Scenarios, based on 100000 Pregnancies</v>
       </c>
-      <c r="J24" s="168"/>
-      <c r="K24" s="168"/>
-      <c r="L24" s="168"/>
-      <c r="M24" s="168"/>
-      <c r="N24" s="168"/>
-      <c r="O24" s="168"/>
-      <c r="P24" s="168"/>
-      <c r="Q24" s="168"/>
-      <c r="R24" s="168"/>
-      <c r="S24" s="168"/>
+      <c r="J24" s="157"/>
+      <c r="K24" s="157"/>
+      <c r="L24" s="157"/>
+      <c r="M24" s="157"/>
+      <c r="N24" s="157"/>
+      <c r="O24" s="157"/>
+      <c r="P24" s="157"/>
+      <c r="Q24" s="157"/>
+      <c r="R24" s="157"/>
+      <c r="S24" s="157"/>
       <c r="T24" s="3"/>
       <c r="W24" s="53">
         <v>0.01</v>
@@ -9081,27 +9081,27 @@
         <v>450</v>
       </c>
     </row>
-    <row r="25" spans="2:34" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="25" spans="2:34" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B25" s="3"/>
-      <c r="C25" s="170" t="s">
+      <c r="C25" s="159" t="s">
         <v>24</v>
       </c>
-      <c r="D25" s="170"/>
+      <c r="D25" s="159"/>
       <c r="E25" s="45"/>
       <c r="F25" s="3"/>
       <c r="G25" s="3"/>
       <c r="H25" s="3"/>
-      <c r="I25" s="169"/>
-      <c r="J25" s="169"/>
-      <c r="K25" s="169"/>
-      <c r="L25" s="169"/>
-      <c r="M25" s="169"/>
-      <c r="N25" s="169"/>
-      <c r="O25" s="169"/>
-      <c r="P25" s="169"/>
-      <c r="Q25" s="169"/>
-      <c r="R25" s="169"/>
-      <c r="S25" s="169"/>
+      <c r="I25" s="158"/>
+      <c r="J25" s="158"/>
+      <c r="K25" s="158"/>
+      <c r="L25" s="158"/>
+      <c r="M25" s="158"/>
+      <c r="N25" s="158"/>
+      <c r="O25" s="158"/>
+      <c r="P25" s="158"/>
+      <c r="Q25" s="158"/>
+      <c r="R25" s="158"/>
+      <c r="S25" s="158"/>
       <c r="T25" s="3"/>
       <c r="W25" s="53">
         <v>0.01</v>
@@ -9140,13 +9140,13 @@
         <v>525</v>
       </c>
     </row>
-    <row r="26" spans="2:34" ht="34" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:34" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="3"/>
-      <c r="C26" s="170"/>
-      <c r="D26" s="170"/>
+      <c r="C26" s="159"/>
+      <c r="D26" s="159"/>
       <c r="E26" s="45"/>
       <c r="F26" s="3"/>
-      <c r="G26" s="156" t="s">
+      <c r="G26" s="160" t="s">
         <v>127</v>
       </c>
       <c r="H26" s="13">
@@ -9234,13 +9234,13 @@
         <v>600</v>
       </c>
     </row>
-    <row r="27" spans="2:34" s="8" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:34" s="8" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B27" s="3"/>
-      <c r="C27" s="170"/>
-      <c r="D27" s="170"/>
+      <c r="C27" s="159"/>
+      <c r="D27" s="159"/>
       <c r="E27" s="45"/>
       <c r="F27" s="33"/>
-      <c r="G27" s="156"/>
+      <c r="G27" s="160"/>
       <c r="H27" s="13">
         <v>0.9</v>
       </c>
@@ -9326,15 +9326,15 @@
         <v>675</v>
       </c>
     </row>
-    <row r="28" spans="2:34" s="8" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:34" s="8" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B28" s="3"/>
-      <c r="C28" s="170" t="s">
+      <c r="C28" s="159" t="s">
         <v>29</v>
       </c>
-      <c r="D28" s="170"/>
+      <c r="D28" s="159"/>
       <c r="E28" s="45"/>
       <c r="F28" s="33"/>
-      <c r="G28" s="156"/>
+      <c r="G28" s="160"/>
       <c r="H28" s="13">
         <v>0.8</v>
       </c>
@@ -9420,13 +9420,13 @@
         <v>750</v>
       </c>
     </row>
-    <row r="29" spans="2:34" s="8" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:34" s="8" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B29" s="33"/>
-      <c r="C29" s="170"/>
-      <c r="D29" s="170"/>
+      <c r="C29" s="159"/>
+      <c r="D29" s="159"/>
       <c r="E29" s="45"/>
       <c r="F29" s="33"/>
-      <c r="G29" s="156"/>
+      <c r="G29" s="160"/>
       <c r="H29" s="13">
         <v>0.7</v>
       </c>
@@ -9512,15 +9512,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="2:34" s="8" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:34" s="8" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B30" s="3"/>
-      <c r="C30" s="170" t="s">
+      <c r="C30" s="159" t="s">
         <v>28</v>
       </c>
-      <c r="D30" s="170"/>
+      <c r="D30" s="159"/>
       <c r="E30" s="45"/>
       <c r="F30" s="33"/>
-      <c r="G30" s="156"/>
+      <c r="G30" s="160"/>
       <c r="H30" s="13">
         <v>0.6</v>
       </c>
@@ -9606,13 +9606,13 @@
         <v>150</v>
       </c>
     </row>
-    <row r="31" spans="2:34" s="8" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:34" s="8" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B31" s="33"/>
-      <c r="C31" s="170"/>
-      <c r="D31" s="170"/>
+      <c r="C31" s="159"/>
+      <c r="D31" s="159"/>
       <c r="E31" s="45"/>
       <c r="F31" s="33"/>
-      <c r="G31" s="156"/>
+      <c r="G31" s="160"/>
       <c r="H31" s="13">
         <v>0.5</v>
       </c>
@@ -9698,15 +9698,15 @@
         <v>300</v>
       </c>
     </row>
-    <row r="32" spans="2:34" s="8" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:34" s="8" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B32" s="33"/>
-      <c r="C32" s="170" t="s">
+      <c r="C32" s="159" t="s">
         <v>26</v>
       </c>
-      <c r="D32" s="170"/>
+      <c r="D32" s="159"/>
       <c r="E32" s="45"/>
       <c r="F32" s="33"/>
-      <c r="G32" s="156"/>
+      <c r="G32" s="160"/>
       <c r="H32" s="13">
         <v>0.4</v>
       </c>
@@ -9792,13 +9792,13 @@
         <v>450</v>
       </c>
     </row>
-    <row r="33" spans="2:34" s="8" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:34" s="8" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B33" s="33"/>
-      <c r="C33" s="170"/>
-      <c r="D33" s="170"/>
+      <c r="C33" s="159"/>
+      <c r="D33" s="159"/>
       <c r="E33" s="45"/>
       <c r="F33" s="33"/>
-      <c r="G33" s="156"/>
+      <c r="G33" s="160"/>
       <c r="H33" s="13">
         <v>0.3</v>
       </c>
@@ -9884,15 +9884,15 @@
         <v>600</v>
       </c>
     </row>
-    <row r="34" spans="2:34" s="8" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:34" s="8" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B34" s="33"/>
-      <c r="C34" s="170" t="s">
+      <c r="C34" s="159" t="s">
         <v>27</v>
       </c>
-      <c r="D34" s="170"/>
+      <c r="D34" s="159"/>
       <c r="E34" s="45"/>
       <c r="F34" s="33"/>
-      <c r="G34" s="156"/>
+      <c r="G34" s="160"/>
       <c r="H34" s="13">
         <v>0.2</v>
       </c>
@@ -9978,13 +9978,13 @@
         <v>750</v>
       </c>
     </row>
-    <row r="35" spans="2:34" s="8" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:34" s="8" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B35" s="33"/>
-      <c r="C35" s="170"/>
-      <c r="D35" s="170"/>
+      <c r="C35" s="159"/>
+      <c r="D35" s="159"/>
       <c r="E35" s="45"/>
       <c r="F35" s="33"/>
-      <c r="G35" s="156"/>
+      <c r="G35" s="160"/>
       <c r="H35" s="13">
         <v>0.1</v>
       </c>
@@ -10070,13 +10070,13 @@
         <v>900</v>
       </c>
     </row>
-    <row r="36" spans="2:34" s="8" customFormat="1" ht="34" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="36" spans="2:34" s="8" customFormat="1" ht="34" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B36" s="33"/>
       <c r="C36" s="33"/>
       <c r="D36" s="33"/>
       <c r="E36" s="33"/>
       <c r="F36" s="33"/>
-      <c r="G36" s="156"/>
+      <c r="G36" s="160"/>
       <c r="H36" s="13">
         <v>0</v>
       </c>
@@ -10162,7 +10162,7 @@
         <v>1050</v>
       </c>
     </row>
-    <row r="37" spans="2:34" s="8" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:34" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B37" s="33"/>
       <c r="C37" s="33"/>
       <c r="D37" s="33"/>
@@ -10241,7 +10241,7 @@
         <v>1200</v>
       </c>
     </row>
-    <row r="38" spans="2:34" s="8" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:34" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B38" s="33"/>
       <c r="C38" s="33"/>
       <c r="D38" s="33"/>
@@ -10249,19 +10249,19 @@
       <c r="F38" s="33"/>
       <c r="G38" s="3"/>
       <c r="H38" s="3"/>
-      <c r="I38" s="165" t="s">
+      <c r="I38" s="154" t="s">
         <v>126</v>
       </c>
-      <c r="J38" s="165"/>
-      <c r="K38" s="165"/>
-      <c r="L38" s="165"/>
-      <c r="M38" s="165"/>
-      <c r="N38" s="165"/>
-      <c r="O38" s="165"/>
-      <c r="P38" s="165"/>
-      <c r="Q38" s="165"/>
-      <c r="R38" s="165"/>
-      <c r="S38" s="165"/>
+      <c r="J38" s="154"/>
+      <c r="K38" s="154"/>
+      <c r="L38" s="154"/>
+      <c r="M38" s="154"/>
+      <c r="N38" s="154"/>
+      <c r="O38" s="154"/>
+      <c r="P38" s="154"/>
+      <c r="Q38" s="154"/>
+      <c r="R38" s="154"/>
+      <c r="S38" s="154"/>
       <c r="T38" s="3"/>
       <c r="W38" s="53">
         <v>0.02</v>
@@ -10300,7 +10300,7 @@
         <v>1350</v>
       </c>
     </row>
-    <row r="39" spans="2:34" s="8" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:34" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B39" s="33"/>
       <c r="C39" s="33"/>
       <c r="D39" s="33"/>
@@ -10357,7 +10357,7 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="40" spans="2:34" s="8" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:34" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B40" s="33"/>
       <c r="C40" s="33"/>
       <c r="D40" s="33"/>
@@ -10414,7 +10414,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="2:34" s="8" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:34" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B41" s="33"/>
       <c r="C41" s="33"/>
       <c r="D41" s="33"/>
@@ -10471,7 +10471,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="42" spans="2:34" s="8" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:34" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="W42" s="53">
         <v>0.03</v>
       </c>
@@ -10509,7 +10509,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="43" spans="2:34" s="8" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:34" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="W43" s="53">
         <v>0.03</v>
       </c>
@@ -10547,7 +10547,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="44" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:34" x14ac:dyDescent="0.2">
       <c r="B44" s="8"/>
       <c r="C44" s="8"/>
       <c r="D44" s="8"/>
@@ -10589,7 +10589,7 @@
         <v>900</v>
       </c>
     </row>
-    <row r="45" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="45" spans="2:34" x14ac:dyDescent="0.2">
       <c r="W45" s="53">
         <v>0.03</v>
       </c>
@@ -10627,7 +10627,7 @@
         <v>1125</v>
       </c>
     </row>
-    <row r="46" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="46" spans="2:34" x14ac:dyDescent="0.2">
       <c r="W46" s="53">
         <v>0.03</v>
       </c>
@@ -10665,7 +10665,7 @@
         <v>1350</v>
       </c>
     </row>
-    <row r="47" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:34" x14ac:dyDescent="0.2">
       <c r="W47" s="53">
         <v>0.03</v>
       </c>
@@ -10703,7 +10703,7 @@
         <v>1575</v>
       </c>
     </row>
-    <row r="48" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:34" x14ac:dyDescent="0.2">
       <c r="W48" s="53">
         <v>0.03</v>
       </c>
@@ -10741,7 +10741,7 @@
         <v>1800</v>
       </c>
     </row>
-    <row r="49" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="49" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W49" s="53">
         <v>0.03</v>
       </c>
@@ -10779,7 +10779,7 @@
         <v>2025</v>
       </c>
     </row>
-    <row r="50" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="50" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W50" s="53">
         <v>0.03</v>
       </c>
@@ -10817,7 +10817,7 @@
         <v>2250</v>
       </c>
     </row>
-    <row r="51" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="51" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W51" s="53">
         <v>0.04</v>
       </c>
@@ -10855,7 +10855,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="52" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W52" s="53">
         <v>0.04</v>
       </c>
@@ -10893,7 +10893,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="53" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="53" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W53" s="53">
         <v>0.04</v>
       </c>
@@ -10931,7 +10931,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="54" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="54" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W54" s="53">
         <v>0.04</v>
       </c>
@@ -10969,7 +10969,7 @@
         <v>900</v>
       </c>
     </row>
-    <row r="55" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="55" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W55" s="53">
         <v>0.04</v>
       </c>
@@ -11007,7 +11007,7 @@
         <v>1200</v>
       </c>
     </row>
-    <row r="56" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="56" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W56" s="53">
         <v>0.04</v>
       </c>
@@ -11045,7 +11045,7 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="57" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="57" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W57" s="53">
         <v>0.04</v>
       </c>
@@ -11083,7 +11083,7 @@
         <v>1800</v>
       </c>
     </row>
-    <row r="58" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="58" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W58" s="53">
         <v>0.04</v>
       </c>
@@ -11121,7 +11121,7 @@
         <v>2100</v>
       </c>
     </row>
-    <row r="59" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="59" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W59" s="53">
         <v>0.04</v>
       </c>
@@ -11159,7 +11159,7 @@
         <v>2400</v>
       </c>
     </row>
-    <row r="60" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="60" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W60" s="53">
         <v>0.04</v>
       </c>
@@ -11197,7 +11197,7 @@
         <v>2700</v>
       </c>
     </row>
-    <row r="61" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="61" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W61" s="53">
         <v>0.04</v>
       </c>
@@ -11235,7 +11235,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="62" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="62" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W62" s="53">
         <v>0.05</v>
       </c>
@@ -11273,7 +11273,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="63" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W63" s="53">
         <v>0.05</v>
       </c>
@@ -11311,7 +11311,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="64" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="64" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W64" s="53">
         <v>0.05</v>
       </c>
@@ -11349,7 +11349,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="65" spans="14:34" x14ac:dyDescent="0.35">
+    <row r="65" spans="14:34" x14ac:dyDescent="0.2">
       <c r="W65" s="53">
         <v>0.05</v>
       </c>
@@ -11387,7 +11387,7 @@
         <v>1125</v>
       </c>
     </row>
-    <row r="66" spans="14:34" x14ac:dyDescent="0.35">
+    <row r="66" spans="14:34" x14ac:dyDescent="0.2">
       <c r="W66" s="53">
         <v>0.05</v>
       </c>
@@ -11425,8 +11425,8 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="67" spans="14:34" x14ac:dyDescent="0.35">
-      <c r="N67" s="166"/>
+    <row r="67" spans="14:34" x14ac:dyDescent="0.2">
+      <c r="N67" s="155"/>
       <c r="O67" s="10"/>
       <c r="P67" s="11"/>
       <c r="Q67" s="11"/>
@@ -11470,8 +11470,8 @@
         <v>1875</v>
       </c>
     </row>
-    <row r="68" spans="14:34" x14ac:dyDescent="0.35">
-      <c r="N68" s="166"/>
+    <row r="68" spans="14:34" x14ac:dyDescent="0.2">
+      <c r="N68" s="155"/>
       <c r="O68" s="10"/>
       <c r="P68" s="11"/>
       <c r="Q68" s="11"/>
@@ -11515,8 +11515,8 @@
         <v>2250</v>
       </c>
     </row>
-    <row r="69" spans="14:34" x14ac:dyDescent="0.35">
-      <c r="N69" s="166"/>
+    <row r="69" spans="14:34" x14ac:dyDescent="0.2">
+      <c r="N69" s="155"/>
       <c r="O69" s="10"/>
       <c r="P69" s="11"/>
       <c r="Q69" s="11"/>
@@ -11560,8 +11560,8 @@
         <v>2625</v>
       </c>
     </row>
-    <row r="70" spans="14:34" x14ac:dyDescent="0.35">
-      <c r="N70" s="166"/>
+    <row r="70" spans="14:34" x14ac:dyDescent="0.2">
+      <c r="N70" s="155"/>
       <c r="O70" s="10"/>
       <c r="P70" s="11"/>
       <c r="Q70" s="11"/>
@@ -11605,8 +11605,8 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="71" spans="14:34" x14ac:dyDescent="0.35">
-      <c r="N71" s="166"/>
+    <row r="71" spans="14:34" x14ac:dyDescent="0.2">
+      <c r="N71" s="155"/>
       <c r="O71" s="10"/>
       <c r="P71" s="11"/>
       <c r="Q71" s="11"/>
@@ -11650,7 +11650,7 @@
         <v>3375</v>
       </c>
     </row>
-    <row r="72" spans="14:34" x14ac:dyDescent="0.35">
+    <row r="72" spans="14:34" x14ac:dyDescent="0.2">
       <c r="P72" s="12"/>
       <c r="Q72" s="12"/>
       <c r="R72" s="12"/>
@@ -11693,12 +11693,12 @@
         <v>3750</v>
       </c>
     </row>
-    <row r="73" spans="14:34" x14ac:dyDescent="0.35">
-      <c r="P73" s="167"/>
-      <c r="Q73" s="167"/>
-      <c r="R73" s="167"/>
-      <c r="S73" s="167"/>
-      <c r="T73" s="167"/>
+    <row r="73" spans="14:34" x14ac:dyDescent="0.2">
+      <c r="P73" s="156"/>
+      <c r="Q73" s="156"/>
+      <c r="R73" s="156"/>
+      <c r="S73" s="156"/>
+      <c r="T73" s="156"/>
       <c r="W73" s="53">
         <v>0.06</v>
       </c>
@@ -11736,7 +11736,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="14:34" x14ac:dyDescent="0.35">
+    <row r="74" spans="14:34" x14ac:dyDescent="0.2">
       <c r="W74" s="53">
         <v>0.06</v>
       </c>
@@ -11774,7 +11774,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="75" spans="14:34" x14ac:dyDescent="0.35">
+    <row r="75" spans="14:34" x14ac:dyDescent="0.2">
       <c r="W75" s="53">
         <v>0.06</v>
       </c>
@@ -11812,7 +11812,7 @@
         <v>900</v>
       </c>
     </row>
-    <row r="76" spans="14:34" x14ac:dyDescent="0.35">
+    <row r="76" spans="14:34" x14ac:dyDescent="0.2">
       <c r="W76" s="53">
         <v>0.06</v>
       </c>
@@ -11850,7 +11850,7 @@
         <v>1350</v>
       </c>
     </row>
-    <row r="77" spans="14:34" x14ac:dyDescent="0.35">
+    <row r="77" spans="14:34" x14ac:dyDescent="0.2">
       <c r="W77" s="53">
         <v>0.06</v>
       </c>
@@ -11888,7 +11888,7 @@
         <v>1800</v>
       </c>
     </row>
-    <row r="78" spans="14:34" x14ac:dyDescent="0.35">
+    <row r="78" spans="14:34" x14ac:dyDescent="0.2">
       <c r="W78" s="53">
         <v>0.06</v>
       </c>
@@ -11926,7 +11926,7 @@
         <v>2250</v>
       </c>
     </row>
-    <row r="79" spans="14:34" x14ac:dyDescent="0.35">
+    <row r="79" spans="14:34" x14ac:dyDescent="0.2">
       <c r="W79" s="53">
         <v>0.06</v>
       </c>
@@ -11964,7 +11964,7 @@
         <v>2700</v>
       </c>
     </row>
-    <row r="80" spans="14:34" x14ac:dyDescent="0.35">
+    <row r="80" spans="14:34" x14ac:dyDescent="0.2">
       <c r="W80" s="53">
         <v>0.06</v>
       </c>
@@ -12002,7 +12002,7 @@
         <v>3150</v>
       </c>
     </row>
-    <row r="81" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="81" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W81" s="53">
         <v>0.06</v>
       </c>
@@ -12040,7 +12040,7 @@
         <v>3600</v>
       </c>
     </row>
-    <row r="82" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="82" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W82" s="53">
         <v>0.06</v>
       </c>
@@ -12078,7 +12078,7 @@
         <v>4050</v>
       </c>
     </row>
-    <row r="83" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="83" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W83" s="53">
         <v>0.06</v>
       </c>
@@ -12116,7 +12116,7 @@
         <v>4500</v>
       </c>
     </row>
-    <row r="84" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="84" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W84" s="53">
         <v>7.0000000000000007E-2</v>
       </c>
@@ -12154,7 +12154,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="85" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W85" s="53">
         <v>7.0000000000000007E-2</v>
       </c>
@@ -12192,7 +12192,7 @@
         <v>525</v>
       </c>
     </row>
-    <row r="86" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="86" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W86" s="53">
         <v>7.0000000000000007E-2</v>
       </c>
@@ -12230,7 +12230,7 @@
         <v>1050</v>
       </c>
     </row>
-    <row r="87" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="87" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W87" s="53">
         <v>7.0000000000000007E-2</v>
       </c>
@@ -12268,7 +12268,7 @@
         <v>1575</v>
       </c>
     </row>
-    <row r="88" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="88" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W88" s="53">
         <v>7.0000000000000007E-2</v>
       </c>
@@ -12306,7 +12306,7 @@
         <v>2100</v>
       </c>
     </row>
-    <row r="89" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="89" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W89" s="53">
         <v>7.0000000000000007E-2</v>
       </c>
@@ -12344,7 +12344,7 @@
         <v>2625</v>
       </c>
     </row>
-    <row r="90" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="90" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W90" s="53">
         <v>7.0000000000000007E-2</v>
       </c>
@@ -12382,7 +12382,7 @@
         <v>3150</v>
       </c>
     </row>
-    <row r="91" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="91" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W91" s="53">
         <v>7.0000000000000007E-2</v>
       </c>
@@ -12420,7 +12420,7 @@
         <v>3675</v>
       </c>
     </row>
-    <row r="92" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="92" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W92" s="53">
         <v>7.0000000000000007E-2</v>
       </c>
@@ -12458,7 +12458,7 @@
         <v>4200</v>
       </c>
     </row>
-    <row r="93" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="93" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W93" s="53">
         <v>7.0000000000000007E-2</v>
       </c>
@@ -12496,7 +12496,7 @@
         <v>4724.9999999999991</v>
       </c>
     </row>
-    <row r="94" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="94" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W94" s="53">
         <v>7.0000000000000007E-2</v>
       </c>
@@ -12534,7 +12534,7 @@
         <v>5250</v>
       </c>
     </row>
-    <row r="95" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="95" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W95" s="53">
         <v>0.08</v>
       </c>
@@ -12572,7 +12572,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="96" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W96" s="53">
         <v>0.08</v>
       </c>
@@ -12610,7 +12610,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="97" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="97" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W97" s="53">
         <v>0.08</v>
       </c>
@@ -12648,7 +12648,7 @@
         <v>1200</v>
       </c>
     </row>
-    <row r="98" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="98" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W98" s="53">
         <v>0.08</v>
       </c>
@@ -12686,7 +12686,7 @@
         <v>1800</v>
       </c>
     </row>
-    <row r="99" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="99" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W99" s="53">
         <v>0.08</v>
       </c>
@@ -12724,7 +12724,7 @@
         <v>2400</v>
       </c>
     </row>
-    <row r="100" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="100" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W100" s="53">
         <v>0.08</v>
       </c>
@@ -12762,7 +12762,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="101" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="101" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W101" s="53">
         <v>0.08</v>
       </c>
@@ -12800,7 +12800,7 @@
         <v>3600</v>
       </c>
     </row>
-    <row r="102" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="102" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W102" s="53">
         <v>0.08</v>
       </c>
@@ -12838,7 +12838,7 @@
         <v>4200</v>
       </c>
     </row>
-    <row r="103" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="103" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W103" s="53">
         <v>0.08</v>
       </c>
@@ -12876,7 +12876,7 @@
         <v>4800</v>
       </c>
     </row>
-    <row r="104" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="104" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W104" s="53">
         <v>0.08</v>
       </c>
@@ -12914,7 +12914,7 @@
         <v>5400</v>
       </c>
     </row>
-    <row r="105" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="105" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W105" s="53">
         <v>0.08</v>
       </c>
@@ -12952,7 +12952,7 @@
         <v>6000</v>
       </c>
     </row>
-    <row r="106" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="106" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W106" s="53">
         <v>0.09</v>
       </c>
@@ -12990,7 +12990,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="107" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W107" s="53">
         <v>0.09</v>
       </c>
@@ -13028,7 +13028,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="108" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="108" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W108" s="53">
         <v>0.09</v>
       </c>
@@ -13066,7 +13066,7 @@
         <v>1350</v>
       </c>
     </row>
-    <row r="109" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="109" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W109" s="53">
         <v>0.09</v>
       </c>
@@ -13104,7 +13104,7 @@
         <v>2025</v>
       </c>
     </row>
-    <row r="110" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="110" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W110" s="53">
         <v>0.09</v>
       </c>
@@ -13142,7 +13142,7 @@
         <v>2700</v>
       </c>
     </row>
-    <row r="111" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="111" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W111" s="53">
         <v>0.09</v>
       </c>
@@ -13180,7 +13180,7 @@
         <v>3375</v>
       </c>
     </row>
-    <row r="112" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="112" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W112" s="53">
         <v>0.09</v>
       </c>
@@ -13218,7 +13218,7 @@
         <v>4050</v>
       </c>
     </row>
-    <row r="113" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="113" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W113" s="53">
         <v>0.09</v>
       </c>
@@ -13256,7 +13256,7 @@
         <v>4725</v>
       </c>
     </row>
-    <row r="114" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="114" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W114" s="53">
         <v>0.09</v>
       </c>
@@ -13294,7 +13294,7 @@
         <v>5400</v>
       </c>
     </row>
-    <row r="115" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="115" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W115" s="53">
         <v>0.09</v>
       </c>
@@ -13332,7 +13332,7 @@
         <v>6075</v>
       </c>
     </row>
-    <row r="116" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="116" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W116" s="53">
         <v>0.09</v>
       </c>
@@ -13370,7 +13370,7 @@
         <v>6750</v>
       </c>
     </row>
-    <row r="117" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="117" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W117" s="53">
         <v>0.1</v>
       </c>
@@ -13408,7 +13408,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="118" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W118" s="53">
         <v>0.1</v>
       </c>
@@ -13446,7 +13446,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="119" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="119" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W119" s="53">
         <v>0.1</v>
       </c>
@@ -13484,7 +13484,7 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="120" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="120" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W120" s="53">
         <v>0.1</v>
       </c>
@@ -13522,7 +13522,7 @@
         <v>2250</v>
       </c>
     </row>
-    <row r="121" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="121" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W121" s="53">
         <v>0.1</v>
       </c>
@@ -13560,7 +13560,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="122" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="122" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W122" s="53">
         <v>0.1</v>
       </c>
@@ -13598,7 +13598,7 @@
         <v>3750</v>
       </c>
     </row>
-    <row r="123" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="123" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W123" s="53">
         <v>0.1</v>
       </c>
@@ -13636,7 +13636,7 @@
         <v>4500</v>
       </c>
     </row>
-    <row r="124" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="124" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W124" s="53">
         <v>0.1</v>
       </c>
@@ -13674,7 +13674,7 @@
         <v>5250</v>
       </c>
     </row>
-    <row r="125" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="125" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W125" s="53">
         <v>0.1</v>
       </c>
@@ -13712,7 +13712,7 @@
         <v>6000</v>
       </c>
     </row>
-    <row r="126" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="126" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W126" s="53">
         <v>0.1</v>
       </c>
@@ -13750,7 +13750,7 @@
         <v>6750</v>
       </c>
     </row>
-    <row r="127" spans="23:34" x14ac:dyDescent="0.35">
+    <row r="127" spans="23:34" x14ac:dyDescent="0.2">
       <c r="W127" s="53">
         <v>0.1</v>
       </c>
@@ -13789,8 +13789,15 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
+  <sheetProtection selectLockedCells="1"/>
   <mergeCells count="17">
+    <mergeCell ref="C3:S3"/>
+    <mergeCell ref="I5:S6"/>
+    <mergeCell ref="G7:G17"/>
+    <mergeCell ref="C14:D15"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="C17:D21"/>
+    <mergeCell ref="I19:S19"/>
     <mergeCell ref="I38:S38"/>
     <mergeCell ref="N67:N71"/>
     <mergeCell ref="P73:T73"/>
@@ -13801,13 +13808,6 @@
     <mergeCell ref="C30:D31"/>
     <mergeCell ref="C32:D33"/>
     <mergeCell ref="C34:D35"/>
-    <mergeCell ref="C3:S3"/>
-    <mergeCell ref="I5:S6"/>
-    <mergeCell ref="G7:G17"/>
-    <mergeCell ref="C14:D15"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="C17:D21"/>
-    <mergeCell ref="I19:S19"/>
   </mergeCells>
   <conditionalFormatting sqref="I7:S17">
     <cfRule type="colorScale" priority="1">
@@ -13864,14 +13864,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{249F9FEB-B6AE-4640-A09E-8C130E6BDF68}">
   <dimension ref="B4:M66"/>
-  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="8.6328125" style="2"/>
-    <col min="3" max="12" width="16.81640625" style="2" customWidth="1"/>
-    <col min="13" max="16384" width="8.6328125" style="2"/>
+    <col min="1" max="2" width="8.6640625" style="2"/>
+    <col min="3" max="12" width="16.83203125" style="2" customWidth="1"/>
+    <col min="13" max="16384" width="8.6640625" style="2"/>
   </cols>
   <sheetData>
-    <row r="4" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B4" s="143"/>
       <c r="C4" s="143"/>
       <c r="D4" s="143"/>
@@ -13885,7 +13885,7 @@
       <c r="L4" s="143"/>
       <c r="M4" s="143"/>
     </row>
-    <row r="5" spans="2:13" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:13" ht="19" x14ac:dyDescent="0.25">
       <c r="B5" s="171" t="s">
         <v>96</v>
       </c>
@@ -13901,7 +13901,7 @@
       <c r="L5" s="171"/>
       <c r="M5" s="171"/>
     </row>
-    <row r="6" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
@@ -13915,7 +13915,7 @@
       <c r="L6" s="3"/>
       <c r="M6" s="3"/>
     </row>
-    <row r="7" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B7" s="66"/>
       <c r="C7" s="65"/>
       <c r="D7" s="66"/>
@@ -13929,7 +13929,7 @@
       <c r="L7" s="66"/>
       <c r="M7" s="66"/>
     </row>
-    <row r="8" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B8" s="3"/>
       <c r="C8" s="62" t="s">
         <v>50</v>
@@ -13945,7 +13945,7 @@
       <c r="L8" s="3"/>
       <c r="M8" s="3"/>
     </row>
-    <row r="9" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B9" s="3"/>
       <c r="C9" s="62" t="s">
         <v>148</v>
@@ -13961,7 +13961,7 @@
       <c r="L9" s="3"/>
       <c r="M9" s="3"/>
     </row>
-    <row r="10" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B10" s="3"/>
       <c r="C10" s="62" t="s">
         <v>51</v>
@@ -13977,7 +13977,7 @@
       <c r="L10" s="3"/>
       <c r="M10" s="3"/>
     </row>
-    <row r="11" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B11" s="3"/>
       <c r="C11" s="62" t="s">
         <v>52</v>
@@ -13993,7 +13993,7 @@
       <c r="L11" s="3"/>
       <c r="M11" s="3"/>
     </row>
-    <row r="12" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B12" s="3"/>
       <c r="C12" s="137" t="s">
         <v>53</v>
@@ -14009,7 +14009,7 @@
       <c r="L12" s="3"/>
       <c r="M12" s="3"/>
     </row>
-    <row r="13" spans="2:13" ht="63.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:13" ht="63.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="3"/>
       <c r="C13" s="172" t="s">
         <v>54</v>
@@ -14025,7 +14025,7 @@
       <c r="L13" s="172"/>
       <c r="M13" s="3"/>
     </row>
-    <row r="14" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B14" s="3"/>
       <c r="C14" s="62" t="s">
         <v>55</v>
@@ -14041,7 +14041,7 @@
       <c r="L14" s="3"/>
       <c r="M14" s="3"/>
     </row>
-    <row r="15" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B15" s="3"/>
       <c r="C15" s="63" t="s">
         <v>56</v>
@@ -14057,7 +14057,7 @@
       <c r="L15" s="3"/>
       <c r="M15" s="3"/>
     </row>
-    <row r="16" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B16" s="3"/>
       <c r="C16" s="63" t="s">
         <v>57</v>
@@ -14073,7 +14073,7 @@
       <c r="L16" s="3"/>
       <c r="M16" s="3"/>
     </row>
-    <row r="17" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B17" s="3"/>
       <c r="C17" s="63" t="s">
         <v>58</v>
@@ -14089,7 +14089,7 @@
       <c r="L17" s="3"/>
       <c r="M17" s="3"/>
     </row>
-    <row r="18" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B18" s="3"/>
       <c r="C18" s="63" t="s">
         <v>59</v>
@@ -14105,7 +14105,7 @@
       <c r="L18" s="3"/>
       <c r="M18" s="3"/>
     </row>
-    <row r="19" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B19" s="3"/>
       <c r="C19" s="63"/>
       <c r="D19" s="3"/>
@@ -14119,7 +14119,7 @@
       <c r="L19" s="3"/>
       <c r="M19" s="3"/>
     </row>
-    <row r="20" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B20" s="66"/>
       <c r="C20" s="67"/>
       <c r="D20" s="66"/>
@@ -14133,7 +14133,7 @@
       <c r="L20" s="66"/>
       <c r="M20" s="66"/>
     </row>
-    <row r="21" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B21" s="3"/>
       <c r="C21" s="62" t="s">
         <v>60</v>
@@ -14149,7 +14149,7 @@
       <c r="L21" s="3"/>
       <c r="M21" s="3"/>
     </row>
-    <row r="22" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B22" s="3"/>
       <c r="C22" s="62" t="s">
         <v>95</v>
@@ -14165,7 +14165,7 @@
       <c r="L22" s="3"/>
       <c r="M22" s="3"/>
     </row>
-    <row r="23" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B23" s="3"/>
       <c r="C23" s="62" t="s">
         <v>61</v>
@@ -14181,7 +14181,7 @@
       <c r="L23" s="3"/>
       <c r="M23" s="3"/>
     </row>
-    <row r="24" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B24" s="3"/>
       <c r="C24" s="62" t="s">
         <v>62</v>
@@ -14197,7 +14197,7 @@
       <c r="L24" s="3"/>
       <c r="M24" s="3"/>
     </row>
-    <row r="25" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B25" s="3"/>
       <c r="C25" s="137" t="s">
         <v>63</v>
@@ -14213,7 +14213,7 @@
       <c r="L25" s="3"/>
       <c r="M25" s="3"/>
     </row>
-    <row r="26" spans="2:13" ht="60.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:13" ht="60.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="3"/>
       <c r="C26" s="172" t="s">
         <v>64</v>
@@ -14229,7 +14229,7 @@
       <c r="L26" s="172"/>
       <c r="M26" s="3"/>
     </row>
-    <row r="27" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B27" s="3"/>
       <c r="C27" s="62" t="s">
         <v>65</v>
@@ -14245,7 +14245,7 @@
       <c r="L27" s="3"/>
       <c r="M27" s="3"/>
     </row>
-    <row r="28" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B28" s="3"/>
       <c r="C28" s="63" t="s">
         <v>66</v>
@@ -14261,7 +14261,7 @@
       <c r="L28" s="3"/>
       <c r="M28" s="3"/>
     </row>
-    <row r="29" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B29" s="3"/>
       <c r="C29" s="63" t="s">
         <v>67</v>
@@ -14277,7 +14277,7 @@
       <c r="L29" s="3"/>
       <c r="M29" s="3"/>
     </row>
-    <row r="30" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B30" s="3"/>
       <c r="C30" s="63"/>
       <c r="D30" s="3"/>
@@ -14291,7 +14291,7 @@
       <c r="L30" s="3"/>
       <c r="M30" s="3"/>
     </row>
-    <row r="31" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B31" s="66"/>
       <c r="C31" s="67"/>
       <c r="D31" s="66"/>
@@ -14305,7 +14305,7 @@
       <c r="L31" s="66"/>
       <c r="M31" s="66"/>
     </row>
-    <row r="32" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B32" s="3"/>
       <c r="C32" s="62" t="s">
         <v>68</v>
@@ -14321,7 +14321,7 @@
       <c r="L32" s="3"/>
       <c r="M32" s="3"/>
     </row>
-    <row r="33" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B33" s="3"/>
       <c r="C33" s="62" t="s">
         <v>94</v>
@@ -14337,7 +14337,7 @@
       <c r="L33" s="3"/>
       <c r="M33" s="3"/>
     </row>
-    <row r="34" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B34" s="3"/>
       <c r="C34" s="62" t="s">
         <v>69</v>
@@ -14353,7 +14353,7 @@
       <c r="L34" s="3"/>
       <c r="M34" s="3"/>
     </row>
-    <row r="35" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B35" s="3"/>
       <c r="C35" s="62" t="s">
         <v>70</v>
@@ -14369,7 +14369,7 @@
       <c r="L35" s="3"/>
       <c r="M35" s="3"/>
     </row>
-    <row r="36" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B36" s="3"/>
       <c r="C36" s="137" t="s">
         <v>71</v>
@@ -14385,7 +14385,7 @@
       <c r="L36" s="3"/>
       <c r="M36" s="3"/>
     </row>
-    <row r="37" spans="2:13" ht="51.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:13" ht="51.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B37" s="3"/>
       <c r="C37" s="172" t="s">
         <v>72</v>
@@ -14401,7 +14401,7 @@
       <c r="L37" s="172"/>
       <c r="M37" s="3"/>
     </row>
-    <row r="38" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B38" s="3"/>
       <c r="C38" s="62" t="s">
         <v>65</v>
@@ -14417,7 +14417,7 @@
       <c r="L38" s="3"/>
       <c r="M38" s="3"/>
     </row>
-    <row r="39" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B39" s="3"/>
       <c r="C39" s="63" t="s">
         <v>73</v>
@@ -14433,7 +14433,7 @@
       <c r="L39" s="3"/>
       <c r="M39" s="3"/>
     </row>
-    <row r="40" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B40" s="3"/>
       <c r="C40" s="63" t="s">
         <v>74</v>
@@ -14449,7 +14449,7 @@
       <c r="L40" s="3"/>
       <c r="M40" s="3"/>
     </row>
-    <row r="41" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B41" s="3"/>
       <c r="C41" s="64"/>
       <c r="D41" s="3"/>
@@ -14463,7 +14463,7 @@
       <c r="L41" s="3"/>
       <c r="M41" s="3"/>
     </row>
-    <row r="42" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B42" s="66"/>
       <c r="C42" s="67"/>
       <c r="D42" s="66"/>
@@ -14477,7 +14477,7 @@
       <c r="L42" s="66"/>
       <c r="M42" s="66"/>
     </row>
-    <row r="43" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B43" s="3"/>
       <c r="C43" s="62" t="s">
         <v>75</v>
@@ -14493,7 +14493,7 @@
       <c r="L43" s="3"/>
       <c r="M43" s="3"/>
     </row>
-    <row r="44" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B44" s="3"/>
       <c r="C44" s="62" t="s">
         <v>93</v>
@@ -14509,7 +14509,7 @@
       <c r="L44" s="3"/>
       <c r="M44" s="3"/>
     </row>
-    <row r="45" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="45" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B45" s="3"/>
       <c r="C45" s="62" t="s">
         <v>76</v>
@@ -14525,7 +14525,7 @@
       <c r="L45" s="3"/>
       <c r="M45" s="3"/>
     </row>
-    <row r="46" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="46" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B46" s="3"/>
       <c r="C46" s="62" t="s">
         <v>77</v>
@@ -14541,7 +14541,7 @@
       <c r="L46" s="3"/>
       <c r="M46" s="3"/>
     </row>
-    <row r="47" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B47" s="3"/>
       <c r="C47" s="137" t="s">
         <v>78</v>
@@ -14557,7 +14557,7 @@
       <c r="L47" s="138"/>
       <c r="M47" s="3"/>
     </row>
-    <row r="48" spans="2:13" ht="54.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:13" ht="54.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B48" s="3"/>
       <c r="C48" s="172" t="s">
         <v>79</v>
@@ -14573,7 +14573,7 @@
       <c r="L48" s="172"/>
       <c r="M48" s="3"/>
     </row>
-    <row r="49" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="49" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B49" s="3"/>
       <c r="C49" s="62" t="s">
         <v>65</v>
@@ -14589,7 +14589,7 @@
       <c r="L49" s="3"/>
       <c r="M49" s="3"/>
     </row>
-    <row r="50" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="50" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B50" s="3"/>
       <c r="C50" s="63" t="s">
         <v>80</v>
@@ -14605,7 +14605,7 @@
       <c r="L50" s="64"/>
       <c r="M50" s="3"/>
     </row>
-    <row r="51" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="51" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B51" s="3"/>
       <c r="C51" s="63" t="s">
         <v>81</v>
@@ -14621,7 +14621,7 @@
       <c r="L51" s="3"/>
       <c r="M51" s="3"/>
     </row>
-    <row r="52" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="52" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B52" s="3"/>
       <c r="C52" s="64"/>
       <c r="D52" s="3"/>
@@ -14635,7 +14635,7 @@
       <c r="L52" s="3"/>
       <c r="M52" s="3"/>
     </row>
-    <row r="53" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="53" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B53" s="66"/>
       <c r="C53" s="67"/>
       <c r="D53" s="66"/>
@@ -14649,7 +14649,7 @@
       <c r="L53" s="66"/>
       <c r="M53" s="66"/>
     </row>
-    <row r="54" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="54" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B54" s="3"/>
       <c r="C54" s="62" t="s">
         <v>82</v>
@@ -14665,7 +14665,7 @@
       <c r="L54" s="3"/>
       <c r="M54" s="3"/>
     </row>
-    <row r="55" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="55" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B55" s="3"/>
       <c r="C55" s="62" t="s">
         <v>92</v>
@@ -14681,7 +14681,7 @@
       <c r="L55" s="3"/>
       <c r="M55" s="3"/>
     </row>
-    <row r="56" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="56" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B56" s="3"/>
       <c r="C56" s="62" t="s">
         <v>83</v>
@@ -14697,7 +14697,7 @@
       <c r="L56" s="3"/>
       <c r="M56" s="3"/>
     </row>
-    <row r="57" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="57" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B57" s="3"/>
       <c r="C57" s="62" t="s">
         <v>84</v>
@@ -14713,7 +14713,7 @@
       <c r="L57" s="3"/>
       <c r="M57" s="3"/>
     </row>
-    <row r="58" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="58" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B58" s="3"/>
       <c r="C58" s="137" t="s">
         <v>85</v>
@@ -14729,7 +14729,7 @@
       <c r="L58" s="3"/>
       <c r="M58" s="3"/>
     </row>
-    <row r="59" spans="2:13" ht="38.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="2:13" ht="38.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B59" s="3"/>
       <c r="C59" s="172" t="s">
         <v>91</v>
@@ -14745,7 +14745,7 @@
       <c r="L59" s="172"/>
       <c r="M59" s="3"/>
     </row>
-    <row r="60" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="60" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B60" s="3"/>
       <c r="C60" s="62" t="s">
         <v>55</v>
@@ -14761,7 +14761,7 @@
       <c r="L60" s="3"/>
       <c r="M60" s="3"/>
     </row>
-    <row r="61" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="61" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B61" s="3"/>
       <c r="C61" s="63" t="s">
         <v>86</v>
@@ -14777,7 +14777,7 @@
       <c r="L61" s="3"/>
       <c r="M61" s="3"/>
     </row>
-    <row r="62" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="62" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B62" s="3"/>
       <c r="C62" s="63" t="s">
         <v>87</v>
@@ -14793,7 +14793,7 @@
       <c r="L62" s="3"/>
       <c r="M62" s="3"/>
     </row>
-    <row r="63" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="63" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B63" s="3"/>
       <c r="C63" s="63" t="s">
         <v>88</v>
@@ -14809,7 +14809,7 @@
       <c r="L63" s="3"/>
       <c r="M63" s="3"/>
     </row>
-    <row r="64" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="64" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B64" s="3"/>
       <c r="C64" s="63" t="s">
         <v>89</v>
@@ -14825,7 +14825,7 @@
       <c r="L64" s="3"/>
       <c r="M64" s="3"/>
     </row>
-    <row r="65" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="65" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B65" s="3"/>
       <c r="C65" s="63" t="s">
         <v>90</v>
@@ -14841,7 +14841,7 @@
       <c r="L65" s="3"/>
       <c r="M65" s="3"/>
     </row>
-    <row r="66" spans="2:13" ht="16" x14ac:dyDescent="0.35">
+    <row r="66" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B66" s="3"/>
       <c r="C66" s="64"/>
       <c r="D66" s="3"/>
@@ -14856,7 +14856,7 @@
       <c r="M66" s="3"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
+  <sheetProtection selectLockedCells="1"/>
   <mergeCells count="6">
     <mergeCell ref="B5:M5"/>
     <mergeCell ref="C13:L13"/>
@@ -14879,16 +14879,16 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F9F18BA-B2E7-43D9-945E-E619C416C78E}">
   <dimension ref="B4:M35"/>
-  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="8.6328125" style="2"/>
+    <col min="1" max="2" width="8.6640625" style="2"/>
     <col min="3" max="3" width="5" style="2" customWidth="1"/>
-    <col min="4" max="12" width="12.453125" style="2" customWidth="1"/>
-    <col min="13" max="13" width="7.453125" style="2" customWidth="1"/>
-    <col min="14" max="16384" width="8.6328125" style="2"/>
+    <col min="4" max="12" width="12.5" style="2" customWidth="1"/>
+    <col min="13" max="13" width="7.5" style="2" customWidth="1"/>
+    <col min="14" max="16384" width="8.6640625" style="2"/>
   </cols>
   <sheetData>
-    <row r="4" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
@@ -14902,7 +14902,7 @@
       <c r="L4" s="3"/>
       <c r="M4" s="3"/>
     </row>
-    <row r="5" spans="2:13" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:13" ht="19" x14ac:dyDescent="0.25">
       <c r="B5" s="3"/>
       <c r="C5" s="171" t="s">
         <v>48</v>
@@ -14918,7 +14918,7 @@
       <c r="L5" s="171"/>
       <c r="M5" s="3"/>
     </row>
-    <row r="6" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
@@ -14932,7 +14932,7 @@
       <c r="L6" s="3"/>
       <c r="M6" s="3"/>
     </row>
-    <row r="7" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B7" s="66"/>
       <c r="C7" s="139" t="s">
         <v>44</v>
@@ -14948,7 +14948,7 @@
       <c r="L7" s="66"/>
       <c r="M7" s="66"/>
     </row>
-    <row r="8" spans="2:13" ht="30.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:13" ht="30.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
       <c r="D8" s="173" t="s">
@@ -14964,7 +14964,7 @@
       <c r="L8" s="173"/>
       <c r="M8" s="3"/>
     </row>
-    <row r="9" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
@@ -14978,23 +14978,23 @@
       <c r="L9" s="3"/>
       <c r="M9" s="3"/>
     </row>
-    <row r="10" spans="2:13" ht="31" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:13" ht="31" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
-      <c r="D10" s="144" t="s">
+      <c r="D10" s="146" t="s">
         <v>146</v>
       </c>
-      <c r="E10" s="144"/>
-      <c r="F10" s="144"/>
-      <c r="G10" s="144"/>
-      <c r="H10" s="144"/>
-      <c r="I10" s="144"/>
-      <c r="J10" s="144"/>
-      <c r="K10" s="144"/>
-      <c r="L10" s="144"/>
+      <c r="E10" s="146"/>
+      <c r="F10" s="146"/>
+      <c r="G10" s="146"/>
+      <c r="H10" s="146"/>
+      <c r="I10" s="146"/>
+      <c r="J10" s="146"/>
+      <c r="K10" s="146"/>
+      <c r="L10" s="146"/>
       <c r="M10" s="3"/>
     </row>
-    <row r="11" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
       <c r="D11" s="34"/>
@@ -15008,23 +15008,23 @@
       <c r="L11" s="34"/>
       <c r="M11" s="3"/>
     </row>
-    <row r="12" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
-      <c r="D12" s="144" t="s">
+      <c r="D12" s="146" t="s">
         <v>101</v>
       </c>
-      <c r="E12" s="144"/>
-      <c r="F12" s="144"/>
-      <c r="G12" s="144"/>
-      <c r="H12" s="144"/>
-      <c r="I12" s="144"/>
-      <c r="J12" s="144"/>
-      <c r="K12" s="144"/>
-      <c r="L12" s="144"/>
+      <c r="E12" s="146"/>
+      <c r="F12" s="146"/>
+      <c r="G12" s="146"/>
+      <c r="H12" s="146"/>
+      <c r="I12" s="146"/>
+      <c r="J12" s="146"/>
+      <c r="K12" s="146"/>
+      <c r="L12" s="146"/>
       <c r="M12" s="3"/>
     </row>
-    <row r="13" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>
@@ -15038,23 +15038,23 @@
       <c r="L13" s="3"/>
       <c r="M13" s="3"/>
     </row>
-    <row r="14" spans="2:13" ht="45.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:13" ht="45.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
-      <c r="D14" s="144" t="s">
+      <c r="D14" s="146" t="s">
         <v>129</v>
       </c>
-      <c r="E14" s="144"/>
-      <c r="F14" s="144"/>
-      <c r="G14" s="144"/>
-      <c r="H14" s="144"/>
-      <c r="I14" s="144"/>
-      <c r="J14" s="144"/>
-      <c r="K14" s="144"/>
-      <c r="L14" s="144"/>
+      <c r="E14" s="146"/>
+      <c r="F14" s="146"/>
+      <c r="G14" s="146"/>
+      <c r="H14" s="146"/>
+      <c r="I14" s="146"/>
+      <c r="J14" s="146"/>
+      <c r="K14" s="146"/>
+      <c r="L14" s="146"/>
       <c r="M14" s="3"/>
     </row>
-    <row r="15" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
       <c r="D15" s="3"/>
@@ -15068,23 +15068,23 @@
       <c r="L15" s="3"/>
       <c r="M15" s="3"/>
     </row>
-    <row r="16" spans="2:13" ht="35" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:13" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
-      <c r="D16" s="144" t="s">
+      <c r="D16" s="146" t="s">
         <v>147</v>
       </c>
-      <c r="E16" s="144"/>
-      <c r="F16" s="144"/>
-      <c r="G16" s="144"/>
-      <c r="H16" s="144"/>
-      <c r="I16" s="144"/>
-      <c r="J16" s="144"/>
-      <c r="K16" s="144"/>
-      <c r="L16" s="144"/>
+      <c r="E16" s="146"/>
+      <c r="F16" s="146"/>
+      <c r="G16" s="146"/>
+      <c r="H16" s="146"/>
+      <c r="I16" s="146"/>
+      <c r="J16" s="146"/>
+      <c r="K16" s="146"/>
+      <c r="L16" s="146"/>
       <c r="M16" s="3"/>
     </row>
-    <row r="17" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
       <c r="D17" s="3"/>
@@ -15098,23 +15098,23 @@
       <c r="L17" s="3"/>
       <c r="M17" s="3"/>
     </row>
-    <row r="18" spans="2:13" ht="28" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:13" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
-      <c r="D18" s="144" t="s">
+      <c r="D18" s="146" t="s">
         <v>97</v>
       </c>
-      <c r="E18" s="144"/>
-      <c r="F18" s="144"/>
-      <c r="G18" s="144"/>
-      <c r="H18" s="144"/>
-      <c r="I18" s="144"/>
-      <c r="J18" s="144"/>
-      <c r="K18" s="144"/>
-      <c r="L18" s="144"/>
+      <c r="E18" s="146"/>
+      <c r="F18" s="146"/>
+      <c r="G18" s="146"/>
+      <c r="H18" s="146"/>
+      <c r="I18" s="146"/>
+      <c r="J18" s="146"/>
+      <c r="K18" s="146"/>
+      <c r="L18" s="146"/>
       <c r="M18" s="3"/>
     </row>
-    <row r="19" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
       <c r="D19" s="34"/>
@@ -15128,23 +15128,23 @@
       <c r="L19" s="34"/>
       <c r="M19" s="3"/>
     </row>
-    <row r="20" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
-      <c r="D20" s="144" t="s">
+      <c r="D20" s="146" t="s">
         <v>130</v>
       </c>
-      <c r="E20" s="144"/>
-      <c r="F20" s="144"/>
-      <c r="G20" s="144"/>
-      <c r="H20" s="144"/>
-      <c r="I20" s="144"/>
-      <c r="J20" s="144"/>
-      <c r="K20" s="144"/>
-      <c r="L20" s="144"/>
+      <c r="E20" s="146"/>
+      <c r="F20" s="146"/>
+      <c r="G20" s="146"/>
+      <c r="H20" s="146"/>
+      <c r="I20" s="146"/>
+      <c r="J20" s="146"/>
+      <c r="K20" s="146"/>
+      <c r="L20" s="146"/>
       <c r="M20" s="3"/>
     </row>
-    <row r="21" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
       <c r="D21" s="3"/>
@@ -15158,7 +15158,7 @@
       <c r="L21" s="3"/>
       <c r="M21" s="3"/>
     </row>
-    <row r="22" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B22" s="3"/>
       <c r="C22" s="3"/>
       <c r="D22" s="3"/>
@@ -15172,7 +15172,7 @@
       <c r="L22" s="3"/>
       <c r="M22" s="3"/>
     </row>
-    <row r="23" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B23" s="66"/>
       <c r="C23" s="139" t="s">
         <v>45</v>
@@ -15188,23 +15188,23 @@
       <c r="L23" s="66"/>
       <c r="M23" s="66"/>
     </row>
-    <row r="24" spans="2:13" ht="32" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:13" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" s="3"/>
       <c r="C24" s="4"/>
-      <c r="D24" s="144" t="s">
+      <c r="D24" s="146" t="s">
         <v>131</v>
       </c>
-      <c r="E24" s="144"/>
-      <c r="F24" s="144"/>
-      <c r="G24" s="144"/>
-      <c r="H24" s="144"/>
-      <c r="I24" s="144"/>
-      <c r="J24" s="144"/>
-      <c r="K24" s="144"/>
-      <c r="L24" s="144"/>
+      <c r="E24" s="146"/>
+      <c r="F24" s="146"/>
+      <c r="G24" s="146"/>
+      <c r="H24" s="146"/>
+      <c r="I24" s="146"/>
+      <c r="J24" s="146"/>
+      <c r="K24" s="146"/>
+      <c r="L24" s="146"/>
       <c r="M24" s="3"/>
     </row>
-    <row r="25" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B25" s="3"/>
       <c r="C25" s="4"/>
       <c r="D25" s="3"/>
@@ -15218,23 +15218,23 @@
       <c r="L25" s="3"/>
       <c r="M25" s="3"/>
     </row>
-    <row r="26" spans="2:13" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:13" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
-      <c r="D26" s="144" t="s">
+      <c r="D26" s="146" t="s">
         <v>132</v>
       </c>
-      <c r="E26" s="144"/>
-      <c r="F26" s="144"/>
-      <c r="G26" s="144"/>
-      <c r="H26" s="144"/>
-      <c r="I26" s="144"/>
-      <c r="J26" s="144"/>
-      <c r="K26" s="144"/>
-      <c r="L26" s="144"/>
+      <c r="E26" s="146"/>
+      <c r="F26" s="146"/>
+      <c r="G26" s="146"/>
+      <c r="H26" s="146"/>
+      <c r="I26" s="146"/>
+      <c r="J26" s="146"/>
+      <c r="K26" s="146"/>
+      <c r="L26" s="146"/>
       <c r="M26" s="3"/>
     </row>
-    <row r="27" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
       <c r="D27" s="3"/>
@@ -15248,23 +15248,23 @@
       <c r="L27" s="3"/>
       <c r="M27" s="3"/>
     </row>
-    <row r="28" spans="2:13" ht="31" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:13" ht="31" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
-      <c r="D28" s="144" t="s">
+      <c r="D28" s="146" t="s">
         <v>98</v>
       </c>
-      <c r="E28" s="144"/>
-      <c r="F28" s="144"/>
-      <c r="G28" s="144"/>
-      <c r="H28" s="144"/>
-      <c r="I28" s="144"/>
-      <c r="J28" s="144"/>
-      <c r="K28" s="144"/>
-      <c r="L28" s="144"/>
+      <c r="E28" s="146"/>
+      <c r="F28" s="146"/>
+      <c r="G28" s="146"/>
+      <c r="H28" s="146"/>
+      <c r="I28" s="146"/>
+      <c r="J28" s="146"/>
+      <c r="K28" s="146"/>
+      <c r="L28" s="146"/>
       <c r="M28" s="3"/>
     </row>
-    <row r="29" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
       <c r="D29" s="3"/>
@@ -15278,23 +15278,23 @@
       <c r="L29" s="3"/>
       <c r="M29" s="3"/>
     </row>
-    <row r="30" spans="2:13" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:13" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B30" s="3"/>
       <c r="C30" s="3"/>
-      <c r="D30" s="144" t="s">
+      <c r="D30" s="146" t="s">
         <v>49</v>
       </c>
-      <c r="E30" s="144"/>
-      <c r="F30" s="144"/>
-      <c r="G30" s="144"/>
-      <c r="H30" s="144"/>
-      <c r="I30" s="144"/>
-      <c r="J30" s="144"/>
-      <c r="K30" s="144"/>
-      <c r="L30" s="144"/>
+      <c r="E30" s="146"/>
+      <c r="F30" s="146"/>
+      <c r="G30" s="146"/>
+      <c r="H30" s="146"/>
+      <c r="I30" s="146"/>
+      <c r="J30" s="146"/>
+      <c r="K30" s="146"/>
+      <c r="L30" s="146"/>
       <c r="M30" s="3"/>
     </row>
-    <row r="31" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B31" s="3"/>
       <c r="C31" s="3"/>
       <c r="D31" s="3"/>
@@ -15308,7 +15308,7 @@
       <c r="L31" s="3"/>
       <c r="M31" s="3"/>
     </row>
-    <row r="32" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
       <c r="D32" s="3"/>
@@ -15322,7 +15322,7 @@
       <c r="L32" s="3"/>
       <c r="M32" s="3"/>
     </row>
-    <row r="33" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B33" s="3"/>
       <c r="C33" s="3"/>
       <c r="D33" s="3"/>
@@ -15336,7 +15336,7 @@
       <c r="L33" s="3"/>
       <c r="M33" s="3"/>
     </row>
-    <row r="34" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B34" s="3"/>
       <c r="C34" s="3"/>
       <c r="D34" s="3"/>
@@ -15350,7 +15350,7 @@
       <c r="L34" s="3"/>
       <c r="M34" s="3"/>
     </row>
-    <row r="35" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B35" s="3"/>
       <c r="C35" s="3"/>
       <c r="D35" s="3"/>
@@ -15365,13 +15365,8 @@
       <c r="M35" s="3"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
+  <sheetProtection selectLockedCells="1"/>
   <mergeCells count="12">
-    <mergeCell ref="C5:L5"/>
-    <mergeCell ref="D20:L20"/>
-    <mergeCell ref="D8:L8"/>
-    <mergeCell ref="D10:L10"/>
-    <mergeCell ref="D26:L26"/>
     <mergeCell ref="D30:L30"/>
     <mergeCell ref="D14:L14"/>
     <mergeCell ref="D12:L12"/>
@@ -15379,6 +15374,11 @@
     <mergeCell ref="D16:L16"/>
     <mergeCell ref="D24:L24"/>
     <mergeCell ref="D28:L28"/>
+    <mergeCell ref="C5:L5"/>
+    <mergeCell ref="D20:L20"/>
+    <mergeCell ref="D8:L8"/>
+    <mergeCell ref="D10:L10"/>
+    <mergeCell ref="D26:L26"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
updates to figures and population params
</commit_message>
<xml_diff>
--- a/Burden-of-Illness-Tool/MADMC B19 Pregancy Outcome Estimate Tool_Sept2025.xlsx
+++ b/Burden-of-Illness-Tool/MADMC B19 Pregancy Outcome Estimate Tool_Sept2025.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ritesh/Desktop/Scenario-Modeling-of-Human-Parvovirus-B19/Burden-of-Illness-Tool/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48435279-3A36-2144-A09E-09DC83770885}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AD92736-0293-054F-AD96-9E382C5CB624}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-30240" yWindow="1620" windowWidth="30260" windowHeight="18980" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="2" r:id="rId1"/>
@@ -3037,6 +3037,27 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="30" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -3044,28 +3065,40 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3084,39 +3117,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -6338,7 +6338,7 @@
       <c r="D48" s="11"/>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="1"/>
+  <sheetProtection sheet="1" selectLockedCells="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -6366,42 +6366,42 @@
       <c r="E1" s="27"/>
     </row>
     <row r="3" spans="1:29" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B3" s="144" t="s">
+      <c r="B3" s="151" t="s">
         <v>143</v>
       </c>
-      <c r="C3" s="144"/>
-      <c r="D3" s="144"/>
-      <c r="E3" s="144"/>
-      <c r="F3" s="144"/>
-      <c r="G3" s="144"/>
-      <c r="H3" s="144"/>
-      <c r="I3" s="144"/>
-      <c r="J3" s="144"/>
-      <c r="K3" s="144"/>
-      <c r="L3" s="144"/>
-      <c r="M3" s="144"/>
-      <c r="N3" s="144"/>
-      <c r="O3" s="144"/>
-      <c r="P3" s="144"/>
-      <c r="Q3" s="144"/>
+      <c r="C3" s="151"/>
+      <c r="D3" s="151"/>
+      <c r="E3" s="151"/>
+      <c r="F3" s="151"/>
+      <c r="G3" s="151"/>
+      <c r="H3" s="151"/>
+      <c r="I3" s="151"/>
+      <c r="J3" s="151"/>
+      <c r="K3" s="151"/>
+      <c r="L3" s="151"/>
+      <c r="M3" s="151"/>
+      <c r="N3" s="151"/>
+      <c r="O3" s="151"/>
+      <c r="P3" s="151"/>
+      <c r="Q3" s="151"/>
     </row>
     <row r="4" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="B4" s="144"/>
-      <c r="C4" s="144"/>
-      <c r="D4" s="144"/>
-      <c r="E4" s="144"/>
-      <c r="F4" s="144"/>
-      <c r="G4" s="144"/>
-      <c r="H4" s="144"/>
-      <c r="I4" s="144"/>
-      <c r="J4" s="144"/>
-      <c r="K4" s="144"/>
-      <c r="L4" s="144"/>
-      <c r="M4" s="144"/>
-      <c r="N4" s="144"/>
-      <c r="O4" s="144"/>
-      <c r="P4" s="144"/>
-      <c r="Q4" s="144"/>
+      <c r="B4" s="151"/>
+      <c r="C4" s="151"/>
+      <c r="D4" s="151"/>
+      <c r="E4" s="151"/>
+      <c r="F4" s="151"/>
+      <c r="G4" s="151"/>
+      <c r="H4" s="151"/>
+      <c r="I4" s="151"/>
+      <c r="J4" s="151"/>
+      <c r="K4" s="151"/>
+      <c r="L4" s="151"/>
+      <c r="M4" s="151"/>
+      <c r="N4" s="151"/>
+      <c r="O4" s="151"/>
+      <c r="P4" s="151"/>
+      <c r="Q4" s="151"/>
     </row>
     <row r="5" spans="1:29" ht="16" x14ac:dyDescent="0.2">
       <c r="B5" s="111"/>
@@ -6483,17 +6483,17 @@
       <c r="F8" s="32"/>
       <c r="G8" s="4"/>
       <c r="H8" s="3"/>
-      <c r="I8" s="145" t="str">
+      <c r="I8" s="152" t="str">
         <f>_xlfn.CONCAT("Based on ", C9, " pregnancies in the population and historic estimates of parvovirus immunity, mother infection risk, fetal infection risk, and risk of severe fetal outcomes (Table 1), the expected number of severe fetal outcomes due to parvovirus is ",C22,". Under a best case scenario of higher immunity, lower infection rates, and lower complication rates, the number of severe fetal outcomes due to PVB19 could be as low as ", F22, ", while under a worst case scenario the number of severe fetal outcomes may be as high as ", G22, " in the population with ", C9, " pregnancies (Figure 1, Table 2).")</f>
         <v>Based on 100000 pregnancies in the population and historic estimates of parvovirus immunity, mother infection risk, fetal infection risk, and risk of severe fetal outcomes (Table 1), the expected number of severe fetal outcomes due to parvovirus is . Under a best case scenario of higher immunity, lower infection rates, and lower complication rates, the number of severe fetal outcomes due to PVB19 could be as low as , while under a worst case scenario the number of severe fetal outcomes may be as high as  in the population with 100000 pregnancies (Figure 1, Table 2).</v>
       </c>
-      <c r="J8" s="145"/>
-      <c r="K8" s="145"/>
-      <c r="L8" s="145"/>
-      <c r="M8" s="145"/>
-      <c r="N8" s="145"/>
-      <c r="O8" s="145"/>
-      <c r="P8" s="145"/>
+      <c r="J8" s="152"/>
+      <c r="K8" s="152"/>
+      <c r="L8" s="152"/>
+      <c r="M8" s="152"/>
+      <c r="N8" s="152"/>
+      <c r="O8" s="152"/>
+      <c r="P8" s="152"/>
       <c r="Q8" s="33"/>
       <c r="R8" s="18"/>
       <c r="X8" s="9"/>
@@ -6520,14 +6520,14 @@
       <c r="F9" s="71"/>
       <c r="G9" s="4"/>
       <c r="H9" s="33"/>
-      <c r="I9" s="145"/>
-      <c r="J9" s="145"/>
-      <c r="K9" s="145"/>
-      <c r="L9" s="145"/>
-      <c r="M9" s="145"/>
-      <c r="N9" s="145"/>
-      <c r="O9" s="145"/>
-      <c r="P9" s="145"/>
+      <c r="I9" s="152"/>
+      <c r="J9" s="152"/>
+      <c r="K9" s="152"/>
+      <c r="L9" s="152"/>
+      <c r="M9" s="152"/>
+      <c r="N9" s="152"/>
+      <c r="O9" s="152"/>
+      <c r="P9" s="152"/>
       <c r="Q9" s="33"/>
       <c r="R9" s="18"/>
       <c r="X9" s="8"/>
@@ -6554,14 +6554,14 @@
       <c r="F10" s="72"/>
       <c r="G10" s="4"/>
       <c r="H10" s="33"/>
-      <c r="I10" s="145"/>
-      <c r="J10" s="145"/>
-      <c r="K10" s="145"/>
-      <c r="L10" s="145"/>
-      <c r="M10" s="145"/>
-      <c r="N10" s="145"/>
-      <c r="O10" s="145"/>
-      <c r="P10" s="145"/>
+      <c r="I10" s="152"/>
+      <c r="J10" s="152"/>
+      <c r="K10" s="152"/>
+      <c r="L10" s="152"/>
+      <c r="M10" s="152"/>
+      <c r="N10" s="152"/>
+      <c r="O10" s="152"/>
+      <c r="P10" s="152"/>
       <c r="Q10" s="33"/>
       <c r="R10" s="18"/>
       <c r="X10" s="8"/>
@@ -6641,12 +6641,12 @@
     </row>
     <row r="13" spans="1:29" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="3"/>
-      <c r="B13" s="149" t="s">
+      <c r="B13" s="146" t="s">
         <v>114</v>
       </c>
-      <c r="C13" s="149"/>
-      <c r="D13" s="149"/>
-      <c r="E13" s="149"/>
+      <c r="C13" s="146"/>
+      <c r="D13" s="146"/>
+      <c r="E13" s="146"/>
       <c r="F13" s="72"/>
       <c r="G13" s="3"/>
       <c r="H13" s="3"/>
@@ -6725,20 +6725,20 @@
     </row>
     <row r="17" spans="1:18" ht="33.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3"/>
-      <c r="B17" s="150" t="s">
+      <c r="B17" s="147" t="s">
         <v>99</v>
       </c>
       <c r="C17" s="77" t="s">
         <v>6</v>
       </c>
-      <c r="D17" s="152" t="s">
+      <c r="D17" s="149" t="s">
         <v>16</v>
       </c>
-      <c r="E17" s="153"/>
-      <c r="F17" s="152" t="s">
+      <c r="E17" s="150"/>
+      <c r="F17" s="149" t="s">
         <v>19</v>
       </c>
-      <c r="G17" s="153"/>
+      <c r="G17" s="150"/>
       <c r="H17" s="75"/>
       <c r="I17" s="5"/>
       <c r="J17" s="5"/>
@@ -6753,7 +6753,7 @@
     </row>
     <row r="18" spans="1:18" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3"/>
-      <c r="B18" s="151"/>
+      <c r="B18" s="148"/>
       <c r="C18" s="78" t="s">
         <v>41</v>
       </c>
@@ -6938,14 +6938,14 @@
     </row>
     <row r="24" spans="1:18" ht="44" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="3"/>
-      <c r="B24" s="148" t="s">
+      <c r="B24" s="145" t="s">
         <v>35</v>
       </c>
-      <c r="C24" s="148"/>
-      <c r="D24" s="148"/>
-      <c r="E24" s="148"/>
-      <c r="F24" s="148"/>
-      <c r="G24" s="148"/>
+      <c r="C24" s="145"/>
+      <c r="D24" s="145"/>
+      <c r="E24" s="145"/>
+      <c r="F24" s="145"/>
+      <c r="G24" s="145"/>
       <c r="H24" s="38"/>
       <c r="I24" s="38"/>
       <c r="J24" s="3"/>
@@ -6960,14 +6960,14 @@
     </row>
     <row r="25" spans="1:18" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="3"/>
-      <c r="B25" s="148" t="s">
+      <c r="B25" s="145" t="s">
         <v>39</v>
       </c>
-      <c r="C25" s="148"/>
-      <c r="D25" s="148"/>
-      <c r="E25" s="148"/>
-      <c r="F25" s="148"/>
-      <c r="G25" s="148"/>
+      <c r="C25" s="145"/>
+      <c r="D25" s="145"/>
+      <c r="E25" s="145"/>
+      <c r="F25" s="145"/>
+      <c r="G25" s="145"/>
       <c r="H25" s="38"/>
       <c r="I25" s="44"/>
       <c r="J25" s="74"/>
@@ -7204,14 +7204,14 @@
     </row>
     <row r="37" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="3"/>
-      <c r="B37" s="147" t="s">
+      <c r="B37" s="153" t="s">
         <v>24</v>
       </c>
-      <c r="C37" s="147"/>
-      <c r="D37" s="147"/>
-      <c r="E37" s="147"/>
-      <c r="F37" s="147"/>
-      <c r="G37" s="147"/>
+      <c r="C37" s="153"/>
+      <c r="D37" s="153"/>
+      <c r="E37" s="153"/>
+      <c r="F37" s="153"/>
+      <c r="G37" s="153"/>
       <c r="H37" s="3"/>
       <c r="I37" s="36"/>
       <c r="J37" s="3"/>
@@ -7226,14 +7226,14 @@
     </row>
     <row r="38" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A38" s="3"/>
-      <c r="B38" s="146" t="s">
+      <c r="B38" s="144" t="s">
         <v>25</v>
       </c>
-      <c r="C38" s="146"/>
-      <c r="D38" s="146"/>
-      <c r="E38" s="146"/>
-      <c r="F38" s="146"/>
-      <c r="G38" s="146"/>
+      <c r="C38" s="144"/>
+      <c r="D38" s="144"/>
+      <c r="E38" s="144"/>
+      <c r="F38" s="144"/>
+      <c r="G38" s="144"/>
       <c r="H38" s="33"/>
       <c r="I38" s="34"/>
       <c r="J38" s="3"/>
@@ -7248,14 +7248,14 @@
     </row>
     <row r="39" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A39" s="3"/>
-      <c r="B39" s="146" t="s">
+      <c r="B39" s="144" t="s">
         <v>30</v>
       </c>
-      <c r="C39" s="146"/>
-      <c r="D39" s="146"/>
-      <c r="E39" s="146"/>
-      <c r="F39" s="146"/>
-      <c r="G39" s="146"/>
+      <c r="C39" s="144"/>
+      <c r="D39" s="144"/>
+      <c r="E39" s="144"/>
+      <c r="F39" s="144"/>
+      <c r="G39" s="144"/>
       <c r="H39" s="33"/>
       <c r="I39" s="34"/>
       <c r="J39" s="3"/>
@@ -7270,14 +7270,14 @@
     </row>
     <row r="40" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="3"/>
-      <c r="B40" s="146" t="s">
+      <c r="B40" s="144" t="s">
         <v>31</v>
       </c>
-      <c r="C40" s="146"/>
-      <c r="D40" s="146"/>
-      <c r="E40" s="146"/>
-      <c r="F40" s="146"/>
-      <c r="G40" s="146"/>
+      <c r="C40" s="144"/>
+      <c r="D40" s="144"/>
+      <c r="E40" s="144"/>
+      <c r="F40" s="144"/>
+      <c r="G40" s="144"/>
       <c r="H40" s="33"/>
       <c r="I40" s="34"/>
       <c r="J40" s="3"/>
@@ -7292,14 +7292,14 @@
     </row>
     <row r="41" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="3"/>
-      <c r="B41" s="146" t="s">
+      <c r="B41" s="144" t="s">
         <v>32</v>
       </c>
-      <c r="C41" s="146"/>
-      <c r="D41" s="146"/>
-      <c r="E41" s="146"/>
-      <c r="F41" s="146"/>
-      <c r="G41" s="146"/>
+      <c r="C41" s="144"/>
+      <c r="D41" s="144"/>
+      <c r="E41" s="144"/>
+      <c r="F41" s="144"/>
+      <c r="G41" s="144"/>
       <c r="H41" s="33"/>
       <c r="I41" s="34"/>
       <c r="J41" s="3"/>
@@ -7439,8 +7439,13 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="1"/>
+  <sheetProtection sheet="1" selectLockedCells="1"/>
   <mergeCells count="13">
+    <mergeCell ref="B3:Q4"/>
+    <mergeCell ref="I8:P10"/>
+    <mergeCell ref="B38:G38"/>
+    <mergeCell ref="B37:G37"/>
+    <mergeCell ref="B39:G39"/>
     <mergeCell ref="B41:G41"/>
     <mergeCell ref="B24:G24"/>
     <mergeCell ref="B25:G25"/>
@@ -7449,11 +7454,6 @@
     <mergeCell ref="D17:E17"/>
     <mergeCell ref="F17:G17"/>
     <mergeCell ref="B40:G40"/>
-    <mergeCell ref="B3:Q4"/>
-    <mergeCell ref="I8:P10"/>
-    <mergeCell ref="B38:G38"/>
-    <mergeCell ref="B37:G37"/>
-    <mergeCell ref="B39:G39"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -7504,25 +7504,25 @@
       <c r="F2" s="7"/>
     </row>
     <row r="3" spans="2:34" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C3" s="161" t="s">
+      <c r="C3" s="154" t="s">
         <v>144</v>
       </c>
-      <c r="D3" s="161"/>
-      <c r="E3" s="161"/>
-      <c r="F3" s="161"/>
-      <c r="G3" s="161"/>
-      <c r="H3" s="161"/>
-      <c r="I3" s="161"/>
-      <c r="J3" s="161"/>
-      <c r="K3" s="161"/>
-      <c r="L3" s="161"/>
-      <c r="M3" s="161"/>
-      <c r="N3" s="161"/>
-      <c r="O3" s="161"/>
-      <c r="P3" s="161"/>
-      <c r="Q3" s="161"/>
-      <c r="R3" s="161"/>
-      <c r="S3" s="161"/>
+      <c r="D3" s="154"/>
+      <c r="E3" s="154"/>
+      <c r="F3" s="154"/>
+      <c r="G3" s="154"/>
+      <c r="H3" s="154"/>
+      <c r="I3" s="154"/>
+      <c r="J3" s="154"/>
+      <c r="K3" s="154"/>
+      <c r="L3" s="154"/>
+      <c r="M3" s="154"/>
+      <c r="N3" s="154"/>
+      <c r="O3" s="154"/>
+      <c r="P3" s="154"/>
+      <c r="Q3" s="154"/>
+      <c r="R3" s="154"/>
+      <c r="S3" s="154"/>
     </row>
     <row r="5" spans="2:34" ht="26.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B5" s="3"/>
@@ -7534,20 +7534,20 @@
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
-      <c r="I5" s="162" t="str">
+      <c r="I5" s="155" t="str">
         <f>_xlfn.CONCAT("Figure 1. Estimated Number of Severe Fetal Outcomes Under Potential Immunity and Infection Rate Scenarios, based on ",D7," Pregnancies")</f>
         <v>Figure 1. Estimated Number of Severe Fetal Outcomes Under Potential Immunity and Infection Rate Scenarios, based on 100000 Pregnancies</v>
       </c>
-      <c r="J5" s="162"/>
-      <c r="K5" s="162"/>
-      <c r="L5" s="162"/>
-      <c r="M5" s="162"/>
-      <c r="N5" s="162"/>
-      <c r="O5" s="162"/>
-      <c r="P5" s="162"/>
-      <c r="Q5" s="162"/>
-      <c r="R5" s="162"/>
-      <c r="S5" s="162"/>
+      <c r="J5" s="155"/>
+      <c r="K5" s="155"/>
+      <c r="L5" s="155"/>
+      <c r="M5" s="155"/>
+      <c r="N5" s="155"/>
+      <c r="O5" s="155"/>
+      <c r="P5" s="155"/>
+      <c r="Q5" s="155"/>
+      <c r="R5" s="155"/>
+      <c r="S5" s="155"/>
       <c r="T5" s="3"/>
       <c r="W5" s="51" t="s">
         <v>22</v>
@@ -7568,17 +7568,17 @@
       <c r="F6" s="3"/>
       <c r="G6" s="3"/>
       <c r="H6" s="3"/>
-      <c r="I6" s="162"/>
-      <c r="J6" s="162"/>
-      <c r="K6" s="162"/>
-      <c r="L6" s="162"/>
-      <c r="M6" s="162"/>
-      <c r="N6" s="162"/>
-      <c r="O6" s="162"/>
-      <c r="P6" s="162"/>
-      <c r="Q6" s="162"/>
-      <c r="R6" s="162"/>
-      <c r="S6" s="162"/>
+      <c r="I6" s="155"/>
+      <c r="J6" s="155"/>
+      <c r="K6" s="155"/>
+      <c r="L6" s="155"/>
+      <c r="M6" s="155"/>
+      <c r="N6" s="155"/>
+      <c r="O6" s="155"/>
+      <c r="P6" s="155"/>
+      <c r="Q6" s="155"/>
+      <c r="R6" s="155"/>
+      <c r="S6" s="155"/>
       <c r="T6" s="3"/>
       <c r="W6" s="52" t="s">
         <v>4</v>
@@ -7621,7 +7621,7 @@
       </c>
       <c r="E7" s="46"/>
       <c r="F7" s="3"/>
-      <c r="G7" s="160" t="s">
+      <c r="G7" s="156" t="s">
         <v>127</v>
       </c>
       <c r="H7" s="13">
@@ -7719,7 +7719,7 @@
       </c>
       <c r="E8" s="47"/>
       <c r="F8" s="3"/>
-      <c r="G8" s="160"/>
+      <c r="G8" s="156"/>
       <c r="H8" s="13">
         <v>0.7</v>
       </c>
@@ -7815,7 +7815,7 @@
       </c>
       <c r="E9" s="47"/>
       <c r="F9" s="3"/>
-      <c r="G9" s="160"/>
+      <c r="G9" s="156"/>
       <c r="H9" s="13">
         <v>0.65</v>
       </c>
@@ -7911,7 +7911,7 @@
       </c>
       <c r="E10" s="48"/>
       <c r="F10" s="3"/>
-      <c r="G10" s="160"/>
+      <c r="G10" s="156"/>
       <c r="H10" s="13">
         <v>0.6</v>
       </c>
@@ -7920,7 +7920,7 @@
         <v>0</v>
       </c>
       <c r="J10" s="28">
-        <f t="shared" si="2"/>
+        <f>AA21</f>
         <v>30</v>
       </c>
       <c r="K10" s="29">
@@ -8003,7 +8003,7 @@
       <c r="D11" s="48"/>
       <c r="E11" s="48"/>
       <c r="F11" s="3"/>
-      <c r="G11" s="160"/>
+      <c r="G11" s="156"/>
       <c r="H11" s="13">
         <v>0.55000000000000004</v>
       </c>
@@ -8095,7 +8095,7 @@
       <c r="D12" s="3"/>
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
-      <c r="G12" s="160"/>
+      <c r="G12" s="156"/>
       <c r="H12" s="13">
         <v>0.5</v>
       </c>
@@ -8189,7 +8189,7 @@
       <c r="D13" s="24"/>
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
-      <c r="G13" s="160"/>
+      <c r="G13" s="156"/>
       <c r="H13" s="13">
         <v>0.45</v>
       </c>
@@ -8277,13 +8277,13 @@
     </row>
     <row r="14" spans="2:34" ht="29" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B14" s="3"/>
-      <c r="C14" s="163" t="s">
+      <c r="C14" s="157" t="s">
         <v>46</v>
       </c>
-      <c r="D14" s="164"/>
+      <c r="D14" s="158"/>
       <c r="E14" s="45"/>
       <c r="F14" s="3"/>
-      <c r="G14" s="160"/>
+      <c r="G14" s="156"/>
       <c r="H14" s="13">
         <v>0.4</v>
       </c>
@@ -8371,11 +8371,11 @@
     </row>
     <row r="15" spans="2:34" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="3"/>
-      <c r="C15" s="165"/>
-      <c r="D15" s="164"/>
+      <c r="C15" s="159"/>
+      <c r="D15" s="158"/>
       <c r="E15" s="45"/>
       <c r="F15" s="3"/>
-      <c r="G15" s="160"/>
+      <c r="G15" s="156"/>
       <c r="H15" s="13">
         <v>0.35</v>
       </c>
@@ -8463,13 +8463,13 @@
     </row>
     <row r="16" spans="2:34" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="3"/>
-      <c r="C16" s="166" t="s">
+      <c r="C16" s="160" t="s">
         <v>47</v>
       </c>
-      <c r="D16" s="167"/>
+      <c r="D16" s="161"/>
       <c r="E16" s="34"/>
       <c r="F16" s="3"/>
-      <c r="G16" s="160"/>
+      <c r="G16" s="156"/>
       <c r="H16" s="13">
         <v>0.3</v>
       </c>
@@ -8557,13 +8557,13 @@
     </row>
     <row r="17" spans="2:34" ht="17" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B17" s="3"/>
-      <c r="C17" s="166" t="s">
+      <c r="C17" s="160" t="s">
         <v>125</v>
       </c>
-      <c r="D17" s="167"/>
+      <c r="D17" s="161"/>
       <c r="E17" s="34"/>
       <c r="F17" s="3"/>
-      <c r="G17" s="160"/>
+      <c r="G17" s="156"/>
       <c r="H17" s="13">
         <v>0.25</v>
       </c>
@@ -8651,8 +8651,8 @@
     </row>
     <row r="18" spans="2:34" x14ac:dyDescent="0.2">
       <c r="B18" s="3"/>
-      <c r="C18" s="168"/>
-      <c r="D18" s="167"/>
+      <c r="C18" s="162"/>
+      <c r="D18" s="161"/>
       <c r="E18" s="34"/>
       <c r="F18" s="3"/>
       <c r="G18" s="3"/>
@@ -8730,25 +8730,25 @@
     </row>
     <row r="19" spans="2:34" x14ac:dyDescent="0.2">
       <c r="B19" s="3"/>
-      <c r="C19" s="168"/>
-      <c r="D19" s="167"/>
+      <c r="C19" s="162"/>
+      <c r="D19" s="161"/>
       <c r="E19" s="34"/>
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
       <c r="H19" s="3"/>
-      <c r="I19" s="154" t="s">
+      <c r="I19" s="165" t="s">
         <v>126</v>
       </c>
-      <c r="J19" s="154"/>
-      <c r="K19" s="154"/>
-      <c r="L19" s="154"/>
-      <c r="M19" s="154"/>
-      <c r="N19" s="154"/>
-      <c r="O19" s="154"/>
-      <c r="P19" s="154"/>
-      <c r="Q19" s="154"/>
-      <c r="R19" s="154"/>
-      <c r="S19" s="154"/>
+      <c r="J19" s="165"/>
+      <c r="K19" s="165"/>
+      <c r="L19" s="165"/>
+      <c r="M19" s="165"/>
+      <c r="N19" s="165"/>
+      <c r="O19" s="165"/>
+      <c r="P19" s="165"/>
+      <c r="Q19" s="165"/>
+      <c r="R19" s="165"/>
+      <c r="S19" s="165"/>
       <c r="T19" s="3"/>
       <c r="W19" s="53">
         <v>0.01</v>
@@ -8789,8 +8789,8 @@
     </row>
     <row r="20" spans="2:34" x14ac:dyDescent="0.2">
       <c r="B20" s="3"/>
-      <c r="C20" s="168"/>
-      <c r="D20" s="167"/>
+      <c r="C20" s="162"/>
+      <c r="D20" s="161"/>
       <c r="E20" s="34"/>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
@@ -8848,8 +8848,8 @@
     </row>
     <row r="21" spans="2:34" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B21" s="3"/>
-      <c r="C21" s="169"/>
-      <c r="D21" s="170"/>
+      <c r="C21" s="163"/>
+      <c r="D21" s="164"/>
       <c r="E21" s="34"/>
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
@@ -9029,20 +9029,20 @@
       <c r="F24" s="3"/>
       <c r="G24" s="3"/>
       <c r="H24" s="3"/>
-      <c r="I24" s="157" t="str">
+      <c r="I24" s="168" t="str">
         <f>_xlfn.CONCAT("Figure 2. Estimated Number of Severe Fetal Outcomes Under all Possible Immunity and Infection Rate Scenarios, based on ",D7," Pregnancies")</f>
         <v>Figure 2. Estimated Number of Severe Fetal Outcomes Under all Possible Immunity and Infection Rate Scenarios, based on 100000 Pregnancies</v>
       </c>
-      <c r="J24" s="157"/>
-      <c r="K24" s="157"/>
-      <c r="L24" s="157"/>
-      <c r="M24" s="157"/>
-      <c r="N24" s="157"/>
-      <c r="O24" s="157"/>
-      <c r="P24" s="157"/>
-      <c r="Q24" s="157"/>
-      <c r="R24" s="157"/>
-      <c r="S24" s="157"/>
+      <c r="J24" s="168"/>
+      <c r="K24" s="168"/>
+      <c r="L24" s="168"/>
+      <c r="M24" s="168"/>
+      <c r="N24" s="168"/>
+      <c r="O24" s="168"/>
+      <c r="P24" s="168"/>
+      <c r="Q24" s="168"/>
+      <c r="R24" s="168"/>
+      <c r="S24" s="168"/>
       <c r="T24" s="3"/>
       <c r="W24" s="53">
         <v>0.01</v>
@@ -9083,25 +9083,25 @@
     </row>
     <row r="25" spans="2:34" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B25" s="3"/>
-      <c r="C25" s="159" t="s">
+      <c r="C25" s="170" t="s">
         <v>24</v>
       </c>
-      <c r="D25" s="159"/>
+      <c r="D25" s="170"/>
       <c r="E25" s="45"/>
       <c r="F25" s="3"/>
       <c r="G25" s="3"/>
       <c r="H25" s="3"/>
-      <c r="I25" s="158"/>
-      <c r="J25" s="158"/>
-      <c r="K25" s="158"/>
-      <c r="L25" s="158"/>
-      <c r="M25" s="158"/>
-      <c r="N25" s="158"/>
-      <c r="O25" s="158"/>
-      <c r="P25" s="158"/>
-      <c r="Q25" s="158"/>
-      <c r="R25" s="158"/>
-      <c r="S25" s="158"/>
+      <c r="I25" s="169"/>
+      <c r="J25" s="169"/>
+      <c r="K25" s="169"/>
+      <c r="L25" s="169"/>
+      <c r="M25" s="169"/>
+      <c r="N25" s="169"/>
+      <c r="O25" s="169"/>
+      <c r="P25" s="169"/>
+      <c r="Q25" s="169"/>
+      <c r="R25" s="169"/>
+      <c r="S25" s="169"/>
       <c r="T25" s="3"/>
       <c r="W25" s="53">
         <v>0.01</v>
@@ -9142,11 +9142,11 @@
     </row>
     <row r="26" spans="2:34" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="3"/>
-      <c r="C26" s="159"/>
-      <c r="D26" s="159"/>
+      <c r="C26" s="170"/>
+      <c r="D26" s="170"/>
       <c r="E26" s="45"/>
       <c r="F26" s="3"/>
-      <c r="G26" s="160" t="s">
+      <c r="G26" s="156" t="s">
         <v>127</v>
       </c>
       <c r="H26" s="13">
@@ -9236,11 +9236,11 @@
     </row>
     <row r="27" spans="2:34" s="8" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B27" s="3"/>
-      <c r="C27" s="159"/>
-      <c r="D27" s="159"/>
+      <c r="C27" s="170"/>
+      <c r="D27" s="170"/>
       <c r="E27" s="45"/>
       <c r="F27" s="33"/>
-      <c r="G27" s="160"/>
+      <c r="G27" s="156"/>
       <c r="H27" s="13">
         <v>0.9</v>
       </c>
@@ -9328,13 +9328,13 @@
     </row>
     <row r="28" spans="2:34" s="8" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B28" s="3"/>
-      <c r="C28" s="159" t="s">
+      <c r="C28" s="170" t="s">
         <v>29</v>
       </c>
-      <c r="D28" s="159"/>
+      <c r="D28" s="170"/>
       <c r="E28" s="45"/>
       <c r="F28" s="33"/>
-      <c r="G28" s="160"/>
+      <c r="G28" s="156"/>
       <c r="H28" s="13">
         <v>0.8</v>
       </c>
@@ -9422,11 +9422,11 @@
     </row>
     <row r="29" spans="2:34" s="8" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B29" s="33"/>
-      <c r="C29" s="159"/>
-      <c r="D29" s="159"/>
+      <c r="C29" s="170"/>
+      <c r="D29" s="170"/>
       <c r="E29" s="45"/>
       <c r="F29" s="33"/>
-      <c r="G29" s="160"/>
+      <c r="G29" s="156"/>
       <c r="H29" s="13">
         <v>0.7</v>
       </c>
@@ -9514,13 +9514,13 @@
     </row>
     <row r="30" spans="2:34" s="8" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B30" s="3"/>
-      <c r="C30" s="159" t="s">
+      <c r="C30" s="170" t="s">
         <v>28</v>
       </c>
-      <c r="D30" s="159"/>
+      <c r="D30" s="170"/>
       <c r="E30" s="45"/>
       <c r="F30" s="33"/>
-      <c r="G30" s="160"/>
+      <c r="G30" s="156"/>
       <c r="H30" s="13">
         <v>0.6</v>
       </c>
@@ -9608,11 +9608,11 @@
     </row>
     <row r="31" spans="2:34" s="8" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B31" s="33"/>
-      <c r="C31" s="159"/>
-      <c r="D31" s="159"/>
+      <c r="C31" s="170"/>
+      <c r="D31" s="170"/>
       <c r="E31" s="45"/>
       <c r="F31" s="33"/>
-      <c r="G31" s="160"/>
+      <c r="G31" s="156"/>
       <c r="H31" s="13">
         <v>0.5</v>
       </c>
@@ -9700,13 +9700,13 @@
     </row>
     <row r="32" spans="2:34" s="8" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B32" s="33"/>
-      <c r="C32" s="159" t="s">
+      <c r="C32" s="170" t="s">
         <v>26</v>
       </c>
-      <c r="D32" s="159"/>
+      <c r="D32" s="170"/>
       <c r="E32" s="45"/>
       <c r="F32" s="33"/>
-      <c r="G32" s="160"/>
+      <c r="G32" s="156"/>
       <c r="H32" s="13">
         <v>0.4</v>
       </c>
@@ -9794,11 +9794,11 @@
     </row>
     <row r="33" spans="2:34" s="8" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B33" s="33"/>
-      <c r="C33" s="159"/>
-      <c r="D33" s="159"/>
+      <c r="C33" s="170"/>
+      <c r="D33" s="170"/>
       <c r="E33" s="45"/>
       <c r="F33" s="33"/>
-      <c r="G33" s="160"/>
+      <c r="G33" s="156"/>
       <c r="H33" s="13">
         <v>0.3</v>
       </c>
@@ -9886,13 +9886,13 @@
     </row>
     <row r="34" spans="2:34" s="8" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B34" s="33"/>
-      <c r="C34" s="159" t="s">
+      <c r="C34" s="170" t="s">
         <v>27</v>
       </c>
-      <c r="D34" s="159"/>
+      <c r="D34" s="170"/>
       <c r="E34" s="45"/>
       <c r="F34" s="33"/>
-      <c r="G34" s="160"/>
+      <c r="G34" s="156"/>
       <c r="H34" s="13">
         <v>0.2</v>
       </c>
@@ -9980,11 +9980,11 @@
     </row>
     <row r="35" spans="2:34" s="8" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B35" s="33"/>
-      <c r="C35" s="159"/>
-      <c r="D35" s="159"/>
+      <c r="C35" s="170"/>
+      <c r="D35" s="170"/>
       <c r="E35" s="45"/>
       <c r="F35" s="33"/>
-      <c r="G35" s="160"/>
+      <c r="G35" s="156"/>
       <c r="H35" s="13">
         <v>0.1</v>
       </c>
@@ -10076,7 +10076,7 @@
       <c r="D36" s="33"/>
       <c r="E36" s="33"/>
       <c r="F36" s="33"/>
-      <c r="G36" s="160"/>
+      <c r="G36" s="156"/>
       <c r="H36" s="13">
         <v>0</v>
       </c>
@@ -10249,19 +10249,19 @@
       <c r="F38" s="33"/>
       <c r="G38" s="3"/>
       <c r="H38" s="3"/>
-      <c r="I38" s="154" t="s">
+      <c r="I38" s="165" t="s">
         <v>126</v>
       </c>
-      <c r="J38" s="154"/>
-      <c r="K38" s="154"/>
-      <c r="L38" s="154"/>
-      <c r="M38" s="154"/>
-      <c r="N38" s="154"/>
-      <c r="O38" s="154"/>
-      <c r="P38" s="154"/>
-      <c r="Q38" s="154"/>
-      <c r="R38" s="154"/>
-      <c r="S38" s="154"/>
+      <c r="J38" s="165"/>
+      <c r="K38" s="165"/>
+      <c r="L38" s="165"/>
+      <c r="M38" s="165"/>
+      <c r="N38" s="165"/>
+      <c r="O38" s="165"/>
+      <c r="P38" s="165"/>
+      <c r="Q38" s="165"/>
+      <c r="R38" s="165"/>
+      <c r="S38" s="165"/>
       <c r="T38" s="3"/>
       <c r="W38" s="53">
         <v>0.02</v>
@@ -11426,7 +11426,7 @@
       </c>
     </row>
     <row r="67" spans="14:34" x14ac:dyDescent="0.2">
-      <c r="N67" s="155"/>
+      <c r="N67" s="166"/>
       <c r="O67" s="10"/>
       <c r="P67" s="11"/>
       <c r="Q67" s="11"/>
@@ -11471,7 +11471,7 @@
       </c>
     </row>
     <row r="68" spans="14:34" x14ac:dyDescent="0.2">
-      <c r="N68" s="155"/>
+      <c r="N68" s="166"/>
       <c r="O68" s="10"/>
       <c r="P68" s="11"/>
       <c r="Q68" s="11"/>
@@ -11516,7 +11516,7 @@
       </c>
     </row>
     <row r="69" spans="14:34" x14ac:dyDescent="0.2">
-      <c r="N69" s="155"/>
+      <c r="N69" s="166"/>
       <c r="O69" s="10"/>
       <c r="P69" s="11"/>
       <c r="Q69" s="11"/>
@@ -11561,7 +11561,7 @@
       </c>
     </row>
     <row r="70" spans="14:34" x14ac:dyDescent="0.2">
-      <c r="N70" s="155"/>
+      <c r="N70" s="166"/>
       <c r="O70" s="10"/>
       <c r="P70" s="11"/>
       <c r="Q70" s="11"/>
@@ -11606,7 +11606,7 @@
       </c>
     </row>
     <row r="71" spans="14:34" x14ac:dyDescent="0.2">
-      <c r="N71" s="155"/>
+      <c r="N71" s="166"/>
       <c r="O71" s="10"/>
       <c r="P71" s="11"/>
       <c r="Q71" s="11"/>
@@ -11694,11 +11694,11 @@
       </c>
     </row>
     <row r="73" spans="14:34" x14ac:dyDescent="0.2">
-      <c r="P73" s="156"/>
-      <c r="Q73" s="156"/>
-      <c r="R73" s="156"/>
-      <c r="S73" s="156"/>
-      <c r="T73" s="156"/>
+      <c r="P73" s="167"/>
+      <c r="Q73" s="167"/>
+      <c r="R73" s="167"/>
+      <c r="S73" s="167"/>
+      <c r="T73" s="167"/>
       <c r="W73" s="53">
         <v>0.06</v>
       </c>
@@ -13789,15 +13789,8 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="1"/>
+  <sheetProtection sheet="1" selectLockedCells="1"/>
   <mergeCells count="17">
-    <mergeCell ref="C3:S3"/>
-    <mergeCell ref="I5:S6"/>
-    <mergeCell ref="G7:G17"/>
-    <mergeCell ref="C14:D15"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="C17:D21"/>
-    <mergeCell ref="I19:S19"/>
     <mergeCell ref="I38:S38"/>
     <mergeCell ref="N67:N71"/>
     <mergeCell ref="P73:T73"/>
@@ -13808,6 +13801,13 @@
     <mergeCell ref="C30:D31"/>
     <mergeCell ref="C32:D33"/>
     <mergeCell ref="C34:D35"/>
+    <mergeCell ref="C3:S3"/>
+    <mergeCell ref="I5:S6"/>
+    <mergeCell ref="G7:G17"/>
+    <mergeCell ref="C14:D15"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="C17:D21"/>
+    <mergeCell ref="I19:S19"/>
   </mergeCells>
   <conditionalFormatting sqref="I7:S17">
     <cfRule type="colorScale" priority="1">
@@ -14856,7 +14856,7 @@
       <c r="M66" s="3"/>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="1"/>
+  <sheetProtection sheet="1" selectLockedCells="1"/>
   <mergeCells count="6">
     <mergeCell ref="B5:M5"/>
     <mergeCell ref="C13:L13"/>
@@ -14981,17 +14981,17 @@
     <row r="10" spans="2:13" ht="31" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
-      <c r="D10" s="146" t="s">
+      <c r="D10" s="144" t="s">
         <v>146</v>
       </c>
-      <c r="E10" s="146"/>
-      <c r="F10" s="146"/>
-      <c r="G10" s="146"/>
-      <c r="H10" s="146"/>
-      <c r="I10" s="146"/>
-      <c r="J10" s="146"/>
-      <c r="K10" s="146"/>
-      <c r="L10" s="146"/>
+      <c r="E10" s="144"/>
+      <c r="F10" s="144"/>
+      <c r="G10" s="144"/>
+      <c r="H10" s="144"/>
+      <c r="I10" s="144"/>
+      <c r="J10" s="144"/>
+      <c r="K10" s="144"/>
+      <c r="L10" s="144"/>
       <c r="M10" s="3"/>
     </row>
     <row r="11" spans="2:13" x14ac:dyDescent="0.2">
@@ -15011,17 +15011,17 @@
     <row r="12" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
-      <c r="D12" s="146" t="s">
+      <c r="D12" s="144" t="s">
         <v>101</v>
       </c>
-      <c r="E12" s="146"/>
-      <c r="F12" s="146"/>
-      <c r="G12" s="146"/>
-      <c r="H12" s="146"/>
-      <c r="I12" s="146"/>
-      <c r="J12" s="146"/>
-      <c r="K12" s="146"/>
-      <c r="L12" s="146"/>
+      <c r="E12" s="144"/>
+      <c r="F12" s="144"/>
+      <c r="G12" s="144"/>
+      <c r="H12" s="144"/>
+      <c r="I12" s="144"/>
+      <c r="J12" s="144"/>
+      <c r="K12" s="144"/>
+      <c r="L12" s="144"/>
       <c r="M12" s="3"/>
     </row>
     <row r="13" spans="2:13" x14ac:dyDescent="0.2">
@@ -15041,17 +15041,17 @@
     <row r="14" spans="2:13" ht="45.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
-      <c r="D14" s="146" t="s">
+      <c r="D14" s="144" t="s">
         <v>129</v>
       </c>
-      <c r="E14" s="146"/>
-      <c r="F14" s="146"/>
-      <c r="G14" s="146"/>
-      <c r="H14" s="146"/>
-      <c r="I14" s="146"/>
-      <c r="J14" s="146"/>
-      <c r="K14" s="146"/>
-      <c r="L14" s="146"/>
+      <c r="E14" s="144"/>
+      <c r="F14" s="144"/>
+      <c r="G14" s="144"/>
+      <c r="H14" s="144"/>
+      <c r="I14" s="144"/>
+      <c r="J14" s="144"/>
+      <c r="K14" s="144"/>
+      <c r="L14" s="144"/>
       <c r="M14" s="3"/>
     </row>
     <row r="15" spans="2:13" x14ac:dyDescent="0.2">
@@ -15071,17 +15071,17 @@
     <row r="16" spans="2:13" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
-      <c r="D16" s="146" t="s">
+      <c r="D16" s="144" t="s">
         <v>147</v>
       </c>
-      <c r="E16" s="146"/>
-      <c r="F16" s="146"/>
-      <c r="G16" s="146"/>
-      <c r="H16" s="146"/>
-      <c r="I16" s="146"/>
-      <c r="J16" s="146"/>
-      <c r="K16" s="146"/>
-      <c r="L16" s="146"/>
+      <c r="E16" s="144"/>
+      <c r="F16" s="144"/>
+      <c r="G16" s="144"/>
+      <c r="H16" s="144"/>
+      <c r="I16" s="144"/>
+      <c r="J16" s="144"/>
+      <c r="K16" s="144"/>
+      <c r="L16" s="144"/>
       <c r="M16" s="3"/>
     </row>
     <row r="17" spans="2:13" x14ac:dyDescent="0.2">
@@ -15101,17 +15101,17 @@
     <row r="18" spans="2:13" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
-      <c r="D18" s="146" t="s">
+      <c r="D18" s="144" t="s">
         <v>97</v>
       </c>
-      <c r="E18" s="146"/>
-      <c r="F18" s="146"/>
-      <c r="G18" s="146"/>
-      <c r="H18" s="146"/>
-      <c r="I18" s="146"/>
-      <c r="J18" s="146"/>
-      <c r="K18" s="146"/>
-      <c r="L18" s="146"/>
+      <c r="E18" s="144"/>
+      <c r="F18" s="144"/>
+      <c r="G18" s="144"/>
+      <c r="H18" s="144"/>
+      <c r="I18" s="144"/>
+      <c r="J18" s="144"/>
+      <c r="K18" s="144"/>
+      <c r="L18" s="144"/>
       <c r="M18" s="3"/>
     </row>
     <row r="19" spans="2:13" x14ac:dyDescent="0.2">
@@ -15131,17 +15131,17 @@
     <row r="20" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
-      <c r="D20" s="146" t="s">
+      <c r="D20" s="144" t="s">
         <v>130</v>
       </c>
-      <c r="E20" s="146"/>
-      <c r="F20" s="146"/>
-      <c r="G20" s="146"/>
-      <c r="H20" s="146"/>
-      <c r="I20" s="146"/>
-      <c r="J20" s="146"/>
-      <c r="K20" s="146"/>
-      <c r="L20" s="146"/>
+      <c r="E20" s="144"/>
+      <c r="F20" s="144"/>
+      <c r="G20" s="144"/>
+      <c r="H20" s="144"/>
+      <c r="I20" s="144"/>
+      <c r="J20" s="144"/>
+      <c r="K20" s="144"/>
+      <c r="L20" s="144"/>
       <c r="M20" s="3"/>
     </row>
     <row r="21" spans="2:13" x14ac:dyDescent="0.2">
@@ -15191,17 +15191,17 @@
     <row r="24" spans="2:13" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" s="3"/>
       <c r="C24" s="4"/>
-      <c r="D24" s="146" t="s">
+      <c r="D24" s="144" t="s">
         <v>131</v>
       </c>
-      <c r="E24" s="146"/>
-      <c r="F24" s="146"/>
-      <c r="G24" s="146"/>
-      <c r="H24" s="146"/>
-      <c r="I24" s="146"/>
-      <c r="J24" s="146"/>
-      <c r="K24" s="146"/>
-      <c r="L24" s="146"/>
+      <c r="E24" s="144"/>
+      <c r="F24" s="144"/>
+      <c r="G24" s="144"/>
+      <c r="H24" s="144"/>
+      <c r="I24" s="144"/>
+      <c r="J24" s="144"/>
+      <c r="K24" s="144"/>
+      <c r="L24" s="144"/>
       <c r="M24" s="3"/>
     </row>
     <row r="25" spans="2:13" x14ac:dyDescent="0.2">
@@ -15221,17 +15221,17 @@
     <row r="26" spans="2:13" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
-      <c r="D26" s="146" t="s">
+      <c r="D26" s="144" t="s">
         <v>132</v>
       </c>
-      <c r="E26" s="146"/>
-      <c r="F26" s="146"/>
-      <c r="G26" s="146"/>
-      <c r="H26" s="146"/>
-      <c r="I26" s="146"/>
-      <c r="J26" s="146"/>
-      <c r="K26" s="146"/>
-      <c r="L26" s="146"/>
+      <c r="E26" s="144"/>
+      <c r="F26" s="144"/>
+      <c r="G26" s="144"/>
+      <c r="H26" s="144"/>
+      <c r="I26" s="144"/>
+      <c r="J26" s="144"/>
+      <c r="K26" s="144"/>
+      <c r="L26" s="144"/>
       <c r="M26" s="3"/>
     </row>
     <row r="27" spans="2:13" x14ac:dyDescent="0.2">
@@ -15251,17 +15251,17 @@
     <row r="28" spans="2:13" ht="31" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
-      <c r="D28" s="146" t="s">
+      <c r="D28" s="144" t="s">
         <v>98</v>
       </c>
-      <c r="E28" s="146"/>
-      <c r="F28" s="146"/>
-      <c r="G28" s="146"/>
-      <c r="H28" s="146"/>
-      <c r="I28" s="146"/>
-      <c r="J28" s="146"/>
-      <c r="K28" s="146"/>
-      <c r="L28" s="146"/>
+      <c r="E28" s="144"/>
+      <c r="F28" s="144"/>
+      <c r="G28" s="144"/>
+      <c r="H28" s="144"/>
+      <c r="I28" s="144"/>
+      <c r="J28" s="144"/>
+      <c r="K28" s="144"/>
+      <c r="L28" s="144"/>
       <c r="M28" s="3"/>
     </row>
     <row r="29" spans="2:13" x14ac:dyDescent="0.2">
@@ -15281,17 +15281,17 @@
     <row r="30" spans="2:13" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B30" s="3"/>
       <c r="C30" s="3"/>
-      <c r="D30" s="146" t="s">
+      <c r="D30" s="144" t="s">
         <v>49</v>
       </c>
-      <c r="E30" s="146"/>
-      <c r="F30" s="146"/>
-      <c r="G30" s="146"/>
-      <c r="H30" s="146"/>
-      <c r="I30" s="146"/>
-      <c r="J30" s="146"/>
-      <c r="K30" s="146"/>
-      <c r="L30" s="146"/>
+      <c r="E30" s="144"/>
+      <c r="F30" s="144"/>
+      <c r="G30" s="144"/>
+      <c r="H30" s="144"/>
+      <c r="I30" s="144"/>
+      <c r="J30" s="144"/>
+      <c r="K30" s="144"/>
+      <c r="L30" s="144"/>
       <c r="M30" s="3"/>
     </row>
     <row r="31" spans="2:13" x14ac:dyDescent="0.2">
@@ -15365,8 +15365,13 @@
       <c r="M35" s="3"/>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="1"/>
+  <sheetProtection sheet="1" selectLockedCells="1"/>
   <mergeCells count="12">
+    <mergeCell ref="C5:L5"/>
+    <mergeCell ref="D20:L20"/>
+    <mergeCell ref="D8:L8"/>
+    <mergeCell ref="D10:L10"/>
+    <mergeCell ref="D26:L26"/>
     <mergeCell ref="D30:L30"/>
     <mergeCell ref="D14:L14"/>
     <mergeCell ref="D12:L12"/>
@@ -15374,11 +15379,6 @@
     <mergeCell ref="D16:L16"/>
     <mergeCell ref="D24:L24"/>
     <mergeCell ref="D28:L28"/>
-    <mergeCell ref="C5:L5"/>
-    <mergeCell ref="D20:L20"/>
-    <mergeCell ref="D8:L8"/>
-    <mergeCell ref="D10:L10"/>
-    <mergeCell ref="D26:L26"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
updating figures with new pregnancy numbers
</commit_message>
<xml_diff>
--- a/Burden-of-Illness-Tool/MADMC B19 Pregancy Outcome Estimate Tool_Sept2025.xlsx
+++ b/Burden-of-Illness-Tool/MADMC B19 Pregancy Outcome Estimate Tool_Sept2025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ritesh/Desktop/Scenario-Modeling-of-Human-Parvovirus-B19/Burden-of-Illness-Tool/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AD92736-0293-054F-AD96-9E382C5CB624}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CBE8594-71BA-044E-82D7-BA9F1232F24F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-30240" yWindow="1620" windowWidth="30260" windowHeight="18980" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-30240" yWindow="1600" windowWidth="30240" windowHeight="18980" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="2" r:id="rId1"/>
@@ -3037,9 +3037,18 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="30" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1" indent="2"/>
     </xf>
@@ -3058,14 +3067,26 @@
     <xf numFmtId="0" fontId="14" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -3073,9 +3094,6 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -3099,24 +3117,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3326,10 +3326,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>500</c:v>
+                  <c:v>3750</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>37.5</c:v>
+                  <c:v>281.25</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3992,13 +3992,13 @@
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>-12.5</c:v>
+                  <c:v>-93.75</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-18.75</c:v>
+                  <c:v>-262.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>18.75</c:v>
+                  <c:v>140.625</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4057,13 +4057,13 @@
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>12.5</c:v>
+                  <c:v>93.75</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>37.5</c:v>
+                  <c:v>-206.25</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-18.75</c:v>
+                  <c:v>-140.625</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6366,42 +6366,42 @@
       <c r="E1" s="27"/>
     </row>
     <row r="3" spans="1:29" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B3" s="151" t="s">
+      <c r="B3" s="144" t="s">
         <v>143</v>
       </c>
-      <c r="C3" s="151"/>
-      <c r="D3" s="151"/>
-      <c r="E3" s="151"/>
-      <c r="F3" s="151"/>
-      <c r="G3" s="151"/>
-      <c r="H3" s="151"/>
-      <c r="I3" s="151"/>
-      <c r="J3" s="151"/>
-      <c r="K3" s="151"/>
-      <c r="L3" s="151"/>
-      <c r="M3" s="151"/>
-      <c r="N3" s="151"/>
-      <c r="O3" s="151"/>
-      <c r="P3" s="151"/>
-      <c r="Q3" s="151"/>
+      <c r="C3" s="144"/>
+      <c r="D3" s="144"/>
+      <c r="E3" s="144"/>
+      <c r="F3" s="144"/>
+      <c r="G3" s="144"/>
+      <c r="H3" s="144"/>
+      <c r="I3" s="144"/>
+      <c r="J3" s="144"/>
+      <c r="K3" s="144"/>
+      <c r="L3" s="144"/>
+      <c r="M3" s="144"/>
+      <c r="N3" s="144"/>
+      <c r="O3" s="144"/>
+      <c r="P3" s="144"/>
+      <c r="Q3" s="144"/>
     </row>
     <row r="4" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="B4" s="151"/>
-      <c r="C4" s="151"/>
-      <c r="D4" s="151"/>
-      <c r="E4" s="151"/>
-      <c r="F4" s="151"/>
-      <c r="G4" s="151"/>
-      <c r="H4" s="151"/>
-      <c r="I4" s="151"/>
-      <c r="J4" s="151"/>
-      <c r="K4" s="151"/>
-      <c r="L4" s="151"/>
-      <c r="M4" s="151"/>
-      <c r="N4" s="151"/>
-      <c r="O4" s="151"/>
-      <c r="P4" s="151"/>
-      <c r="Q4" s="151"/>
+      <c r="B4" s="144"/>
+      <c r="C4" s="144"/>
+      <c r="D4" s="144"/>
+      <c r="E4" s="144"/>
+      <c r="F4" s="144"/>
+      <c r="G4" s="144"/>
+      <c r="H4" s="144"/>
+      <c r="I4" s="144"/>
+      <c r="J4" s="144"/>
+      <c r="K4" s="144"/>
+      <c r="L4" s="144"/>
+      <c r="M4" s="144"/>
+      <c r="N4" s="144"/>
+      <c r="O4" s="144"/>
+      <c r="P4" s="144"/>
+      <c r="Q4" s="144"/>
     </row>
     <row r="5" spans="1:29" ht="16" x14ac:dyDescent="0.2">
       <c r="B5" s="111"/>
@@ -6483,17 +6483,17 @@
       <c r="F8" s="32"/>
       <c r="G8" s="4"/>
       <c r="H8" s="3"/>
-      <c r="I8" s="152" t="str">
+      <c r="I8" s="145" t="str">
         <f>_xlfn.CONCAT("Based on ", C9, " pregnancies in the population and historic estimates of parvovirus immunity, mother infection risk, fetal infection risk, and risk of severe fetal outcomes (Table 1), the expected number of severe fetal outcomes due to parvovirus is ",C22,". Under a best case scenario of higher immunity, lower infection rates, and lower complication rates, the number of severe fetal outcomes due to PVB19 could be as low as ", F22, ", while under a worst case scenario the number of severe fetal outcomes may be as high as ", G22, " in the population with ", C9, " pregnancies (Figure 1, Table 2).")</f>
         <v>Based on 100000 pregnancies in the population and historic estimates of parvovirus immunity, mother infection risk, fetal infection risk, and risk of severe fetal outcomes (Table 1), the expected number of severe fetal outcomes due to parvovirus is . Under a best case scenario of higher immunity, lower infection rates, and lower complication rates, the number of severe fetal outcomes due to PVB19 could be as low as , while under a worst case scenario the number of severe fetal outcomes may be as high as  in the population with 100000 pregnancies (Figure 1, Table 2).</v>
       </c>
-      <c r="J8" s="152"/>
-      <c r="K8" s="152"/>
-      <c r="L8" s="152"/>
-      <c r="M8" s="152"/>
-      <c r="N8" s="152"/>
-      <c r="O8" s="152"/>
-      <c r="P8" s="152"/>
+      <c r="J8" s="145"/>
+      <c r="K8" s="145"/>
+      <c r="L8" s="145"/>
+      <c r="M8" s="145"/>
+      <c r="N8" s="145"/>
+      <c r="O8" s="145"/>
+      <c r="P8" s="145"/>
       <c r="Q8" s="33"/>
       <c r="R8" s="18"/>
       <c r="X8" s="9"/>
@@ -6520,14 +6520,14 @@
       <c r="F9" s="71"/>
       <c r="G9" s="4"/>
       <c r="H9" s="33"/>
-      <c r="I9" s="152"/>
-      <c r="J9" s="152"/>
-      <c r="K9" s="152"/>
-      <c r="L9" s="152"/>
-      <c r="M9" s="152"/>
-      <c r="N9" s="152"/>
-      <c r="O9" s="152"/>
-      <c r="P9" s="152"/>
+      <c r="I9" s="145"/>
+      <c r="J9" s="145"/>
+      <c r="K9" s="145"/>
+      <c r="L9" s="145"/>
+      <c r="M9" s="145"/>
+      <c r="N9" s="145"/>
+      <c r="O9" s="145"/>
+      <c r="P9" s="145"/>
       <c r="Q9" s="33"/>
       <c r="R9" s="18"/>
       <c r="X9" s="8"/>
@@ -6554,14 +6554,14 @@
       <c r="F10" s="72"/>
       <c r="G10" s="4"/>
       <c r="H10" s="33"/>
-      <c r="I10" s="152"/>
-      <c r="J10" s="152"/>
-      <c r="K10" s="152"/>
-      <c r="L10" s="152"/>
-      <c r="M10" s="152"/>
-      <c r="N10" s="152"/>
-      <c r="O10" s="152"/>
-      <c r="P10" s="152"/>
+      <c r="I10" s="145"/>
+      <c r="J10" s="145"/>
+      <c r="K10" s="145"/>
+      <c r="L10" s="145"/>
+      <c r="M10" s="145"/>
+      <c r="N10" s="145"/>
+      <c r="O10" s="145"/>
+      <c r="P10" s="145"/>
       <c r="Q10" s="33"/>
       <c r="R10" s="18"/>
       <c r="X10" s="8"/>
@@ -6577,7 +6577,7 @@
         <v>112</v>
       </c>
       <c r="C11" s="110">
-        <v>0.01</v>
+        <v>7.4999999999999997E-2</v>
       </c>
       <c r="D11" s="110">
         <v>5.0000000000000001E-3</v>
@@ -6641,12 +6641,12 @@
     </row>
     <row r="13" spans="1:29" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="3"/>
-      <c r="B13" s="146" t="s">
+      <c r="B13" s="149" t="s">
         <v>114</v>
       </c>
-      <c r="C13" s="146"/>
-      <c r="D13" s="146"/>
-      <c r="E13" s="146"/>
+      <c r="C13" s="149"/>
+      <c r="D13" s="149"/>
+      <c r="E13" s="149"/>
       <c r="F13" s="72"/>
       <c r="G13" s="3"/>
       <c r="H13" s="3"/>
@@ -6725,20 +6725,20 @@
     </row>
     <row r="17" spans="1:18" ht="33.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3"/>
-      <c r="B17" s="147" t="s">
+      <c r="B17" s="150" t="s">
         <v>99</v>
       </c>
       <c r="C17" s="77" t="s">
         <v>6</v>
       </c>
-      <c r="D17" s="149" t="s">
+      <c r="D17" s="152" t="s">
         <v>16</v>
       </c>
-      <c r="E17" s="150"/>
-      <c r="F17" s="149" t="s">
+      <c r="E17" s="153"/>
+      <c r="F17" s="152" t="s">
         <v>19</v>
       </c>
-      <c r="G17" s="150"/>
+      <c r="G17" s="153"/>
       <c r="H17" s="75"/>
       <c r="I17" s="5"/>
       <c r="J17" s="5"/>
@@ -6753,7 +6753,7 @@
     </row>
     <row r="18" spans="1:18" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3"/>
-      <c r="B18" s="148"/>
+      <c r="B18" s="151"/>
       <c r="C18" s="78" t="s">
         <v>41</v>
       </c>
@@ -6825,18 +6825,18 @@
       </c>
       <c r="C20" s="54">
         <f>C19*C11</f>
-        <v>500</v>
+        <v>3750</v>
       </c>
       <c r="D20" s="79">
         <f>D19*C11</f>
-        <v>750</v>
+        <v>5625</v>
       </c>
       <c r="E20" s="76">
         <f t="shared" ref="E20:G21" si="0">E19*C11</f>
-        <v>250</v>
+        <v>1875</v>
       </c>
       <c r="F20" s="76">
-        <f t="shared" si="0"/>
+        <f>F19*D11</f>
         <v>125</v>
       </c>
       <c r="G20" s="132">
@@ -6862,15 +6862,15 @@
       </c>
       <c r="C21" s="133">
         <f>C20*C12</f>
-        <v>37.5</v>
+        <v>281.25</v>
       </c>
       <c r="D21" s="134">
         <f>D20*C12</f>
-        <v>56.25</v>
+        <v>421.875</v>
       </c>
       <c r="E21" s="135">
         <f t="shared" si="0"/>
-        <v>18.75</v>
+        <v>140.625</v>
       </c>
       <c r="F21" s="135">
         <f t="shared" si="0"/>
@@ -6938,14 +6938,14 @@
     </row>
     <row r="24" spans="1:18" ht="44" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="3"/>
-      <c r="B24" s="145" t="s">
+      <c r="B24" s="148" t="s">
         <v>35</v>
       </c>
-      <c r="C24" s="145"/>
-      <c r="D24" s="145"/>
-      <c r="E24" s="145"/>
-      <c r="F24" s="145"/>
-      <c r="G24" s="145"/>
+      <c r="C24" s="148"/>
+      <c r="D24" s="148"/>
+      <c r="E24" s="148"/>
+      <c r="F24" s="148"/>
+      <c r="G24" s="148"/>
       <c r="H24" s="38"/>
       <c r="I24" s="38"/>
       <c r="J24" s="3"/>
@@ -6960,14 +6960,14 @@
     </row>
     <row r="25" spans="1:18" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="3"/>
-      <c r="B25" s="145" t="s">
+      <c r="B25" s="148" t="s">
         <v>39</v>
       </c>
-      <c r="C25" s="145"/>
-      <c r="D25" s="145"/>
-      <c r="E25" s="145"/>
-      <c r="F25" s="145"/>
-      <c r="G25" s="145"/>
+      <c r="C25" s="148"/>
+      <c r="D25" s="148"/>
+      <c r="E25" s="148"/>
+      <c r="F25" s="148"/>
+      <c r="G25" s="148"/>
       <c r="H25" s="38"/>
       <c r="I25" s="44"/>
       <c r="J25" s="74"/>
@@ -7204,14 +7204,14 @@
     </row>
     <row r="37" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="3"/>
-      <c r="B37" s="153" t="s">
+      <c r="B37" s="147" t="s">
         <v>24</v>
       </c>
-      <c r="C37" s="153"/>
-      <c r="D37" s="153"/>
-      <c r="E37" s="153"/>
-      <c r="F37" s="153"/>
-      <c r="G37" s="153"/>
+      <c r="C37" s="147"/>
+      <c r="D37" s="147"/>
+      <c r="E37" s="147"/>
+      <c r="F37" s="147"/>
+      <c r="G37" s="147"/>
       <c r="H37" s="3"/>
       <c r="I37" s="36"/>
       <c r="J37" s="3"/>
@@ -7226,14 +7226,14 @@
     </row>
     <row r="38" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A38" s="3"/>
-      <c r="B38" s="144" t="s">
+      <c r="B38" s="146" t="s">
         <v>25</v>
       </c>
-      <c r="C38" s="144"/>
-      <c r="D38" s="144"/>
-      <c r="E38" s="144"/>
-      <c r="F38" s="144"/>
-      <c r="G38" s="144"/>
+      <c r="C38" s="146"/>
+      <c r="D38" s="146"/>
+      <c r="E38" s="146"/>
+      <c r="F38" s="146"/>
+      <c r="G38" s="146"/>
       <c r="H38" s="33"/>
       <c r="I38" s="34"/>
       <c r="J38" s="3"/>
@@ -7248,14 +7248,14 @@
     </row>
     <row r="39" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A39" s="3"/>
-      <c r="B39" s="144" t="s">
+      <c r="B39" s="146" t="s">
         <v>30</v>
       </c>
-      <c r="C39" s="144"/>
-      <c r="D39" s="144"/>
-      <c r="E39" s="144"/>
-      <c r="F39" s="144"/>
-      <c r="G39" s="144"/>
+      <c r="C39" s="146"/>
+      <c r="D39" s="146"/>
+      <c r="E39" s="146"/>
+      <c r="F39" s="146"/>
+      <c r="G39" s="146"/>
       <c r="H39" s="33"/>
       <c r="I39" s="34"/>
       <c r="J39" s="3"/>
@@ -7270,14 +7270,14 @@
     </row>
     <row r="40" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="3"/>
-      <c r="B40" s="144" t="s">
+      <c r="B40" s="146" t="s">
         <v>31</v>
       </c>
-      <c r="C40" s="144"/>
-      <c r="D40" s="144"/>
-      <c r="E40" s="144"/>
-      <c r="F40" s="144"/>
-      <c r="G40" s="144"/>
+      <c r="C40" s="146"/>
+      <c r="D40" s="146"/>
+      <c r="E40" s="146"/>
+      <c r="F40" s="146"/>
+      <c r="G40" s="146"/>
       <c r="H40" s="33"/>
       <c r="I40" s="34"/>
       <c r="J40" s="3"/>
@@ -7292,14 +7292,14 @@
     </row>
     <row r="41" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="3"/>
-      <c r="B41" s="144" t="s">
+      <c r="B41" s="146" t="s">
         <v>32</v>
       </c>
-      <c r="C41" s="144"/>
-      <c r="D41" s="144"/>
-      <c r="E41" s="144"/>
-      <c r="F41" s="144"/>
-      <c r="G41" s="144"/>
+      <c r="C41" s="146"/>
+      <c r="D41" s="146"/>
+      <c r="E41" s="146"/>
+      <c r="F41" s="146"/>
+      <c r="G41" s="146"/>
       <c r="H41" s="33"/>
       <c r="I41" s="34"/>
       <c r="J41" s="3"/>
@@ -7369,23 +7369,23 @@
       </c>
       <c r="C47" s="41">
         <f>F47-E47</f>
-        <v>-12.5</v>
+        <v>-93.75</v>
       </c>
       <c r="D47" s="41">
         <f>G47-E47</f>
-        <v>12.5</v>
+        <v>93.75</v>
       </c>
       <c r="E47" s="41">
         <f>C21</f>
-        <v>37.5</v>
+        <v>281.25</v>
       </c>
       <c r="F47" s="1">
         <f>C20*D12</f>
-        <v>25</v>
+        <v>187.5</v>
       </c>
       <c r="G47" s="1">
         <f>C20*E12</f>
-        <v>50</v>
+        <v>375</v>
       </c>
     </row>
     <row r="48" spans="1:18" ht="32" x14ac:dyDescent="0.2">
@@ -7394,15 +7394,15 @@
       </c>
       <c r="C48" s="41">
         <f>F48-E48</f>
-        <v>-18.75</v>
+        <v>-262.5</v>
       </c>
       <c r="D48" s="41">
         <f>G48-E48</f>
-        <v>37.5</v>
+        <v>-206.25</v>
       </c>
       <c r="E48" s="41">
         <f>C21</f>
-        <v>37.5</v>
+        <v>281.25</v>
       </c>
       <c r="F48" s="1">
         <f>(C9-(C9*C10))*D11*C12</f>
@@ -7419,33 +7419,28 @@
       </c>
       <c r="C49" s="41">
         <f>F49-E49</f>
-        <v>18.75</v>
+        <v>140.625</v>
       </c>
       <c r="D49" s="41">
         <f>G49-E49</f>
-        <v>-18.75</v>
+        <v>-140.625</v>
       </c>
       <c r="E49" s="41">
         <f>C21</f>
-        <v>37.5</v>
+        <v>281.25</v>
       </c>
       <c r="F49" s="1">
         <f>(C9-(C9*D10))*C11*C12</f>
-        <v>56.25</v>
+        <v>421.875</v>
       </c>
       <c r="G49" s="1">
         <f>(C9-(C9*E10))*C11*C12</f>
-        <v>18.75</v>
+        <v>140.625</v>
       </c>
     </row>
   </sheetData>
   <sheetProtection sheet="1" selectLockedCells="1"/>
   <mergeCells count="13">
-    <mergeCell ref="B3:Q4"/>
-    <mergeCell ref="I8:P10"/>
-    <mergeCell ref="B38:G38"/>
-    <mergeCell ref="B37:G37"/>
-    <mergeCell ref="B39:G39"/>
     <mergeCell ref="B41:G41"/>
     <mergeCell ref="B24:G24"/>
     <mergeCell ref="B25:G25"/>
@@ -7454,6 +7449,11 @@
     <mergeCell ref="D17:E17"/>
     <mergeCell ref="F17:G17"/>
     <mergeCell ref="B40:G40"/>
+    <mergeCell ref="B3:Q4"/>
+    <mergeCell ref="I8:P10"/>
+    <mergeCell ref="B38:G38"/>
+    <mergeCell ref="B37:G37"/>
+    <mergeCell ref="B39:G39"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -7504,25 +7504,25 @@
       <c r="F2" s="7"/>
     </row>
     <row r="3" spans="2:34" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C3" s="154" t="s">
+      <c r="C3" s="161" t="s">
         <v>144</v>
       </c>
-      <c r="D3" s="154"/>
-      <c r="E3" s="154"/>
-      <c r="F3" s="154"/>
-      <c r="G3" s="154"/>
-      <c r="H3" s="154"/>
-      <c r="I3" s="154"/>
-      <c r="J3" s="154"/>
-      <c r="K3" s="154"/>
-      <c r="L3" s="154"/>
-      <c r="M3" s="154"/>
-      <c r="N3" s="154"/>
-      <c r="O3" s="154"/>
-      <c r="P3" s="154"/>
-      <c r="Q3" s="154"/>
-      <c r="R3" s="154"/>
-      <c r="S3" s="154"/>
+      <c r="D3" s="161"/>
+      <c r="E3" s="161"/>
+      <c r="F3" s="161"/>
+      <c r="G3" s="161"/>
+      <c r="H3" s="161"/>
+      <c r="I3" s="161"/>
+      <c r="J3" s="161"/>
+      <c r="K3" s="161"/>
+      <c r="L3" s="161"/>
+      <c r="M3" s="161"/>
+      <c r="N3" s="161"/>
+      <c r="O3" s="161"/>
+      <c r="P3" s="161"/>
+      <c r="Q3" s="161"/>
+      <c r="R3" s="161"/>
+      <c r="S3" s="161"/>
     </row>
     <row r="5" spans="2:34" ht="26.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B5" s="3"/>
@@ -7534,20 +7534,20 @@
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
-      <c r="I5" s="155" t="str">
+      <c r="I5" s="162" t="str">
         <f>_xlfn.CONCAT("Figure 1. Estimated Number of Severe Fetal Outcomes Under Potential Immunity and Infection Rate Scenarios, based on ",D7," Pregnancies")</f>
         <v>Figure 1. Estimated Number of Severe Fetal Outcomes Under Potential Immunity and Infection Rate Scenarios, based on 100000 Pregnancies</v>
       </c>
-      <c r="J5" s="155"/>
-      <c r="K5" s="155"/>
-      <c r="L5" s="155"/>
-      <c r="M5" s="155"/>
-      <c r="N5" s="155"/>
-      <c r="O5" s="155"/>
-      <c r="P5" s="155"/>
-      <c r="Q5" s="155"/>
-      <c r="R5" s="155"/>
-      <c r="S5" s="155"/>
+      <c r="J5" s="162"/>
+      <c r="K5" s="162"/>
+      <c r="L5" s="162"/>
+      <c r="M5" s="162"/>
+      <c r="N5" s="162"/>
+      <c r="O5" s="162"/>
+      <c r="P5" s="162"/>
+      <c r="Q5" s="162"/>
+      <c r="R5" s="162"/>
+      <c r="S5" s="162"/>
       <c r="T5" s="3"/>
       <c r="W5" s="51" t="s">
         <v>22</v>
@@ -7568,17 +7568,17 @@
       <c r="F6" s="3"/>
       <c r="G6" s="3"/>
       <c r="H6" s="3"/>
-      <c r="I6" s="155"/>
-      <c r="J6" s="155"/>
-      <c r="K6" s="155"/>
-      <c r="L6" s="155"/>
-      <c r="M6" s="155"/>
-      <c r="N6" s="155"/>
-      <c r="O6" s="155"/>
-      <c r="P6" s="155"/>
-      <c r="Q6" s="155"/>
-      <c r="R6" s="155"/>
-      <c r="S6" s="155"/>
+      <c r="I6" s="162"/>
+      <c r="J6" s="162"/>
+      <c r="K6" s="162"/>
+      <c r="L6" s="162"/>
+      <c r="M6" s="162"/>
+      <c r="N6" s="162"/>
+      <c r="O6" s="162"/>
+      <c r="P6" s="162"/>
+      <c r="Q6" s="162"/>
+      <c r="R6" s="162"/>
+      <c r="S6" s="162"/>
       <c r="T6" s="3"/>
       <c r="W6" s="52" t="s">
         <v>4</v>
@@ -7621,7 +7621,7 @@
       </c>
       <c r="E7" s="46"/>
       <c r="F7" s="3"/>
-      <c r="G7" s="156" t="s">
+      <c r="G7" s="160" t="s">
         <v>127</v>
       </c>
       <c r="H7" s="13">
@@ -7719,7 +7719,7 @@
       </c>
       <c r="E8" s="47"/>
       <c r="F8" s="3"/>
-      <c r="G8" s="156"/>
+      <c r="G8" s="160"/>
       <c r="H8" s="13">
         <v>0.7</v>
       </c>
@@ -7815,7 +7815,7 @@
       </c>
       <c r="E9" s="47"/>
       <c r="F9" s="3"/>
-      <c r="G9" s="156"/>
+      <c r="G9" s="160"/>
       <c r="H9" s="13">
         <v>0.65</v>
       </c>
@@ -7911,7 +7911,7 @@
       </c>
       <c r="E10" s="48"/>
       <c r="F10" s="3"/>
-      <c r="G10" s="156"/>
+      <c r="G10" s="160"/>
       <c r="H10" s="13">
         <v>0.6</v>
       </c>
@@ -8003,7 +8003,7 @@
       <c r="D11" s="48"/>
       <c r="E11" s="48"/>
       <c r="F11" s="3"/>
-      <c r="G11" s="156"/>
+      <c r="G11" s="160"/>
       <c r="H11" s="13">
         <v>0.55000000000000004</v>
       </c>
@@ -8095,7 +8095,7 @@
       <c r="D12" s="3"/>
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
-      <c r="G12" s="156"/>
+      <c r="G12" s="160"/>
       <c r="H12" s="13">
         <v>0.5</v>
       </c>
@@ -8189,7 +8189,7 @@
       <c r="D13" s="24"/>
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
-      <c r="G13" s="156"/>
+      <c r="G13" s="160"/>
       <c r="H13" s="13">
         <v>0.45</v>
       </c>
@@ -8277,13 +8277,13 @@
     </row>
     <row r="14" spans="2:34" ht="29" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B14" s="3"/>
-      <c r="C14" s="157" t="s">
+      <c r="C14" s="163" t="s">
         <v>46</v>
       </c>
-      <c r="D14" s="158"/>
+      <c r="D14" s="164"/>
       <c r="E14" s="45"/>
       <c r="F14" s="3"/>
-      <c r="G14" s="156"/>
+      <c r="G14" s="160"/>
       <c r="H14" s="13">
         <v>0.4</v>
       </c>
@@ -8371,11 +8371,11 @@
     </row>
     <row r="15" spans="2:34" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="3"/>
-      <c r="C15" s="159"/>
-      <c r="D15" s="158"/>
+      <c r="C15" s="165"/>
+      <c r="D15" s="164"/>
       <c r="E15" s="45"/>
       <c r="F15" s="3"/>
-      <c r="G15" s="156"/>
+      <c r="G15" s="160"/>
       <c r="H15" s="13">
         <v>0.35</v>
       </c>
@@ -8463,13 +8463,13 @@
     </row>
     <row r="16" spans="2:34" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="3"/>
-      <c r="C16" s="160" t="s">
+      <c r="C16" s="166" t="s">
         <v>47</v>
       </c>
-      <c r="D16" s="161"/>
+      <c r="D16" s="167"/>
       <c r="E16" s="34"/>
       <c r="F16" s="3"/>
-      <c r="G16" s="156"/>
+      <c r="G16" s="160"/>
       <c r="H16" s="13">
         <v>0.3</v>
       </c>
@@ -8557,13 +8557,13 @@
     </row>
     <row r="17" spans="2:34" ht="17" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B17" s="3"/>
-      <c r="C17" s="160" t="s">
+      <c r="C17" s="166" t="s">
         <v>125</v>
       </c>
-      <c r="D17" s="161"/>
+      <c r="D17" s="167"/>
       <c r="E17" s="34"/>
       <c r="F17" s="3"/>
-      <c r="G17" s="156"/>
+      <c r="G17" s="160"/>
       <c r="H17" s="13">
         <v>0.25</v>
       </c>
@@ -8651,8 +8651,8 @@
     </row>
     <row r="18" spans="2:34" x14ac:dyDescent="0.2">
       <c r="B18" s="3"/>
-      <c r="C18" s="162"/>
-      <c r="D18" s="161"/>
+      <c r="C18" s="168"/>
+      <c r="D18" s="167"/>
       <c r="E18" s="34"/>
       <c r="F18" s="3"/>
       <c r="G18" s="3"/>
@@ -8730,25 +8730,25 @@
     </row>
     <row r="19" spans="2:34" x14ac:dyDescent="0.2">
       <c r="B19" s="3"/>
-      <c r="C19" s="162"/>
-      <c r="D19" s="161"/>
+      <c r="C19" s="168"/>
+      <c r="D19" s="167"/>
       <c r="E19" s="34"/>
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
       <c r="H19" s="3"/>
-      <c r="I19" s="165" t="s">
+      <c r="I19" s="154" t="s">
         <v>126</v>
       </c>
-      <c r="J19" s="165"/>
-      <c r="K19" s="165"/>
-      <c r="L19" s="165"/>
-      <c r="M19" s="165"/>
-      <c r="N19" s="165"/>
-      <c r="O19" s="165"/>
-      <c r="P19" s="165"/>
-      <c r="Q19" s="165"/>
-      <c r="R19" s="165"/>
-      <c r="S19" s="165"/>
+      <c r="J19" s="154"/>
+      <c r="K19" s="154"/>
+      <c r="L19" s="154"/>
+      <c r="M19" s="154"/>
+      <c r="N19" s="154"/>
+      <c r="O19" s="154"/>
+      <c r="P19" s="154"/>
+      <c r="Q19" s="154"/>
+      <c r="R19" s="154"/>
+      <c r="S19" s="154"/>
       <c r="T19" s="3"/>
       <c r="W19" s="53">
         <v>0.01</v>
@@ -8789,8 +8789,8 @@
     </row>
     <row r="20" spans="2:34" x14ac:dyDescent="0.2">
       <c r="B20" s="3"/>
-      <c r="C20" s="162"/>
-      <c r="D20" s="161"/>
+      <c r="C20" s="168"/>
+      <c r="D20" s="167"/>
       <c r="E20" s="34"/>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
@@ -8848,8 +8848,8 @@
     </row>
     <row r="21" spans="2:34" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B21" s="3"/>
-      <c r="C21" s="163"/>
-      <c r="D21" s="164"/>
+      <c r="C21" s="169"/>
+      <c r="D21" s="170"/>
       <c r="E21" s="34"/>
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
@@ -9029,20 +9029,20 @@
       <c r="F24" s="3"/>
       <c r="G24" s="3"/>
       <c r="H24" s="3"/>
-      <c r="I24" s="168" t="str">
+      <c r="I24" s="157" t="str">
         <f>_xlfn.CONCAT("Figure 2. Estimated Number of Severe Fetal Outcomes Under all Possible Immunity and Infection Rate Scenarios, based on ",D7," Pregnancies")</f>
         <v>Figure 2. Estimated Number of Severe Fetal Outcomes Under all Possible Immunity and Infection Rate Scenarios, based on 100000 Pregnancies</v>
       </c>
-      <c r="J24" s="168"/>
-      <c r="K24" s="168"/>
-      <c r="L24" s="168"/>
-      <c r="M24" s="168"/>
-      <c r="N24" s="168"/>
-      <c r="O24" s="168"/>
-      <c r="P24" s="168"/>
-      <c r="Q24" s="168"/>
-      <c r="R24" s="168"/>
-      <c r="S24" s="168"/>
+      <c r="J24" s="157"/>
+      <c r="K24" s="157"/>
+      <c r="L24" s="157"/>
+      <c r="M24" s="157"/>
+      <c r="N24" s="157"/>
+      <c r="O24" s="157"/>
+      <c r="P24" s="157"/>
+      <c r="Q24" s="157"/>
+      <c r="R24" s="157"/>
+      <c r="S24" s="157"/>
       <c r="T24" s="3"/>
       <c r="W24" s="53">
         <v>0.01</v>
@@ -9083,25 +9083,25 @@
     </row>
     <row r="25" spans="2:34" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B25" s="3"/>
-      <c r="C25" s="170" t="s">
+      <c r="C25" s="159" t="s">
         <v>24</v>
       </c>
-      <c r="D25" s="170"/>
+      <c r="D25" s="159"/>
       <c r="E25" s="45"/>
       <c r="F25" s="3"/>
       <c r="G25" s="3"/>
       <c r="H25" s="3"/>
-      <c r="I25" s="169"/>
-      <c r="J25" s="169"/>
-      <c r="K25" s="169"/>
-      <c r="L25" s="169"/>
-      <c r="M25" s="169"/>
-      <c r="N25" s="169"/>
-      <c r="O25" s="169"/>
-      <c r="P25" s="169"/>
-      <c r="Q25" s="169"/>
-      <c r="R25" s="169"/>
-      <c r="S25" s="169"/>
+      <c r="I25" s="158"/>
+      <c r="J25" s="158"/>
+      <c r="K25" s="158"/>
+      <c r="L25" s="158"/>
+      <c r="M25" s="158"/>
+      <c r="N25" s="158"/>
+      <c r="O25" s="158"/>
+      <c r="P25" s="158"/>
+      <c r="Q25" s="158"/>
+      <c r="R25" s="158"/>
+      <c r="S25" s="158"/>
       <c r="T25" s="3"/>
       <c r="W25" s="53">
         <v>0.01</v>
@@ -9142,11 +9142,11 @@
     </row>
     <row r="26" spans="2:34" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="3"/>
-      <c r="C26" s="170"/>
-      <c r="D26" s="170"/>
+      <c r="C26" s="159"/>
+      <c r="D26" s="159"/>
       <c r="E26" s="45"/>
       <c r="F26" s="3"/>
-      <c r="G26" s="156" t="s">
+      <c r="G26" s="160" t="s">
         <v>127</v>
       </c>
       <c r="H26" s="13">
@@ -9236,11 +9236,11 @@
     </row>
     <row r="27" spans="2:34" s="8" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B27" s="3"/>
-      <c r="C27" s="170"/>
-      <c r="D27" s="170"/>
+      <c r="C27" s="159"/>
+      <c r="D27" s="159"/>
       <c r="E27" s="45"/>
       <c r="F27" s="33"/>
-      <c r="G27" s="156"/>
+      <c r="G27" s="160"/>
       <c r="H27" s="13">
         <v>0.9</v>
       </c>
@@ -9328,13 +9328,13 @@
     </row>
     <row r="28" spans="2:34" s="8" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B28" s="3"/>
-      <c r="C28" s="170" t="s">
+      <c r="C28" s="159" t="s">
         <v>29</v>
       </c>
-      <c r="D28" s="170"/>
+      <c r="D28" s="159"/>
       <c r="E28" s="45"/>
       <c r="F28" s="33"/>
-      <c r="G28" s="156"/>
+      <c r="G28" s="160"/>
       <c r="H28" s="13">
         <v>0.8</v>
       </c>
@@ -9422,11 +9422,11 @@
     </row>
     <row r="29" spans="2:34" s="8" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B29" s="33"/>
-      <c r="C29" s="170"/>
-      <c r="D29" s="170"/>
+      <c r="C29" s="159"/>
+      <c r="D29" s="159"/>
       <c r="E29" s="45"/>
       <c r="F29" s="33"/>
-      <c r="G29" s="156"/>
+      <c r="G29" s="160"/>
       <c r="H29" s="13">
         <v>0.7</v>
       </c>
@@ -9514,13 +9514,13 @@
     </row>
     <row r="30" spans="2:34" s="8" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B30" s="3"/>
-      <c r="C30" s="170" t="s">
+      <c r="C30" s="159" t="s">
         <v>28</v>
       </c>
-      <c r="D30" s="170"/>
+      <c r="D30" s="159"/>
       <c r="E30" s="45"/>
       <c r="F30" s="33"/>
-      <c r="G30" s="156"/>
+      <c r="G30" s="160"/>
       <c r="H30" s="13">
         <v>0.6</v>
       </c>
@@ -9608,11 +9608,11 @@
     </row>
     <row r="31" spans="2:34" s="8" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B31" s="33"/>
-      <c r="C31" s="170"/>
-      <c r="D31" s="170"/>
+      <c r="C31" s="159"/>
+      <c r="D31" s="159"/>
       <c r="E31" s="45"/>
       <c r="F31" s="33"/>
-      <c r="G31" s="156"/>
+      <c r="G31" s="160"/>
       <c r="H31" s="13">
         <v>0.5</v>
       </c>
@@ -9700,13 +9700,13 @@
     </row>
     <row r="32" spans="2:34" s="8" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B32" s="33"/>
-      <c r="C32" s="170" t="s">
+      <c r="C32" s="159" t="s">
         <v>26</v>
       </c>
-      <c r="D32" s="170"/>
+      <c r="D32" s="159"/>
       <c r="E32" s="45"/>
       <c r="F32" s="33"/>
-      <c r="G32" s="156"/>
+      <c r="G32" s="160"/>
       <c r="H32" s="13">
         <v>0.4</v>
       </c>
@@ -9794,11 +9794,11 @@
     </row>
     <row r="33" spans="2:34" s="8" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B33" s="33"/>
-      <c r="C33" s="170"/>
-      <c r="D33" s="170"/>
+      <c r="C33" s="159"/>
+      <c r="D33" s="159"/>
       <c r="E33" s="45"/>
       <c r="F33" s="33"/>
-      <c r="G33" s="156"/>
+      <c r="G33" s="160"/>
       <c r="H33" s="13">
         <v>0.3</v>
       </c>
@@ -9886,13 +9886,13 @@
     </row>
     <row r="34" spans="2:34" s="8" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B34" s="33"/>
-      <c r="C34" s="170" t="s">
+      <c r="C34" s="159" t="s">
         <v>27</v>
       </c>
-      <c r="D34" s="170"/>
+      <c r="D34" s="159"/>
       <c r="E34" s="45"/>
       <c r="F34" s="33"/>
-      <c r="G34" s="156"/>
+      <c r="G34" s="160"/>
       <c r="H34" s="13">
         <v>0.2</v>
       </c>
@@ -9980,11 +9980,11 @@
     </row>
     <row r="35" spans="2:34" s="8" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B35" s="33"/>
-      <c r="C35" s="170"/>
-      <c r="D35" s="170"/>
+      <c r="C35" s="159"/>
+      <c r="D35" s="159"/>
       <c r="E35" s="45"/>
       <c r="F35" s="33"/>
-      <c r="G35" s="156"/>
+      <c r="G35" s="160"/>
       <c r="H35" s="13">
         <v>0.1</v>
       </c>
@@ -10076,7 +10076,7 @@
       <c r="D36" s="33"/>
       <c r="E36" s="33"/>
       <c r="F36" s="33"/>
-      <c r="G36" s="156"/>
+      <c r="G36" s="160"/>
       <c r="H36" s="13">
         <v>0</v>
       </c>
@@ -10249,19 +10249,19 @@
       <c r="F38" s="33"/>
       <c r="G38" s="3"/>
       <c r="H38" s="3"/>
-      <c r="I38" s="165" t="s">
+      <c r="I38" s="154" t="s">
         <v>126</v>
       </c>
-      <c r="J38" s="165"/>
-      <c r="K38" s="165"/>
-      <c r="L38" s="165"/>
-      <c r="M38" s="165"/>
-      <c r="N38" s="165"/>
-      <c r="O38" s="165"/>
-      <c r="P38" s="165"/>
-      <c r="Q38" s="165"/>
-      <c r="R38" s="165"/>
-      <c r="S38" s="165"/>
+      <c r="J38" s="154"/>
+      <c r="K38" s="154"/>
+      <c r="L38" s="154"/>
+      <c r="M38" s="154"/>
+      <c r="N38" s="154"/>
+      <c r="O38" s="154"/>
+      <c r="P38" s="154"/>
+      <c r="Q38" s="154"/>
+      <c r="R38" s="154"/>
+      <c r="S38" s="154"/>
       <c r="T38" s="3"/>
       <c r="W38" s="53">
         <v>0.02</v>
@@ -11426,7 +11426,7 @@
       </c>
     </row>
     <row r="67" spans="14:34" x14ac:dyDescent="0.2">
-      <c r="N67" s="166"/>
+      <c r="N67" s="155"/>
       <c r="O67" s="10"/>
       <c r="P67" s="11"/>
       <c r="Q67" s="11"/>
@@ -11471,7 +11471,7 @@
       </c>
     </row>
     <row r="68" spans="14:34" x14ac:dyDescent="0.2">
-      <c r="N68" s="166"/>
+      <c r="N68" s="155"/>
       <c r="O68" s="10"/>
       <c r="P68" s="11"/>
       <c r="Q68" s="11"/>
@@ -11516,7 +11516,7 @@
       </c>
     </row>
     <row r="69" spans="14:34" x14ac:dyDescent="0.2">
-      <c r="N69" s="166"/>
+      <c r="N69" s="155"/>
       <c r="O69" s="10"/>
       <c r="P69" s="11"/>
       <c r="Q69" s="11"/>
@@ -11561,7 +11561,7 @@
       </c>
     </row>
     <row r="70" spans="14:34" x14ac:dyDescent="0.2">
-      <c r="N70" s="166"/>
+      <c r="N70" s="155"/>
       <c r="O70" s="10"/>
       <c r="P70" s="11"/>
       <c r="Q70" s="11"/>
@@ -11606,7 +11606,7 @@
       </c>
     </row>
     <row r="71" spans="14:34" x14ac:dyDescent="0.2">
-      <c r="N71" s="166"/>
+      <c r="N71" s="155"/>
       <c r="O71" s="10"/>
       <c r="P71" s="11"/>
       <c r="Q71" s="11"/>
@@ -11694,11 +11694,11 @@
       </c>
     </row>
     <row r="73" spans="14:34" x14ac:dyDescent="0.2">
-      <c r="P73" s="167"/>
-      <c r="Q73" s="167"/>
-      <c r="R73" s="167"/>
-      <c r="S73" s="167"/>
-      <c r="T73" s="167"/>
+      <c r="P73" s="156"/>
+      <c r="Q73" s="156"/>
+      <c r="R73" s="156"/>
+      <c r="S73" s="156"/>
+      <c r="T73" s="156"/>
       <c r="W73" s="53">
         <v>0.06</v>
       </c>
@@ -13791,6 +13791,13 @@
   </sheetData>
   <sheetProtection sheet="1" selectLockedCells="1"/>
   <mergeCells count="17">
+    <mergeCell ref="C3:S3"/>
+    <mergeCell ref="I5:S6"/>
+    <mergeCell ref="G7:G17"/>
+    <mergeCell ref="C14:D15"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="C17:D21"/>
+    <mergeCell ref="I19:S19"/>
     <mergeCell ref="I38:S38"/>
     <mergeCell ref="N67:N71"/>
     <mergeCell ref="P73:T73"/>
@@ -13801,13 +13808,6 @@
     <mergeCell ref="C30:D31"/>
     <mergeCell ref="C32:D33"/>
     <mergeCell ref="C34:D35"/>
-    <mergeCell ref="C3:S3"/>
-    <mergeCell ref="I5:S6"/>
-    <mergeCell ref="G7:G17"/>
-    <mergeCell ref="C14:D15"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="C17:D21"/>
-    <mergeCell ref="I19:S19"/>
   </mergeCells>
   <conditionalFormatting sqref="I7:S17">
     <cfRule type="colorScale" priority="1">
@@ -14981,17 +14981,17 @@
     <row r="10" spans="2:13" ht="31" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
-      <c r="D10" s="144" t="s">
+      <c r="D10" s="146" t="s">
         <v>146</v>
       </c>
-      <c r="E10" s="144"/>
-      <c r="F10" s="144"/>
-      <c r="G10" s="144"/>
-      <c r="H10" s="144"/>
-      <c r="I10" s="144"/>
-      <c r="J10" s="144"/>
-      <c r="K10" s="144"/>
-      <c r="L10" s="144"/>
+      <c r="E10" s="146"/>
+      <c r="F10" s="146"/>
+      <c r="G10" s="146"/>
+      <c r="H10" s="146"/>
+      <c r="I10" s="146"/>
+      <c r="J10" s="146"/>
+      <c r="K10" s="146"/>
+      <c r="L10" s="146"/>
       <c r="M10" s="3"/>
     </row>
     <row r="11" spans="2:13" x14ac:dyDescent="0.2">
@@ -15011,17 +15011,17 @@
     <row r="12" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
-      <c r="D12" s="144" t="s">
+      <c r="D12" s="146" t="s">
         <v>101</v>
       </c>
-      <c r="E12" s="144"/>
-      <c r="F12" s="144"/>
-      <c r="G12" s="144"/>
-      <c r="H12" s="144"/>
-      <c r="I12" s="144"/>
-      <c r="J12" s="144"/>
-      <c r="K12" s="144"/>
-      <c r="L12" s="144"/>
+      <c r="E12" s="146"/>
+      <c r="F12" s="146"/>
+      <c r="G12" s="146"/>
+      <c r="H12" s="146"/>
+      <c r="I12" s="146"/>
+      <c r="J12" s="146"/>
+      <c r="K12" s="146"/>
+      <c r="L12" s="146"/>
       <c r="M12" s="3"/>
     </row>
     <row r="13" spans="2:13" x14ac:dyDescent="0.2">
@@ -15041,17 +15041,17 @@
     <row r="14" spans="2:13" ht="45.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
-      <c r="D14" s="144" t="s">
+      <c r="D14" s="146" t="s">
         <v>129</v>
       </c>
-      <c r="E14" s="144"/>
-      <c r="F14" s="144"/>
-      <c r="G14" s="144"/>
-      <c r="H14" s="144"/>
-      <c r="I14" s="144"/>
-      <c r="J14" s="144"/>
-      <c r="K14" s="144"/>
-      <c r="L14" s="144"/>
+      <c r="E14" s="146"/>
+      <c r="F14" s="146"/>
+      <c r="G14" s="146"/>
+      <c r="H14" s="146"/>
+      <c r="I14" s="146"/>
+      <c r="J14" s="146"/>
+      <c r="K14" s="146"/>
+      <c r="L14" s="146"/>
       <c r="M14" s="3"/>
     </row>
     <row r="15" spans="2:13" x14ac:dyDescent="0.2">
@@ -15071,17 +15071,17 @@
     <row r="16" spans="2:13" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
-      <c r="D16" s="144" t="s">
+      <c r="D16" s="146" t="s">
         <v>147</v>
       </c>
-      <c r="E16" s="144"/>
-      <c r="F16" s="144"/>
-      <c r="G16" s="144"/>
-      <c r="H16" s="144"/>
-      <c r="I16" s="144"/>
-      <c r="J16" s="144"/>
-      <c r="K16" s="144"/>
-      <c r="L16" s="144"/>
+      <c r="E16" s="146"/>
+      <c r="F16" s="146"/>
+      <c r="G16" s="146"/>
+      <c r="H16" s="146"/>
+      <c r="I16" s="146"/>
+      <c r="J16" s="146"/>
+      <c r="K16" s="146"/>
+      <c r="L16" s="146"/>
       <c r="M16" s="3"/>
     </row>
     <row r="17" spans="2:13" x14ac:dyDescent="0.2">
@@ -15101,17 +15101,17 @@
     <row r="18" spans="2:13" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
-      <c r="D18" s="144" t="s">
+      <c r="D18" s="146" t="s">
         <v>97</v>
       </c>
-      <c r="E18" s="144"/>
-      <c r="F18" s="144"/>
-      <c r="G18" s="144"/>
-      <c r="H18" s="144"/>
-      <c r="I18" s="144"/>
-      <c r="J18" s="144"/>
-      <c r="K18" s="144"/>
-      <c r="L18" s="144"/>
+      <c r="E18" s="146"/>
+      <c r="F18" s="146"/>
+      <c r="G18" s="146"/>
+      <c r="H18" s="146"/>
+      <c r="I18" s="146"/>
+      <c r="J18" s="146"/>
+      <c r="K18" s="146"/>
+      <c r="L18" s="146"/>
       <c r="M18" s="3"/>
     </row>
     <row r="19" spans="2:13" x14ac:dyDescent="0.2">
@@ -15131,17 +15131,17 @@
     <row r="20" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
-      <c r="D20" s="144" t="s">
+      <c r="D20" s="146" t="s">
         <v>130</v>
       </c>
-      <c r="E20" s="144"/>
-      <c r="F20" s="144"/>
-      <c r="G20" s="144"/>
-      <c r="H20" s="144"/>
-      <c r="I20" s="144"/>
-      <c r="J20" s="144"/>
-      <c r="K20" s="144"/>
-      <c r="L20" s="144"/>
+      <c r="E20" s="146"/>
+      <c r="F20" s="146"/>
+      <c r="G20" s="146"/>
+      <c r="H20" s="146"/>
+      <c r="I20" s="146"/>
+      <c r="J20" s="146"/>
+      <c r="K20" s="146"/>
+      <c r="L20" s="146"/>
       <c r="M20" s="3"/>
     </row>
     <row r="21" spans="2:13" x14ac:dyDescent="0.2">
@@ -15191,17 +15191,17 @@
     <row r="24" spans="2:13" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" s="3"/>
       <c r="C24" s="4"/>
-      <c r="D24" s="144" t="s">
+      <c r="D24" s="146" t="s">
         <v>131</v>
       </c>
-      <c r="E24" s="144"/>
-      <c r="F24" s="144"/>
-      <c r="G24" s="144"/>
-      <c r="H24" s="144"/>
-      <c r="I24" s="144"/>
-      <c r="J24" s="144"/>
-      <c r="K24" s="144"/>
-      <c r="L24" s="144"/>
+      <c r="E24" s="146"/>
+      <c r="F24" s="146"/>
+      <c r="G24" s="146"/>
+      <c r="H24" s="146"/>
+      <c r="I24" s="146"/>
+      <c r="J24" s="146"/>
+      <c r="K24" s="146"/>
+      <c r="L24" s="146"/>
       <c r="M24" s="3"/>
     </row>
     <row r="25" spans="2:13" x14ac:dyDescent="0.2">
@@ -15221,17 +15221,17 @@
     <row r="26" spans="2:13" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
-      <c r="D26" s="144" t="s">
+      <c r="D26" s="146" t="s">
         <v>132</v>
       </c>
-      <c r="E26" s="144"/>
-      <c r="F26" s="144"/>
-      <c r="G26" s="144"/>
-      <c r="H26" s="144"/>
-      <c r="I26" s="144"/>
-      <c r="J26" s="144"/>
-      <c r="K26" s="144"/>
-      <c r="L26" s="144"/>
+      <c r="E26" s="146"/>
+      <c r="F26" s="146"/>
+      <c r="G26" s="146"/>
+      <c r="H26" s="146"/>
+      <c r="I26" s="146"/>
+      <c r="J26" s="146"/>
+      <c r="K26" s="146"/>
+      <c r="L26" s="146"/>
       <c r="M26" s="3"/>
     </row>
     <row r="27" spans="2:13" x14ac:dyDescent="0.2">
@@ -15251,17 +15251,17 @@
     <row r="28" spans="2:13" ht="31" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
-      <c r="D28" s="144" t="s">
+      <c r="D28" s="146" t="s">
         <v>98</v>
       </c>
-      <c r="E28" s="144"/>
-      <c r="F28" s="144"/>
-      <c r="G28" s="144"/>
-      <c r="H28" s="144"/>
-      <c r="I28" s="144"/>
-      <c r="J28" s="144"/>
-      <c r="K28" s="144"/>
-      <c r="L28" s="144"/>
+      <c r="E28" s="146"/>
+      <c r="F28" s="146"/>
+      <c r="G28" s="146"/>
+      <c r="H28" s="146"/>
+      <c r="I28" s="146"/>
+      <c r="J28" s="146"/>
+      <c r="K28" s="146"/>
+      <c r="L28" s="146"/>
       <c r="M28" s="3"/>
     </row>
     <row r="29" spans="2:13" x14ac:dyDescent="0.2">
@@ -15281,17 +15281,17 @@
     <row r="30" spans="2:13" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B30" s="3"/>
       <c r="C30" s="3"/>
-      <c r="D30" s="144" t="s">
+      <c r="D30" s="146" t="s">
         <v>49</v>
       </c>
-      <c r="E30" s="144"/>
-      <c r="F30" s="144"/>
-      <c r="G30" s="144"/>
-      <c r="H30" s="144"/>
-      <c r="I30" s="144"/>
-      <c r="J30" s="144"/>
-      <c r="K30" s="144"/>
-      <c r="L30" s="144"/>
+      <c r="E30" s="146"/>
+      <c r="F30" s="146"/>
+      <c r="G30" s="146"/>
+      <c r="H30" s="146"/>
+      <c r="I30" s="146"/>
+      <c r="J30" s="146"/>
+      <c r="K30" s="146"/>
+      <c r="L30" s="146"/>
       <c r="M30" s="3"/>
     </row>
     <row r="31" spans="2:13" x14ac:dyDescent="0.2">
@@ -15367,11 +15367,6 @@
   </sheetData>
   <sheetProtection sheet="1" selectLockedCells="1"/>
   <mergeCells count="12">
-    <mergeCell ref="C5:L5"/>
-    <mergeCell ref="D20:L20"/>
-    <mergeCell ref="D8:L8"/>
-    <mergeCell ref="D10:L10"/>
-    <mergeCell ref="D26:L26"/>
     <mergeCell ref="D30:L30"/>
     <mergeCell ref="D14:L14"/>
     <mergeCell ref="D12:L12"/>
@@ -15379,6 +15374,11 @@
     <mergeCell ref="D16:L16"/>
     <mergeCell ref="D24:L24"/>
     <mergeCell ref="D28:L28"/>
+    <mergeCell ref="C5:L5"/>
+    <mergeCell ref="D20:L20"/>
+    <mergeCell ref="D8:L8"/>
+    <mergeCell ref="D10:L10"/>
+    <mergeCell ref="D26:L26"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>